<commit_message>
actualice estados de cuentas, y habilite el ingreso a las ctas 60296 y 60297
</commit_message>
<xml_diff>
--- a/excel/CLIENTES_PERMISOS.xlsx
+++ b/excel/CLIENTES_PERMISOS.xlsx
@@ -22,7 +22,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="1153" uniqueCount="391">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="1159" uniqueCount="393">
   <si>
     <t>CUENTA</t>
   </si>
@@ -1195,6 +1195,12 @@
   </si>
   <si>
     <t>ISRAEL CORDOBA</t>
+  </si>
+  <si>
+    <t>CORRALON LAS MORADAS</t>
+  </si>
+  <si>
+    <t>FERRETERIA JULIO</t>
   </si>
 </sst>
 </file>
@@ -1547,7 +1553,7 @@
   <sheetPr>
     <outlinePr summaryBelow="0" summaryRight="0"/>
   </sheetPr>
-  <dimension ref="A1:D384"/>
+  <dimension ref="A1:D386"/>
   <sheetFormatPr baseColWidth="10" defaultColWidth="12.5703125" defaultRowHeight="15.75" customHeight="1" x14ac:dyDescent="0.2"/>
   <cols>
     <col min="2" max="2" width="34" customWidth="1"/>
@@ -6331,66 +6337,66 @@
     </row>
     <row r="342" spans="1:4" ht="15.75" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A342" s="6">
-        <v>60299</v>
+        <v>60296</v>
       </c>
       <c r="B342" t="s">
-        <v>388</v>
+        <v>391</v>
       </c>
       <c r="C342" s="1" t="s">
         <v>4</v>
       </c>
       <c r="D342" s="12" t="s">
-        <v>5</v>
+        <v>8</v>
       </c>
     </row>
     <row r="343" spans="1:4" ht="15.75" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A343" s="6">
-        <v>61004</v>
+        <v>60297</v>
       </c>
       <c r="B343" t="s">
-        <v>293</v>
+        <v>392</v>
       </c>
       <c r="C343" s="1" t="s">
         <v>4</v>
       </c>
-      <c r="D343" s="15" t="s">
+      <c r="D343" s="12" t="s">
         <v>5</v>
       </c>
     </row>
     <row r="344" spans="1:4" ht="15.75" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A344" s="6">
-        <v>61009</v>
+        <v>60299</v>
       </c>
       <c r="B344" t="s">
-        <v>294</v>
+        <v>388</v>
       </c>
       <c r="C344" s="1" t="s">
         <v>4</v>
       </c>
       <c r="D344" s="12" t="s">
-        <v>8</v>
+        <v>5</v>
       </c>
     </row>
     <row r="345" spans="1:4" ht="15.75" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A345" s="6">
-        <v>61012</v>
+        <v>61004</v>
       </c>
       <c r="B345" t="s">
-        <v>295</v>
+        <v>293</v>
       </c>
       <c r="C345" s="1" t="s">
         <v>4</v>
       </c>
-      <c r="D345" s="12" t="s">
-        <v>8</v>
+      <c r="D345" s="15" t="s">
+        <v>5</v>
       </c>
     </row>
     <row r="346" spans="1:4" ht="15.75" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A346" s="6">
-        <v>61018</v>
+        <v>61009</v>
       </c>
       <c r="B346" t="s">
-        <v>296</v>
+        <v>294</v>
       </c>
       <c r="C346" s="1" t="s">
         <v>4</v>
@@ -6401,10 +6407,10 @@
     </row>
     <row r="347" spans="1:4" ht="15.75" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A347" s="6">
-        <v>61102</v>
+        <v>61012</v>
       </c>
       <c r="B347" t="s">
-        <v>297</v>
+        <v>295</v>
       </c>
       <c r="C347" s="1" t="s">
         <v>4</v>
@@ -6415,24 +6421,24 @@
     </row>
     <row r="348" spans="1:4" ht="15.75" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A348" s="6">
-        <v>61205</v>
+        <v>61018</v>
       </c>
       <c r="B348" t="s">
-        <v>298</v>
+        <v>296</v>
       </c>
       <c r="C348" s="1" t="s">
         <v>4</v>
       </c>
-      <c r="D348" s="15" t="s">
-        <v>5</v>
+      <c r="D348" s="12" t="s">
+        <v>8</v>
       </c>
     </row>
     <row r="349" spans="1:4" ht="15.75" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A349" s="6">
-        <v>70100</v>
+        <v>61102</v>
       </c>
       <c r="B349" t="s">
-        <v>299</v>
+        <v>297</v>
       </c>
       <c r="C349" s="1" t="s">
         <v>4</v>
@@ -6443,10 +6449,10 @@
     </row>
     <row r="350" spans="1:4" ht="15.75" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A350" s="6">
-        <v>70101</v>
+        <v>61205</v>
       </c>
       <c r="B350" t="s">
-        <v>300</v>
+        <v>298</v>
       </c>
       <c r="C350" s="1" t="s">
         <v>4</v>
@@ -6457,38 +6463,38 @@
     </row>
     <row r="351" spans="1:4" ht="15.75" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A351" s="6">
-        <v>70102</v>
+        <v>70100</v>
       </c>
       <c r="B351" t="s">
-        <v>301</v>
+        <v>299</v>
       </c>
       <c r="C351" s="1" t="s">
         <v>4</v>
       </c>
-      <c r="D351" s="15" t="s">
-        <v>5</v>
+      <c r="D351" s="12" t="s">
+        <v>8</v>
       </c>
     </row>
     <row r="352" spans="1:4" ht="15.75" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A352" s="6">
-        <v>70103</v>
+        <v>70101</v>
       </c>
       <c r="B352" t="s">
-        <v>302</v>
+        <v>300</v>
       </c>
       <c r="C352" s="1" t="s">
         <v>4</v>
       </c>
-      <c r="D352" s="12" t="s">
-        <v>8</v>
+      <c r="D352" s="15" t="s">
+        <v>5</v>
       </c>
     </row>
     <row r="353" spans="1:4" ht="15.75" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A353" s="6">
-        <v>70106</v>
+        <v>70102</v>
       </c>
       <c r="B353" t="s">
-        <v>303</v>
+        <v>301</v>
       </c>
       <c r="C353" s="1" t="s">
         <v>4</v>
@@ -6499,10 +6505,10 @@
     </row>
     <row r="354" spans="1:4" ht="15.75" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A354" s="6">
-        <v>70109</v>
+        <v>70103</v>
       </c>
       <c r="B354" t="s">
-        <v>304</v>
+        <v>302</v>
       </c>
       <c r="C354" s="1" t="s">
         <v>4</v>
@@ -6513,10 +6519,10 @@
     </row>
     <row r="355" spans="1:4" ht="15.75" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A355" s="6">
-        <v>70113</v>
+        <v>70106</v>
       </c>
       <c r="B355" t="s">
-        <v>305</v>
+        <v>303</v>
       </c>
       <c r="C355" s="1" t="s">
         <v>4</v>
@@ -6527,66 +6533,66 @@
     </row>
     <row r="356" spans="1:4" ht="15.75" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A356" s="6">
-        <v>70114</v>
+        <v>70109</v>
       </c>
       <c r="B356" t="s">
-        <v>325</v>
+        <v>304</v>
       </c>
       <c r="C356" s="1" t="s">
         <v>4</v>
       </c>
-      <c r="D356" s="9" t="s">
-        <v>9</v>
+      <c r="D356" s="12" t="s">
+        <v>8</v>
       </c>
     </row>
     <row r="357" spans="1:4" ht="15.75" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A357" s="6">
-        <v>70115</v>
+        <v>70113</v>
       </c>
       <c r="B357" t="s">
-        <v>331</v>
+        <v>305</v>
       </c>
       <c r="C357" s="1" t="s">
         <v>4</v>
       </c>
-      <c r="D357" s="9" t="s">
-        <v>9</v>
+      <c r="D357" s="15" t="s">
+        <v>5</v>
       </c>
     </row>
     <row r="358" spans="1:4" ht="15.75" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A358" s="6">
-        <v>70638</v>
+        <v>70114</v>
       </c>
       <c r="B358" t="s">
-        <v>306</v>
+        <v>325</v>
       </c>
       <c r="C358" s="1" t="s">
         <v>4</v>
       </c>
-      <c r="D358" s="12" t="s">
-        <v>8</v>
+      <c r="D358" s="9" t="s">
+        <v>9</v>
       </c>
     </row>
     <row r="359" spans="1:4" ht="15.75" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A359" s="6">
-        <v>70639</v>
+        <v>70115</v>
       </c>
       <c r="B359" t="s">
-        <v>307</v>
+        <v>331</v>
       </c>
       <c r="C359" s="1" t="s">
         <v>4</v>
       </c>
-      <c r="D359" s="12" t="s">
-        <v>8</v>
+      <c r="D359" s="9" t="s">
+        <v>9</v>
       </c>
     </row>
     <row r="360" spans="1:4" ht="15.75" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A360" s="6">
-        <v>70640</v>
+        <v>70638</v>
       </c>
       <c r="B360" t="s">
-        <v>308</v>
+        <v>306</v>
       </c>
       <c r="C360" s="1" t="s">
         <v>4</v>
@@ -6597,10 +6603,10 @@
     </row>
     <row r="361" spans="1:4" ht="15.75" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A361" s="6">
-        <v>70642</v>
+        <v>70639</v>
       </c>
       <c r="B361" t="s">
-        <v>309</v>
+        <v>307</v>
       </c>
       <c r="C361" s="1" t="s">
         <v>4</v>
@@ -6611,10 +6617,10 @@
     </row>
     <row r="362" spans="1:4" ht="15.75" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A362" s="6">
-        <v>90504</v>
+        <v>70640</v>
       </c>
       <c r="B362" t="s">
-        <v>310</v>
+        <v>308</v>
       </c>
       <c r="C362" s="1" t="s">
         <v>4</v>
@@ -6625,10 +6631,10 @@
     </row>
     <row r="363" spans="1:4" ht="15.75" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A363" s="6">
-        <v>90509</v>
+        <v>70642</v>
       </c>
       <c r="B363" t="s">
-        <v>311</v>
+        <v>309</v>
       </c>
       <c r="C363" s="1" t="s">
         <v>4</v>
@@ -6639,24 +6645,24 @@
     </row>
     <row r="364" spans="1:4" ht="15.75" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A364" s="6">
-        <v>90602</v>
+        <v>90504</v>
       </c>
       <c r="B364" t="s">
-        <v>312</v>
+        <v>310</v>
       </c>
       <c r="C364" s="1" t="s">
         <v>4</v>
       </c>
-      <c r="D364" s="15" t="s">
-        <v>5</v>
+      <c r="D364" s="12" t="s">
+        <v>8</v>
       </c>
     </row>
     <row r="365" spans="1:4" ht="15.75" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A365" s="6">
-        <v>90621</v>
+        <v>90509</v>
       </c>
       <c r="B365" t="s">
-        <v>313</v>
+        <v>311</v>
       </c>
       <c r="C365" s="1" t="s">
         <v>4</v>
@@ -6667,66 +6673,66 @@
     </row>
     <row r="366" spans="1:4" ht="15.75" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A366" s="6">
-        <v>90622</v>
+        <v>90602</v>
       </c>
       <c r="B366" t="s">
-        <v>333</v>
+        <v>312</v>
       </c>
       <c r="C366" s="1" t="s">
         <v>4</v>
       </c>
-      <c r="D366" s="9" t="s">
+      <c r="D366" s="15" t="s">
         <v>5</v>
       </c>
     </row>
     <row r="367" spans="1:4" ht="15.75" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A367" s="6">
-        <v>90631</v>
-      </c>
-      <c r="B367" s="8" t="s">
-        <v>342</v>
+        <v>90621</v>
+      </c>
+      <c r="B367" t="s">
+        <v>313</v>
       </c>
       <c r="C367" s="1" t="s">
         <v>4</v>
       </c>
-      <c r="D367" s="9" t="s">
-        <v>5</v>
+      <c r="D367" s="12" t="s">
+        <v>8</v>
       </c>
     </row>
     <row r="368" spans="1:4" ht="15.75" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A368" s="6">
-        <v>90658</v>
+        <v>90622</v>
       </c>
       <c r="B368" t="s">
-        <v>314</v>
+        <v>333</v>
       </c>
       <c r="C368" s="1" t="s">
         <v>4</v>
       </c>
-      <c r="D368" s="12" t="s">
-        <v>8</v>
+      <c r="D368" s="9" t="s">
+        <v>5</v>
       </c>
     </row>
     <row r="369" spans="1:4" ht="15.75" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A369" s="6">
-        <v>90660</v>
-      </c>
-      <c r="B369" t="s">
-        <v>315</v>
+        <v>90631</v>
+      </c>
+      <c r="B369" s="8" t="s">
+        <v>342</v>
       </c>
       <c r="C369" s="1" t="s">
         <v>4</v>
       </c>
-      <c r="D369" s="12" t="s">
-        <v>8</v>
+      <c r="D369" s="9" t="s">
+        <v>5</v>
       </c>
     </row>
     <row r="370" spans="1:4" ht="15.75" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A370" s="6">
-        <v>90668</v>
+        <v>90658</v>
       </c>
       <c r="B370" t="s">
-        <v>316</v>
+        <v>314</v>
       </c>
       <c r="C370" s="1" t="s">
         <v>4</v>
@@ -6737,10 +6743,10 @@
     </row>
     <row r="371" spans="1:4" ht="15.75" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A371" s="6">
-        <v>90671</v>
+        <v>90660</v>
       </c>
       <c r="B371" t="s">
-        <v>317</v>
+        <v>315</v>
       </c>
       <c r="C371" s="1" t="s">
         <v>4</v>
@@ -6751,10 +6757,10 @@
     </row>
     <row r="372" spans="1:4" ht="15.75" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A372" s="6">
-        <v>90679</v>
+        <v>90668</v>
       </c>
       <c r="B372" t="s">
-        <v>318</v>
+        <v>316</v>
       </c>
       <c r="C372" s="1" t="s">
         <v>4</v>
@@ -6765,10 +6771,10 @@
     </row>
     <row r="373" spans="1:4" ht="15.75" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A373" s="6">
-        <v>90683</v>
+        <v>90671</v>
       </c>
       <c r="B373" t="s">
-        <v>319</v>
+        <v>317</v>
       </c>
       <c r="C373" s="1" t="s">
         <v>4</v>
@@ -6779,10 +6785,10 @@
     </row>
     <row r="374" spans="1:4" ht="15.75" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A374" s="6">
-        <v>90705</v>
+        <v>90679</v>
       </c>
       <c r="B374" t="s">
-        <v>320</v>
+        <v>318</v>
       </c>
       <c r="C374" s="1" t="s">
         <v>4</v>
@@ -6793,10 +6799,10 @@
     </row>
     <row r="375" spans="1:4" ht="15.75" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A375" s="6">
-        <v>90706</v>
+        <v>90683</v>
       </c>
       <c r="B375" t="s">
-        <v>321</v>
+        <v>319</v>
       </c>
       <c r="C375" s="1" t="s">
         <v>4</v>
@@ -6807,10 +6813,10 @@
     </row>
     <row r="376" spans="1:4" ht="15.75" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A376" s="6">
-        <v>90708</v>
+        <v>90705</v>
       </c>
       <c r="B376" t="s">
-        <v>322</v>
+        <v>320</v>
       </c>
       <c r="C376" s="1" t="s">
         <v>4</v>
@@ -6821,10 +6827,10 @@
     </row>
     <row r="377" spans="1:4" ht="15.75" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A377" s="6">
-        <v>90709</v>
+        <v>90706</v>
       </c>
       <c r="B377" t="s">
-        <v>323</v>
+        <v>321</v>
       </c>
       <c r="C377" s="1" t="s">
         <v>4</v>
@@ -6835,10 +6841,10 @@
     </row>
     <row r="378" spans="1:4" ht="15.75" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A378" s="6">
-        <v>1218</v>
+        <v>90708</v>
       </c>
       <c r="B378" t="s">
-        <v>382</v>
+        <v>322</v>
       </c>
       <c r="C378" s="1" t="s">
         <v>4</v>
@@ -6849,10 +6855,10 @@
     </row>
     <row r="379" spans="1:4" ht="15.75" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A379" s="6">
-        <v>1959</v>
-      </c>
-      <c r="B379" s="8" t="s">
-        <v>383</v>
+        <v>90709</v>
+      </c>
+      <c r="B379" t="s">
+        <v>323</v>
       </c>
       <c r="C379" s="1" t="s">
         <v>4</v>
@@ -6863,10 +6869,10 @@
     </row>
     <row r="380" spans="1:4" ht="15.75" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A380" s="6">
-        <v>5625</v>
-      </c>
-      <c r="B380" s="8" t="s">
-        <v>384</v>
+        <v>1218</v>
+      </c>
+      <c r="B380" t="s">
+        <v>382</v>
       </c>
       <c r="C380" s="1" t="s">
         <v>4</v>
@@ -6877,10 +6883,10 @@
     </row>
     <row r="381" spans="1:4" ht="15.75" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A381" s="6">
-        <v>1817</v>
+        <v>1959</v>
       </c>
       <c r="B381" s="8" t="s">
-        <v>389</v>
+        <v>383</v>
       </c>
       <c r="C381" s="1" t="s">
         <v>4</v>
@@ -6891,10 +6897,10 @@
     </row>
     <row r="382" spans="1:4" ht="15.75" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A382" s="6">
-        <v>5737</v>
+        <v>5625</v>
       </c>
       <c r="B382" s="8" t="s">
-        <v>390</v>
+        <v>384</v>
       </c>
       <c r="C382" s="1" t="s">
         <v>4</v>
@@ -6905,29 +6911,57 @@
     </row>
     <row r="383" spans="1:4" ht="15.75" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A383" s="6">
-        <v>60295</v>
+        <v>1817</v>
       </c>
       <c r="B383" s="8" t="s">
-        <v>385</v>
+        <v>389</v>
       </c>
       <c r="C383" s="1" t="s">
         <v>4</v>
       </c>
-      <c r="D383" s="9" t="s">
+      <c r="D383" s="12" t="s">
         <v>8</v>
       </c>
     </row>
     <row r="384" spans="1:4" ht="15.75" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A384" s="6">
+        <v>5737</v>
+      </c>
+      <c r="B384" s="8" t="s">
+        <v>390</v>
+      </c>
+      <c r="C384" s="1" t="s">
+        <v>4</v>
+      </c>
+      <c r="D384" s="12" t="s">
+        <v>8</v>
+      </c>
+    </row>
+    <row r="385" spans="1:4" ht="15.75" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
+      <c r="A385" s="6">
+        <v>60295</v>
+      </c>
+      <c r="B385" s="8" t="s">
+        <v>385</v>
+      </c>
+      <c r="C385" s="1" t="s">
+        <v>4</v>
+      </c>
+      <c r="D385" s="9" t="s">
+        <v>8</v>
+      </c>
+    </row>
+    <row r="386" spans="1:4" ht="15.75" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
+      <c r="A386" s="6">
         <v>1045</v>
       </c>
-      <c r="B384" s="8" t="s">
+      <c r="B386" s="8" t="s">
         <v>386</v>
       </c>
-      <c r="C384" s="1" t="s">
-        <v>4</v>
-      </c>
-      <c r="D384" s="9" t="s">
+      <c r="C386" s="1" t="s">
+        <v>4</v>
+      </c>
+      <c r="D386" s="9" t="s">
         <v>5</v>
       </c>
     </row>

</xml_diff>

<commit_message>
actualice estado de cuenta 60243
</commit_message>
<xml_diff>
--- a/excel/CLIENTES_PERMISOS.xlsx
+++ b/excel/CLIENTES_PERMISOS.xlsx
@@ -22,7 +22,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="1171" uniqueCount="398">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="1171" uniqueCount="397">
   <si>
     <t>CUENTA</t>
   </si>
@@ -1210,9 +1210,6 @@
   </si>
   <si>
     <t>FERRETERIA GRACIELA</t>
-  </si>
-  <si>
-    <t>C</t>
   </si>
   <si>
     <t>DEPOSITO</t>
@@ -1595,7 +1592,7 @@
         <v>1</v>
       </c>
       <c r="B2" s="1" t="s">
-        <v>397</v>
+        <v>396</v>
       </c>
       <c r="C2" s="1" t="s">
         <v>4</v>
@@ -6039,7 +6036,7 @@
         <v>4</v>
       </c>
       <c r="D319" s="7" t="s">
-        <v>396</v>
+        <v>9</v>
       </c>
     </row>
     <row r="320" spans="1:4" ht="15.75" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">

</xml_diff>

<commit_message>
actualice listas de precios, estados de cuentas, subi imagenes de codigo zi-26-3-26
</commit_message>
<xml_diff>
--- a/excel/CLIENTES_PERMISOS.xlsx
+++ b/excel/CLIENTES_PERMISOS.xlsx
@@ -15,14 +15,14 @@
     <sheet name="Hoja 1" sheetId="1" r:id="rId1"/>
   </sheets>
   <definedNames>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'Hoja 1'!$A$1:$D$338</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'Hoja 1'!$A$1:$D$339</definedName>
   </definedNames>
   <calcPr calcId="162913"/>
 </workbook>
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="1171" uniqueCount="397">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="1174" uniqueCount="398">
   <si>
     <t>CUENTA</t>
   </si>
@@ -1213,6 +1213,9 @@
   </si>
   <si>
     <t>DEPOSITO</t>
+  </si>
+  <si>
+    <t>FERRETERIA NOR-CINTI</t>
   </si>
 </sst>
 </file>
@@ -1565,7 +1568,7 @@
   <sheetPr>
     <outlinePr summaryBelow="0" summaryRight="0"/>
   </sheetPr>
-  <dimension ref="A1:D390"/>
+  <dimension ref="A1:D391"/>
   <sheetFormatPr baseColWidth="10" defaultColWidth="12.5703125" defaultRowHeight="15.75" customHeight="1" x14ac:dyDescent="0.2"/>
   <cols>
     <col min="2" max="2" width="34" customWidth="1"/>
@@ -5313,66 +5316,66 @@
     </row>
     <row r="268" spans="1:4" ht="15.75" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A268" s="6">
-        <v>50230</v>
+        <v>50833</v>
       </c>
       <c r="B268" s="8" t="s">
-        <v>379</v>
+        <v>397</v>
       </c>
       <c r="C268" s="1" t="s">
         <v>4</v>
       </c>
       <c r="D268" s="11" t="s">
-        <v>5</v>
+        <v>8</v>
       </c>
     </row>
     <row r="269" spans="1:4" ht="15.75" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A269" s="6">
-        <v>60103</v>
-      </c>
-      <c r="B269" t="s">
-        <v>237</v>
+        <v>50230</v>
+      </c>
+      <c r="B269" s="8" t="s">
+        <v>379</v>
       </c>
       <c r="C269" s="1" t="s">
         <v>4</v>
       </c>
-      <c r="D269" s="13" t="s">
+      <c r="D269" s="11" t="s">
         <v>5</v>
       </c>
     </row>
     <row r="270" spans="1:4" ht="15.75" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A270" s="6">
-        <v>60109</v>
+        <v>60103</v>
       </c>
       <c r="B270" t="s">
-        <v>328</v>
+        <v>237</v>
       </c>
       <c r="C270" s="1" t="s">
         <v>4</v>
       </c>
-      <c r="D270" s="11" t="s">
-        <v>9</v>
+      <c r="D270" s="13" t="s">
+        <v>5</v>
       </c>
     </row>
     <row r="271" spans="1:4" ht="15.75" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A271" s="6">
-        <v>60124</v>
+        <v>60109</v>
       </c>
       <c r="B271" t="s">
-        <v>238</v>
+        <v>328</v>
       </c>
       <c r="C271" s="1" t="s">
         <v>4</v>
       </c>
-      <c r="D271" s="13" t="s">
-        <v>5</v>
+      <c r="D271" s="11" t="s">
+        <v>9</v>
       </c>
     </row>
     <row r="272" spans="1:4" ht="15.75" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A272" s="6">
-        <v>60125</v>
+        <v>60124</v>
       </c>
       <c r="B272" t="s">
-        <v>239</v>
+        <v>238</v>
       </c>
       <c r="C272" s="1" t="s">
         <v>4</v>
@@ -5383,80 +5386,80 @@
     </row>
     <row r="273" spans="1:4" ht="15.75" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A273" s="6">
-        <v>60126</v>
+        <v>60125</v>
       </c>
       <c r="B273" t="s">
-        <v>240</v>
+        <v>239</v>
       </c>
       <c r="C273" s="1" t="s">
         <v>4</v>
       </c>
-      <c r="D273" s="10" t="s">
-        <v>8</v>
+      <c r="D273" s="13" t="s">
+        <v>5</v>
       </c>
     </row>
     <row r="274" spans="1:4" ht="15.75" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A274" s="6">
-        <v>60128</v>
+        <v>60126</v>
       </c>
       <c r="B274" t="s">
-        <v>241</v>
+        <v>240</v>
       </c>
       <c r="C274" s="1" t="s">
         <v>4</v>
       </c>
-      <c r="D274" s="3" t="s">
-        <v>5</v>
+      <c r="D274" s="10" t="s">
+        <v>8</v>
       </c>
     </row>
     <row r="275" spans="1:4" ht="15.75" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A275" s="6">
-        <v>60130</v>
+        <v>60128</v>
       </c>
       <c r="B275" t="s">
-        <v>242</v>
+        <v>241</v>
       </c>
       <c r="C275" s="1" t="s">
         <v>4</v>
       </c>
-      <c r="D275" s="1" t="s">
-        <v>8</v>
+      <c r="D275" s="3" t="s">
+        <v>5</v>
       </c>
     </row>
     <row r="276" spans="1:4" ht="15.75" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A276" s="6">
-        <v>60133</v>
+        <v>60130</v>
       </c>
       <c r="B276" t="s">
-        <v>243</v>
+        <v>242</v>
       </c>
       <c r="C276" s="1" t="s">
         <v>4</v>
       </c>
-      <c r="D276" s="13" t="s">
-        <v>5</v>
+      <c r="D276" s="1" t="s">
+        <v>8</v>
       </c>
     </row>
     <row r="277" spans="1:4" ht="15.75" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A277" s="6">
-        <v>60134</v>
+        <v>60133</v>
       </c>
       <c r="B277" t="s">
-        <v>244</v>
+        <v>243</v>
       </c>
       <c r="C277" s="1" t="s">
         <v>4</v>
       </c>
-      <c r="D277" s="1" t="s">
-        <v>8</v>
+      <c r="D277" s="13" t="s">
+        <v>5</v>
       </c>
     </row>
     <row r="278" spans="1:4" ht="15.75" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A278" s="6">
-        <v>60137</v>
+        <v>60134</v>
       </c>
       <c r="B278" t="s">
-        <v>245</v>
+        <v>244</v>
       </c>
       <c r="C278" s="1" t="s">
         <v>4</v>
@@ -5467,10 +5470,10 @@
     </row>
     <row r="279" spans="1:4" ht="15.75" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A279" s="6">
-        <v>60139</v>
+        <v>60137</v>
       </c>
       <c r="B279" t="s">
-        <v>246</v>
+        <v>245</v>
       </c>
       <c r="C279" s="1" t="s">
         <v>4</v>
@@ -5481,10 +5484,10 @@
     </row>
     <row r="280" spans="1:4" ht="15.75" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A280" s="6">
-        <v>60142</v>
+        <v>60139</v>
       </c>
       <c r="B280" t="s">
-        <v>247</v>
+        <v>246</v>
       </c>
       <c r="C280" s="1" t="s">
         <v>4</v>
@@ -5495,10 +5498,10 @@
     </row>
     <row r="281" spans="1:4" ht="15.75" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A281" s="6">
-        <v>60148</v>
+        <v>60142</v>
       </c>
       <c r="B281" t="s">
-        <v>248</v>
+        <v>247</v>
       </c>
       <c r="C281" s="1" t="s">
         <v>4</v>
@@ -5509,10 +5512,10 @@
     </row>
     <row r="282" spans="1:4" ht="15.75" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A282" s="6">
-        <v>60149</v>
+        <v>60148</v>
       </c>
       <c r="B282" t="s">
-        <v>249</v>
+        <v>248</v>
       </c>
       <c r="C282" s="1" t="s">
         <v>4</v>
@@ -5523,66 +5526,66 @@
     </row>
     <row r="283" spans="1:4" ht="15.75" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A283" s="6">
-        <v>60150</v>
+        <v>60149</v>
       </c>
       <c r="B283" t="s">
-        <v>332</v>
+        <v>249</v>
       </c>
       <c r="C283" s="1" t="s">
         <v>4</v>
       </c>
-      <c r="D283" s="13" t="s">
-        <v>5</v>
+      <c r="D283" s="1" t="s">
+        <v>8</v>
       </c>
     </row>
     <row r="284" spans="1:4" ht="15.75" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A284" s="6">
-        <v>60158</v>
+        <v>60150</v>
       </c>
       <c r="B284" t="s">
-        <v>250</v>
+        <v>332</v>
       </c>
       <c r="C284" s="1" t="s">
         <v>4</v>
       </c>
-      <c r="D284" s="10" t="s">
-        <v>8</v>
+      <c r="D284" s="13" t="s">
+        <v>5</v>
       </c>
     </row>
     <row r="285" spans="1:4" ht="15.75" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A285" s="6">
-        <v>60159</v>
+        <v>60158</v>
       </c>
       <c r="B285" t="s">
-        <v>251</v>
+        <v>250</v>
       </c>
       <c r="C285" s="1" t="s">
         <v>4</v>
       </c>
-      <c r="D285" s="1" t="s">
+      <c r="D285" s="10" t="s">
         <v>8</v>
       </c>
     </row>
     <row r="286" spans="1:4" ht="15.75" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A286" s="6">
-        <v>60162</v>
+        <v>60159</v>
       </c>
       <c r="B286" t="s">
-        <v>252</v>
+        <v>251</v>
       </c>
       <c r="C286" s="1" t="s">
         <v>4</v>
       </c>
-      <c r="D286" s="13" t="s">
-        <v>5</v>
+      <c r="D286" s="1" t="s">
+        <v>8</v>
       </c>
     </row>
     <row r="287" spans="1:4" ht="15.75" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A287" s="6">
-        <v>60163</v>
+        <v>60162</v>
       </c>
       <c r="B287" t="s">
-        <v>253</v>
+        <v>252</v>
       </c>
       <c r="C287" s="1" t="s">
         <v>4</v>
@@ -5593,24 +5596,24 @@
     </row>
     <row r="288" spans="1:4" ht="15.75" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A288" s="6">
-        <v>60165</v>
+        <v>60163</v>
       </c>
       <c r="B288" t="s">
-        <v>254</v>
+        <v>253</v>
       </c>
       <c r="C288" s="1" t="s">
         <v>4</v>
       </c>
-      <c r="D288" s="1" t="s">
-        <v>8</v>
+      <c r="D288" s="13" t="s">
+        <v>5</v>
       </c>
     </row>
     <row r="289" spans="1:4" ht="15.75" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A289" s="6">
-        <v>60169</v>
+        <v>60165</v>
       </c>
       <c r="B289" t="s">
-        <v>255</v>
+        <v>254</v>
       </c>
       <c r="C289" s="1" t="s">
         <v>4</v>
@@ -5621,52 +5624,52 @@
     </row>
     <row r="290" spans="1:4" ht="15.75" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A290" s="6">
-        <v>60170</v>
-      </c>
-      <c r="B290" s="8" t="s">
-        <v>337</v>
+        <v>60169</v>
+      </c>
+      <c r="B290" t="s">
+        <v>255</v>
       </c>
       <c r="C290" s="1" t="s">
         <v>4</v>
       </c>
-      <c r="D290" s="11" t="s">
+      <c r="D290" s="1" t="s">
         <v>8</v>
       </c>
     </row>
     <row r="291" spans="1:4" ht="15.75" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A291" s="6">
-        <v>60172</v>
-      </c>
-      <c r="B291" t="s">
-        <v>256</v>
+        <v>60170</v>
+      </c>
+      <c r="B291" s="8" t="s">
+        <v>337</v>
       </c>
       <c r="C291" s="1" t="s">
         <v>4</v>
       </c>
-      <c r="D291" s="1" t="s">
+      <c r="D291" s="11" t="s">
         <v>8</v>
       </c>
     </row>
     <row r="292" spans="1:4" ht="15.75" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A292" s="6">
-        <v>60174</v>
+        <v>60172</v>
       </c>
       <c r="B292" t="s">
-        <v>257</v>
+        <v>256</v>
       </c>
       <c r="C292" s="1" t="s">
         <v>4</v>
       </c>
-      <c r="D292" s="13" t="s">
-        <v>5</v>
+      <c r="D292" s="1" t="s">
+        <v>8</v>
       </c>
     </row>
     <row r="293" spans="1:4" ht="15.75" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A293" s="6">
-        <v>60176</v>
+        <v>60174</v>
       </c>
       <c r="B293" t="s">
-        <v>258</v>
+        <v>257</v>
       </c>
       <c r="C293" s="1" t="s">
         <v>4</v>
@@ -5677,52 +5680,52 @@
     </row>
     <row r="294" spans="1:4" ht="15.75" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A294" s="6">
-        <v>60178</v>
+        <v>60176</v>
       </c>
       <c r="B294" t="s">
-        <v>259</v>
+        <v>258</v>
       </c>
       <c r="C294" s="1" t="s">
         <v>4</v>
       </c>
-      <c r="D294" s="1" t="s">
-        <v>8</v>
+      <c r="D294" s="13" t="s">
+        <v>5</v>
       </c>
     </row>
     <row r="295" spans="1:4" ht="15.75" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A295" s="6">
-        <v>60180</v>
+        <v>60178</v>
       </c>
       <c r="B295" t="s">
-        <v>260</v>
+        <v>259</v>
       </c>
       <c r="C295" s="1" t="s">
         <v>4</v>
       </c>
-      <c r="D295" s="10" t="s">
+      <c r="D295" s="1" t="s">
         <v>8</v>
       </c>
     </row>
     <row r="296" spans="1:4" ht="15.75" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A296" s="6">
-        <v>60184</v>
+        <v>60180</v>
       </c>
       <c r="B296" t="s">
-        <v>261</v>
+        <v>260</v>
       </c>
       <c r="C296" s="1" t="s">
         <v>4</v>
       </c>
-      <c r="D296" s="1" t="s">
+      <c r="D296" s="10" t="s">
         <v>8</v>
       </c>
     </row>
     <row r="297" spans="1:4" ht="15.75" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A297" s="6">
-        <v>60190</v>
+        <v>60184</v>
       </c>
       <c r="B297" t="s">
-        <v>262</v>
+        <v>261</v>
       </c>
       <c r="C297" s="1" t="s">
         <v>4</v>
@@ -5733,24 +5736,24 @@
     </row>
     <row r="298" spans="1:4" ht="15.75" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A298" s="6">
-        <v>60191</v>
+        <v>60190</v>
       </c>
       <c r="B298" t="s">
-        <v>263</v>
+        <v>262</v>
       </c>
       <c r="C298" s="1" t="s">
         <v>4</v>
       </c>
-      <c r="D298" s="10" t="s">
+      <c r="D298" s="1" t="s">
         <v>8</v>
       </c>
     </row>
     <row r="299" spans="1:4" ht="15.75" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A299" s="6">
-        <v>60192</v>
+        <v>60191</v>
       </c>
       <c r="B299" t="s">
-        <v>264</v>
+        <v>263</v>
       </c>
       <c r="C299" s="1" t="s">
         <v>4</v>
@@ -5761,10 +5764,10 @@
     </row>
     <row r="300" spans="1:4" ht="15.75" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A300" s="6">
-        <v>60195</v>
+        <v>60192</v>
       </c>
       <c r="B300" t="s">
-        <v>265</v>
+        <v>264</v>
       </c>
       <c r="C300" s="1" t="s">
         <v>4</v>
@@ -5775,10 +5778,10 @@
     </row>
     <row r="301" spans="1:4" ht="15.75" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A301" s="6">
-        <v>60196</v>
+        <v>60195</v>
       </c>
       <c r="B301" t="s">
-        <v>266</v>
+        <v>265</v>
       </c>
       <c r="C301" s="1" t="s">
         <v>4</v>
@@ -5789,10 +5792,10 @@
     </row>
     <row r="302" spans="1:4" ht="15.75" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A302" s="6">
-        <v>60198</v>
+        <v>60196</v>
       </c>
       <c r="B302" t="s">
-        <v>267</v>
+        <v>266</v>
       </c>
       <c r="C302" s="1" t="s">
         <v>4</v>
@@ -5803,52 +5806,52 @@
     </row>
     <row r="303" spans="1:4" ht="15.75" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A303" s="6">
-        <v>60201</v>
+        <v>60198</v>
       </c>
       <c r="B303" t="s">
-        <v>268</v>
+        <v>267</v>
       </c>
       <c r="C303" s="1" t="s">
         <v>4</v>
       </c>
-      <c r="D303" t="s">
-        <v>9</v>
+      <c r="D303" s="10" t="s">
+        <v>8</v>
       </c>
     </row>
     <row r="304" spans="1:4" ht="15.75" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A304" s="6">
-        <v>60202</v>
+        <v>60201</v>
       </c>
       <c r="B304" t="s">
-        <v>269</v>
+        <v>268</v>
       </c>
       <c r="C304" s="1" t="s">
         <v>4</v>
       </c>
-      <c r="D304" s="13" t="s">
-        <v>5</v>
+      <c r="D304" t="s">
+        <v>9</v>
       </c>
     </row>
     <row r="305" spans="1:4" ht="15.75" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A305" s="6">
-        <v>60204</v>
+        <v>60202</v>
       </c>
       <c r="B305" t="s">
-        <v>270</v>
+        <v>269</v>
       </c>
       <c r="C305" s="1" t="s">
         <v>4</v>
       </c>
-      <c r="D305" s="1" t="s">
-        <v>8</v>
+      <c r="D305" s="13" t="s">
+        <v>5</v>
       </c>
     </row>
     <row r="306" spans="1:4" ht="15.75" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A306" s="6">
-        <v>60205</v>
+        <v>60204</v>
       </c>
       <c r="B306" t="s">
-        <v>271</v>
+        <v>270</v>
       </c>
       <c r="C306" s="1" t="s">
         <v>4</v>
@@ -5859,10 +5862,10 @@
     </row>
     <row r="307" spans="1:4" ht="15.75" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A307" s="6">
-        <v>60206</v>
+        <v>60205</v>
       </c>
       <c r="B307" t="s">
-        <v>272</v>
+        <v>271</v>
       </c>
       <c r="C307" s="1" t="s">
         <v>4</v>
@@ -5873,220 +5876,220 @@
     </row>
     <row r="308" spans="1:4" ht="15.75" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A308" s="6">
-        <v>60209</v>
+        <v>60206</v>
       </c>
       <c r="B308" t="s">
-        <v>273</v>
+        <v>272</v>
       </c>
       <c r="C308" s="1" t="s">
         <v>4</v>
       </c>
-      <c r="D308" s="10" t="s">
+      <c r="D308" s="1" t="s">
         <v>8</v>
       </c>
     </row>
     <row r="309" spans="1:4" ht="15.75" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A309" s="6">
-        <v>60211</v>
+        <v>60209</v>
       </c>
       <c r="B309" t="s">
-        <v>274</v>
+        <v>273</v>
       </c>
       <c r="C309" s="1" t="s">
         <v>4</v>
       </c>
-      <c r="D309" s="1" t="s">
+      <c r="D309" s="10" t="s">
         <v>8</v>
       </c>
     </row>
     <row r="310" spans="1:4" ht="15.75" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A310" s="6">
-        <v>60215</v>
+        <v>60211</v>
       </c>
       <c r="B310" t="s">
-        <v>275</v>
+        <v>274</v>
       </c>
       <c r="C310" s="1" t="s">
         <v>4</v>
       </c>
-      <c r="D310" s="10" t="s">
+      <c r="D310" s="1" t="s">
         <v>8</v>
       </c>
     </row>
     <row r="311" spans="1:4" ht="15.75" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A311" s="6">
-        <v>60216</v>
+        <v>60215</v>
       </c>
       <c r="B311" t="s">
-        <v>381</v>
+        <v>275</v>
       </c>
       <c r="C311" s="1" t="s">
         <v>4</v>
       </c>
       <c r="D311" s="10" t="s">
-        <v>9</v>
+        <v>8</v>
       </c>
     </row>
     <row r="312" spans="1:4" ht="15.75" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A312" s="6">
-        <v>60217</v>
+        <v>60216</v>
       </c>
       <c r="B312" t="s">
-        <v>276</v>
+        <v>381</v>
       </c>
       <c r="C312" s="1" t="s">
         <v>4</v>
       </c>
       <c r="D312" s="10" t="s">
-        <v>8</v>
+        <v>9</v>
       </c>
     </row>
     <row r="313" spans="1:4" ht="15.75" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A313" s="6">
-        <v>60219</v>
+        <v>60217</v>
       </c>
       <c r="B313" t="s">
-        <v>277</v>
+        <v>276</v>
       </c>
       <c r="C313" s="1" t="s">
         <v>4</v>
       </c>
-      <c r="D313" s="1" t="s">
+      <c r="D313" s="10" t="s">
         <v>8</v>
       </c>
     </row>
     <row r="314" spans="1:4" ht="15.75" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A314" s="6">
-        <v>60222</v>
+        <v>60219</v>
       </c>
       <c r="B314" t="s">
-        <v>278</v>
+        <v>277</v>
       </c>
       <c r="C314" s="1" t="s">
         <v>4</v>
       </c>
-      <c r="D314" s="10" t="s">
+      <c r="D314" s="1" t="s">
         <v>8</v>
       </c>
     </row>
     <row r="315" spans="1:4" ht="15.75" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A315" s="6">
-        <v>60225</v>
+        <v>60222</v>
       </c>
       <c r="B315" t="s">
-        <v>279</v>
+        <v>278</v>
       </c>
       <c r="C315" s="1" t="s">
         <v>4</v>
       </c>
-      <c r="D315" s="17" t="s">
-        <v>9</v>
+      <c r="D315" s="10" t="s">
+        <v>8</v>
       </c>
     </row>
     <row r="316" spans="1:4" ht="15.75" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A316" s="6">
-        <v>60230</v>
+        <v>60225</v>
       </c>
       <c r="B316" t="s">
-        <v>280</v>
+        <v>279</v>
       </c>
       <c r="C316" s="1" t="s">
         <v>4</v>
       </c>
-      <c r="D316" s="10" t="s">
-        <v>8</v>
+      <c r="D316" s="17" t="s">
+        <v>9</v>
       </c>
     </row>
     <row r="317" spans="1:4" ht="15.75" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A317" s="6">
-        <v>60241</v>
-      </c>
-      <c r="B317" s="8" t="s">
-        <v>338</v>
+        <v>60230</v>
+      </c>
+      <c r="B317" t="s">
+        <v>280</v>
       </c>
       <c r="C317" s="1" t="s">
         <v>4</v>
       </c>
-      <c r="D317" s="7" t="s">
-        <v>9</v>
+      <c r="D317" s="10" t="s">
+        <v>8</v>
       </c>
     </row>
     <row r="318" spans="1:4" ht="15.75" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A318" s="6">
-        <v>60242</v>
+        <v>60241</v>
       </c>
       <c r="B318" s="8" t="s">
-        <v>341</v>
+        <v>338</v>
       </c>
       <c r="C318" s="1" t="s">
         <v>4</v>
       </c>
       <c r="D318" s="7" t="s">
-        <v>5</v>
+        <v>9</v>
       </c>
     </row>
     <row r="319" spans="1:4" ht="15.75" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A319" s="6">
-        <v>60243</v>
+        <v>60242</v>
       </c>
       <c r="B319" s="8" t="s">
-        <v>395</v>
+        <v>341</v>
       </c>
       <c r="C319" s="1" t="s">
         <v>4</v>
       </c>
       <c r="D319" s="7" t="s">
-        <v>9</v>
+        <v>5</v>
       </c>
     </row>
     <row r="320" spans="1:4" ht="15.75" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A320" s="6">
-        <v>60245</v>
+        <v>60243</v>
       </c>
       <c r="B320" s="8" t="s">
-        <v>387</v>
+        <v>395</v>
       </c>
       <c r="C320" s="1" t="s">
         <v>4</v>
       </c>
       <c r="D320" s="7" t="s">
-        <v>5</v>
+        <v>9</v>
       </c>
     </row>
     <row r="321" spans="1:4" ht="15.75" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A321" s="6">
-        <v>60250</v>
+        <v>60245</v>
       </c>
       <c r="B321" s="8" t="s">
-        <v>339</v>
+        <v>387</v>
       </c>
       <c r="C321" s="1" t="s">
         <v>4</v>
       </c>
-      <c r="D321" s="11" t="s">
-        <v>8</v>
+      <c r="D321" s="7" t="s">
+        <v>5</v>
       </c>
     </row>
     <row r="322" spans="1:4" ht="15.75" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A322" s="6">
-        <v>60253</v>
-      </c>
-      <c r="B322" t="s">
-        <v>281</v>
+        <v>60250</v>
+      </c>
+      <c r="B322" s="8" t="s">
+        <v>339</v>
       </c>
       <c r="C322" s="1" t="s">
         <v>4</v>
       </c>
-      <c r="D322" s="1" t="s">
+      <c r="D322" s="11" t="s">
         <v>8</v>
       </c>
     </row>
     <row r="323" spans="1:4" ht="15.75" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A323" s="6">
-        <v>60254</v>
+        <v>60253</v>
       </c>
       <c r="B323" t="s">
-        <v>282</v>
+        <v>281</v>
       </c>
       <c r="C323" s="1" t="s">
         <v>4</v>
@@ -6097,10 +6100,10 @@
     </row>
     <row r="324" spans="1:4" ht="15.75" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A324" s="6">
-        <v>60257</v>
+        <v>60254</v>
       </c>
       <c r="B324" t="s">
-        <v>283</v>
+        <v>282</v>
       </c>
       <c r="C324" s="1" t="s">
         <v>4</v>
@@ -6111,10 +6114,10 @@
     </row>
     <row r="325" spans="1:4" ht="15.75" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A325" s="6">
-        <v>60258</v>
+        <v>60257</v>
       </c>
       <c r="B325" t="s">
-        <v>284</v>
+        <v>283</v>
       </c>
       <c r="C325" s="1" t="s">
         <v>4</v>
@@ -6125,66 +6128,66 @@
     </row>
     <row r="326" spans="1:4" ht="15.75" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A326" s="6">
-        <v>60266</v>
-      </c>
-      <c r="B326" s="8" t="s">
-        <v>343</v>
+        <v>60258</v>
+      </c>
+      <c r="B326" t="s">
+        <v>284</v>
       </c>
       <c r="C326" s="1" t="s">
         <v>4</v>
       </c>
-      <c r="D326" s="11" t="s">
+      <c r="D326" s="1" t="s">
         <v>8</v>
       </c>
     </row>
     <row r="327" spans="1:4" ht="15.75" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A327" s="6">
-        <v>60269</v>
-      </c>
-      <c r="B327" t="s">
-        <v>285</v>
+        <v>60266</v>
+      </c>
+      <c r="B327" s="8" t="s">
+        <v>343</v>
       </c>
       <c r="C327" s="1" t="s">
         <v>4</v>
       </c>
-      <c r="D327" s="10" t="s">
+      <c r="D327" s="11" t="s">
         <v>8</v>
       </c>
     </row>
     <row r="328" spans="1:4" ht="15.75" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A328" s="6">
-        <v>60270</v>
+        <v>60269</v>
       </c>
       <c r="B328" t="s">
-        <v>286</v>
+        <v>285</v>
       </c>
       <c r="C328" s="1" t="s">
         <v>4</v>
       </c>
-      <c r="D328" s="1" t="s">
-        <v>9</v>
+      <c r="D328" s="10" t="s">
+        <v>8</v>
       </c>
     </row>
     <row r="329" spans="1:4" ht="15.75" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A329" s="6">
-        <v>60272</v>
+        <v>60270</v>
       </c>
       <c r="B329" t="s">
-        <v>287</v>
+        <v>286</v>
       </c>
       <c r="C329" s="1" t="s">
         <v>4</v>
       </c>
       <c r="D329" s="1" t="s">
-        <v>8</v>
+        <v>9</v>
       </c>
     </row>
     <row r="330" spans="1:4" ht="15.75" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A330" s="6">
-        <v>60274</v>
+        <v>60272</v>
       </c>
       <c r="B330" t="s">
-        <v>380</v>
+        <v>287</v>
       </c>
       <c r="C330" s="1" t="s">
         <v>4</v>
@@ -6195,10 +6198,10 @@
     </row>
     <row r="331" spans="1:4" ht="15.75" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A331" s="6">
-        <v>60275</v>
+        <v>60274</v>
       </c>
       <c r="B331" t="s">
-        <v>288</v>
+        <v>380</v>
       </c>
       <c r="C331" s="1" t="s">
         <v>4</v>
@@ -6209,10 +6212,10 @@
     </row>
     <row r="332" spans="1:4" ht="15.75" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A332" s="6">
-        <v>60276</v>
+        <v>60275</v>
       </c>
       <c r="B332" t="s">
-        <v>289</v>
+        <v>288</v>
       </c>
       <c r="C332" s="1" t="s">
         <v>4</v>
@@ -6223,108 +6226,108 @@
     </row>
     <row r="333" spans="1:4" ht="15.75" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A333" s="6">
-        <v>60278</v>
+        <v>60276</v>
       </c>
       <c r="B333" t="s">
-        <v>290</v>
+        <v>289</v>
       </c>
       <c r="C333" s="1" t="s">
         <v>4</v>
       </c>
-      <c r="D333" s="13" t="s">
+      <c r="D333" s="1" t="s">
         <v>8</v>
       </c>
     </row>
     <row r="334" spans="1:4" ht="15.75" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A334" s="6">
-        <v>60279</v>
+        <v>60278</v>
       </c>
       <c r="B334" t="s">
-        <v>291</v>
+        <v>290</v>
       </c>
       <c r="C334" s="1" t="s">
         <v>4</v>
       </c>
-      <c r="D334" s="1" t="s">
+      <c r="D334" s="13" t="s">
         <v>8</v>
       </c>
     </row>
     <row r="335" spans="1:4" ht="15.75" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A335" s="6">
-        <v>60280</v>
+        <v>60279</v>
       </c>
       <c r="B335" t="s">
-        <v>292</v>
+        <v>291</v>
       </c>
       <c r="C335" s="1" t="s">
         <v>4</v>
       </c>
       <c r="D335" s="1" t="s">
-        <v>5</v>
+        <v>8</v>
       </c>
     </row>
     <row r="336" spans="1:4" ht="15.75" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A336" s="6">
-        <v>60281</v>
-      </c>
-      <c r="B336" s="8" t="s">
-        <v>336</v>
+        <v>60280</v>
+      </c>
+      <c r="B336" t="s">
+        <v>292</v>
       </c>
       <c r="C336" s="1" t="s">
         <v>4</v>
       </c>
-      <c r="D336" s="11" t="s">
-        <v>9</v>
+      <c r="D336" s="1" t="s">
+        <v>5</v>
       </c>
     </row>
     <row r="337" spans="1:4" ht="15.75" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A337" s="6">
-        <v>60282</v>
+        <v>60281</v>
       </c>
       <c r="B337" s="8" t="s">
-        <v>340</v>
+        <v>336</v>
       </c>
       <c r="C337" s="1" t="s">
         <v>4</v>
       </c>
       <c r="D337" s="11" t="s">
-        <v>5</v>
+        <v>9</v>
       </c>
     </row>
     <row r="338" spans="1:4" ht="15.75" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A338" s="6">
-        <v>60283</v>
-      </c>
-      <c r="B338" t="s">
-        <v>378</v>
+        <v>60282</v>
+      </c>
+      <c r="B338" s="8" t="s">
+        <v>340</v>
       </c>
       <c r="C338" s="1" t="s">
         <v>4</v>
       </c>
-      <c r="D338" s="1" t="s">
-        <v>8</v>
+      <c r="D338" s="11" t="s">
+        <v>5</v>
       </c>
     </row>
     <row r="339" spans="1:4" ht="15.75" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A339" s="6">
-        <v>60284</v>
-      </c>
-      <c r="B339" s="8" t="s">
-        <v>335</v>
+        <v>60283</v>
+      </c>
+      <c r="B339" t="s">
+        <v>378</v>
       </c>
       <c r="C339" s="1" t="s">
         <v>4</v>
       </c>
-      <c r="D339" s="9" t="s">
-        <v>5</v>
+      <c r="D339" s="1" t="s">
+        <v>8</v>
       </c>
     </row>
     <row r="340" spans="1:4" ht="15.75" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A340" s="6">
-        <v>60285</v>
+        <v>60284</v>
       </c>
       <c r="B340" s="8" t="s">
-        <v>350</v>
+        <v>335</v>
       </c>
       <c r="C340" s="1" t="s">
         <v>4</v>
@@ -6335,10 +6338,10 @@
     </row>
     <row r="341" spans="1:4" ht="15.75" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A341" s="6">
-        <v>60286</v>
+        <v>60285</v>
       </c>
       <c r="B341" s="8" t="s">
-        <v>334</v>
+        <v>350</v>
       </c>
       <c r="C341" s="1" t="s">
         <v>4</v>
@@ -6349,52 +6352,52 @@
     </row>
     <row r="342" spans="1:4" ht="15.75" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A342" s="6">
-        <v>60287</v>
-      </c>
-      <c r="B342" t="s">
-        <v>377</v>
+        <v>60286</v>
+      </c>
+      <c r="B342" s="8" t="s">
+        <v>334</v>
       </c>
       <c r="C342" s="1" t="s">
         <v>4</v>
       </c>
-      <c r="D342" s="12" t="s">
+      <c r="D342" s="9" t="s">
         <v>5</v>
       </c>
     </row>
     <row r="343" spans="1:4" ht="15.75" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A343" s="6">
-        <v>60289</v>
+        <v>60287</v>
       </c>
       <c r="B343" t="s">
-        <v>374</v>
+        <v>377</v>
       </c>
       <c r="C343" s="1" t="s">
         <v>4</v>
       </c>
       <c r="D343" s="12" t="s">
-        <v>9</v>
+        <v>5</v>
       </c>
     </row>
     <row r="344" spans="1:4" ht="15.75" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A344" s="6">
-        <v>60290</v>
+        <v>60289</v>
       </c>
       <c r="B344" t="s">
-        <v>375</v>
+        <v>374</v>
       </c>
       <c r="C344" s="1" t="s">
         <v>4</v>
       </c>
       <c r="D344" s="12" t="s">
-        <v>5</v>
+        <v>9</v>
       </c>
     </row>
     <row r="345" spans="1:4" ht="15.75" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A345" s="6">
-        <v>60291</v>
+        <v>60290</v>
       </c>
       <c r="B345" t="s">
-        <v>376</v>
+        <v>375</v>
       </c>
       <c r="C345" s="1" t="s">
         <v>4</v>
@@ -6405,38 +6408,38 @@
     </row>
     <row r="346" spans="1:4" ht="15.75" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A346" s="6">
-        <v>60296</v>
+        <v>60291</v>
       </c>
       <c r="B346" t="s">
-        <v>391</v>
+        <v>376</v>
       </c>
       <c r="C346" s="1" t="s">
         <v>4</v>
       </c>
       <c r="D346" s="12" t="s">
-        <v>8</v>
+        <v>5</v>
       </c>
     </row>
     <row r="347" spans="1:4" ht="15.75" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A347" s="6">
-        <v>60297</v>
+        <v>60296</v>
       </c>
       <c r="B347" t="s">
-        <v>392</v>
+        <v>391</v>
       </c>
       <c r="C347" s="1" t="s">
         <v>4</v>
       </c>
       <c r="D347" s="12" t="s">
-        <v>5</v>
+        <v>8</v>
       </c>
     </row>
     <row r="348" spans="1:4" ht="15.75" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A348" s="6">
-        <v>60299</v>
+        <v>60297</v>
       </c>
       <c r="B348" t="s">
-        <v>388</v>
+        <v>392</v>
       </c>
       <c r="C348" s="1" t="s">
         <v>4</v>
@@ -6447,38 +6450,38 @@
     </row>
     <row r="349" spans="1:4" ht="15.75" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A349" s="6">
-        <v>61004</v>
+        <v>60299</v>
       </c>
       <c r="B349" t="s">
-        <v>293</v>
+        <v>388</v>
       </c>
       <c r="C349" s="1" t="s">
         <v>4</v>
       </c>
-      <c r="D349" s="15" t="s">
+      <c r="D349" s="12" t="s">
         <v>5</v>
       </c>
     </row>
     <row r="350" spans="1:4" ht="15.75" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A350" s="6">
-        <v>61009</v>
+        <v>61004</v>
       </c>
       <c r="B350" t="s">
-        <v>294</v>
+        <v>293</v>
       </c>
       <c r="C350" s="1" t="s">
         <v>4</v>
       </c>
-      <c r="D350" s="12" t="s">
-        <v>8</v>
+      <c r="D350" s="15" t="s">
+        <v>5</v>
       </c>
     </row>
     <row r="351" spans="1:4" ht="15.75" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A351" s="6">
-        <v>61012</v>
+        <v>61009</v>
       </c>
       <c r="B351" t="s">
-        <v>295</v>
+        <v>294</v>
       </c>
       <c r="C351" s="1" t="s">
         <v>4</v>
@@ -6489,10 +6492,10 @@
     </row>
     <row r="352" spans="1:4" ht="15.75" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A352" s="6">
-        <v>61018</v>
+        <v>61012</v>
       </c>
       <c r="B352" t="s">
-        <v>296</v>
+        <v>295</v>
       </c>
       <c r="C352" s="1" t="s">
         <v>4</v>
@@ -6503,10 +6506,10 @@
     </row>
     <row r="353" spans="1:4" ht="15.75" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A353" s="6">
-        <v>61102</v>
+        <v>61018</v>
       </c>
       <c r="B353" t="s">
-        <v>297</v>
+        <v>296</v>
       </c>
       <c r="C353" s="1" t="s">
         <v>4</v>
@@ -6517,52 +6520,52 @@
     </row>
     <row r="354" spans="1:4" ht="15.75" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A354" s="6">
-        <v>61205</v>
+        <v>61102</v>
       </c>
       <c r="B354" t="s">
-        <v>298</v>
+        <v>297</v>
       </c>
       <c r="C354" s="1" t="s">
         <v>4</v>
       </c>
-      <c r="D354" s="15" t="s">
-        <v>5</v>
+      <c r="D354" s="12" t="s">
+        <v>8</v>
       </c>
     </row>
     <row r="355" spans="1:4" ht="15.75" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A355" s="6">
-        <v>70100</v>
+        <v>61205</v>
       </c>
       <c r="B355" t="s">
-        <v>299</v>
+        <v>298</v>
       </c>
       <c r="C355" s="1" t="s">
         <v>4</v>
       </c>
-      <c r="D355" s="12" t="s">
-        <v>8</v>
+      <c r="D355" s="15" t="s">
+        <v>5</v>
       </c>
     </row>
     <row r="356" spans="1:4" ht="15.75" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A356" s="6">
-        <v>70101</v>
+        <v>70100</v>
       </c>
       <c r="B356" t="s">
-        <v>300</v>
+        <v>299</v>
       </c>
       <c r="C356" s="1" t="s">
         <v>4</v>
       </c>
-      <c r="D356" s="15" t="s">
-        <v>5</v>
+      <c r="D356" s="12" t="s">
+        <v>8</v>
       </c>
     </row>
     <row r="357" spans="1:4" ht="15.75" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A357" s="6">
-        <v>70102</v>
+        <v>70101</v>
       </c>
       <c r="B357" t="s">
-        <v>301</v>
+        <v>300</v>
       </c>
       <c r="C357" s="1" t="s">
         <v>4</v>
@@ -6573,80 +6576,80 @@
     </row>
     <row r="358" spans="1:4" ht="15.75" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A358" s="6">
-        <v>70103</v>
+        <v>70102</v>
       </c>
       <c r="B358" t="s">
-        <v>302</v>
+        <v>301</v>
       </c>
       <c r="C358" s="1" t="s">
         <v>4</v>
       </c>
-      <c r="D358" s="12" t="s">
-        <v>8</v>
+      <c r="D358" s="15" t="s">
+        <v>5</v>
       </c>
     </row>
     <row r="359" spans="1:4" ht="15.75" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A359" s="6">
-        <v>70106</v>
+        <v>70103</v>
       </c>
       <c r="B359" t="s">
-        <v>303</v>
+        <v>302</v>
       </c>
       <c r="C359" s="1" t="s">
         <v>4</v>
       </c>
-      <c r="D359" s="15" t="s">
-        <v>5</v>
+      <c r="D359" s="12" t="s">
+        <v>8</v>
       </c>
     </row>
     <row r="360" spans="1:4" ht="15.75" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A360" s="6">
-        <v>70109</v>
+        <v>70106</v>
       </c>
       <c r="B360" t="s">
-        <v>304</v>
+        <v>303</v>
       </c>
       <c r="C360" s="1" t="s">
         <v>4</v>
       </c>
-      <c r="D360" s="12" t="s">
-        <v>8</v>
+      <c r="D360" s="15" t="s">
+        <v>5</v>
       </c>
     </row>
     <row r="361" spans="1:4" ht="15.75" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A361" s="6">
-        <v>70113</v>
+        <v>70109</v>
       </c>
       <c r="B361" t="s">
-        <v>305</v>
+        <v>304</v>
       </c>
       <c r="C361" s="1" t="s">
         <v>4</v>
       </c>
-      <c r="D361" s="15" t="s">
-        <v>5</v>
+      <c r="D361" s="12" t="s">
+        <v>8</v>
       </c>
     </row>
     <row r="362" spans="1:4" ht="15.75" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A362" s="6">
-        <v>70114</v>
+        <v>70113</v>
       </c>
       <c r="B362" t="s">
-        <v>325</v>
+        <v>305</v>
       </c>
       <c r="C362" s="1" t="s">
         <v>4</v>
       </c>
-      <c r="D362" s="9" t="s">
-        <v>9</v>
+      <c r="D362" s="15" t="s">
+        <v>5</v>
       </c>
     </row>
     <row r="363" spans="1:4" ht="15.75" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A363" s="6">
-        <v>70115</v>
+        <v>70114</v>
       </c>
       <c r="B363" t="s">
-        <v>331</v>
+        <v>325</v>
       </c>
       <c r="C363" s="1" t="s">
         <v>4</v>
@@ -6657,24 +6660,24 @@
     </row>
     <row r="364" spans="1:4" ht="15.75" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A364" s="6">
-        <v>70638</v>
+        <v>70115</v>
       </c>
       <c r="B364" t="s">
-        <v>306</v>
+        <v>331</v>
       </c>
       <c r="C364" s="1" t="s">
         <v>4</v>
       </c>
-      <c r="D364" s="12" t="s">
-        <v>8</v>
+      <c r="D364" s="9" t="s">
+        <v>9</v>
       </c>
     </row>
     <row r="365" spans="1:4" ht="15.75" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A365" s="6">
-        <v>70639</v>
+        <v>70638</v>
       </c>
       <c r="B365" t="s">
-        <v>307</v>
+        <v>306</v>
       </c>
       <c r="C365" s="1" t="s">
         <v>4</v>
@@ -6685,10 +6688,10 @@
     </row>
     <row r="366" spans="1:4" ht="15.75" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A366" s="6">
-        <v>70640</v>
+        <v>70639</v>
       </c>
       <c r="B366" t="s">
-        <v>308</v>
+        <v>307</v>
       </c>
       <c r="C366" s="1" t="s">
         <v>4</v>
@@ -6699,10 +6702,10 @@
     </row>
     <row r="367" spans="1:4" ht="15.75" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A367" s="6">
-        <v>70642</v>
+        <v>70640</v>
       </c>
       <c r="B367" t="s">
-        <v>309</v>
+        <v>308</v>
       </c>
       <c r="C367" s="1" t="s">
         <v>4</v>
@@ -6713,10 +6716,10 @@
     </row>
     <row r="368" spans="1:4" ht="15.75" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A368" s="6">
-        <v>90504</v>
+        <v>70642</v>
       </c>
       <c r="B368" t="s">
-        <v>310</v>
+        <v>309</v>
       </c>
       <c r="C368" s="1" t="s">
         <v>4</v>
@@ -6727,10 +6730,10 @@
     </row>
     <row r="369" spans="1:4" ht="15.75" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A369" s="6">
-        <v>90509</v>
+        <v>90504</v>
       </c>
       <c r="B369" t="s">
-        <v>311</v>
+        <v>310</v>
       </c>
       <c r="C369" s="1" t="s">
         <v>4</v>
@@ -6741,52 +6744,52 @@
     </row>
     <row r="370" spans="1:4" ht="15.75" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A370" s="6">
-        <v>90602</v>
+        <v>90509</v>
       </c>
       <c r="B370" t="s">
-        <v>312</v>
+        <v>311</v>
       </c>
       <c r="C370" s="1" t="s">
         <v>4</v>
       </c>
-      <c r="D370" s="15" t="s">
-        <v>5</v>
+      <c r="D370" s="12" t="s">
+        <v>8</v>
       </c>
     </row>
     <row r="371" spans="1:4" ht="15.75" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A371" s="6">
-        <v>90621</v>
+        <v>90602</v>
       </c>
       <c r="B371" t="s">
-        <v>313</v>
+        <v>312</v>
       </c>
       <c r="C371" s="1" t="s">
         <v>4</v>
       </c>
-      <c r="D371" s="12" t="s">
-        <v>8</v>
+      <c r="D371" s="15" t="s">
+        <v>5</v>
       </c>
     </row>
     <row r="372" spans="1:4" ht="15.75" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A372" s="6">
-        <v>90622</v>
+        <v>90621</v>
       </c>
       <c r="B372" t="s">
-        <v>333</v>
+        <v>313</v>
       </c>
       <c r="C372" s="1" t="s">
         <v>4</v>
       </c>
-      <c r="D372" s="9" t="s">
-        <v>5</v>
+      <c r="D372" s="12" t="s">
+        <v>8</v>
       </c>
     </row>
     <row r="373" spans="1:4" ht="15.75" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A373" s="6">
-        <v>90631</v>
-      </c>
-      <c r="B373" s="8" t="s">
-        <v>342</v>
+        <v>90622</v>
+      </c>
+      <c r="B373" t="s">
+        <v>333</v>
       </c>
       <c r="C373" s="1" t="s">
         <v>4</v>
@@ -6797,24 +6800,24 @@
     </row>
     <row r="374" spans="1:4" ht="15.75" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A374" s="6">
-        <v>90658</v>
-      </c>
-      <c r="B374" t="s">
-        <v>314</v>
+        <v>90631</v>
+      </c>
+      <c r="B374" s="8" t="s">
+        <v>342</v>
       </c>
       <c r="C374" s="1" t="s">
         <v>4</v>
       </c>
-      <c r="D374" s="12" t="s">
-        <v>8</v>
+      <c r="D374" s="9" t="s">
+        <v>5</v>
       </c>
     </row>
     <row r="375" spans="1:4" ht="15.75" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A375" s="6">
-        <v>90660</v>
+        <v>90658</v>
       </c>
       <c r="B375" t="s">
-        <v>315</v>
+        <v>314</v>
       </c>
       <c r="C375" s="1" t="s">
         <v>4</v>
@@ -6825,10 +6828,10 @@
     </row>
     <row r="376" spans="1:4" ht="15.75" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A376" s="6">
-        <v>90668</v>
+        <v>90660</v>
       </c>
       <c r="B376" t="s">
-        <v>316</v>
+        <v>315</v>
       </c>
       <c r="C376" s="1" t="s">
         <v>4</v>
@@ -6839,10 +6842,10 @@
     </row>
     <row r="377" spans="1:4" ht="15.75" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A377" s="6">
-        <v>90671</v>
+        <v>90668</v>
       </c>
       <c r="B377" t="s">
-        <v>317</v>
+        <v>316</v>
       </c>
       <c r="C377" s="1" t="s">
         <v>4</v>
@@ -6853,10 +6856,10 @@
     </row>
     <row r="378" spans="1:4" ht="15.75" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A378" s="6">
-        <v>90679</v>
+        <v>90671</v>
       </c>
       <c r="B378" t="s">
-        <v>318</v>
+        <v>317</v>
       </c>
       <c r="C378" s="1" t="s">
         <v>4</v>
@@ -6867,10 +6870,10 @@
     </row>
     <row r="379" spans="1:4" ht="15.75" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A379" s="6">
-        <v>90683</v>
+        <v>90679</v>
       </c>
       <c r="B379" t="s">
-        <v>319</v>
+        <v>318</v>
       </c>
       <c r="C379" s="1" t="s">
         <v>4</v>
@@ -6881,10 +6884,10 @@
     </row>
     <row r="380" spans="1:4" ht="15.75" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A380" s="6">
-        <v>90705</v>
+        <v>90683</v>
       </c>
       <c r="B380" t="s">
-        <v>320</v>
+        <v>319</v>
       </c>
       <c r="C380" s="1" t="s">
         <v>4</v>
@@ -6895,10 +6898,10 @@
     </row>
     <row r="381" spans="1:4" ht="15.75" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A381" s="6">
-        <v>90706</v>
+        <v>90705</v>
       </c>
       <c r="B381" t="s">
-        <v>321</v>
+        <v>320</v>
       </c>
       <c r="C381" s="1" t="s">
         <v>4</v>
@@ -6909,10 +6912,10 @@
     </row>
     <row r="382" spans="1:4" ht="15.75" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A382" s="6">
-        <v>90708</v>
+        <v>90706</v>
       </c>
       <c r="B382" t="s">
-        <v>322</v>
+        <v>321</v>
       </c>
       <c r="C382" s="1" t="s">
         <v>4</v>
@@ -6923,10 +6926,10 @@
     </row>
     <row r="383" spans="1:4" ht="15.75" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A383" s="6">
-        <v>90709</v>
+        <v>90708</v>
       </c>
       <c r="B383" t="s">
-        <v>323</v>
+        <v>322</v>
       </c>
       <c r="C383" s="1" t="s">
         <v>4</v>
@@ -6937,10 +6940,10 @@
     </row>
     <row r="384" spans="1:4" ht="15.75" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A384" s="6">
-        <v>1218</v>
+        <v>90709</v>
       </c>
       <c r="B384" t="s">
-        <v>382</v>
+        <v>323</v>
       </c>
       <c r="C384" s="1" t="s">
         <v>4</v>
@@ -6951,10 +6954,10 @@
     </row>
     <row r="385" spans="1:4" ht="15.75" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A385" s="6">
-        <v>1959</v>
-      </c>
-      <c r="B385" s="8" t="s">
-        <v>383</v>
+        <v>1218</v>
+      </c>
+      <c r="B385" t="s">
+        <v>382</v>
       </c>
       <c r="C385" s="1" t="s">
         <v>4</v>
@@ -6965,10 +6968,10 @@
     </row>
     <row r="386" spans="1:4" ht="15.75" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A386" s="6">
-        <v>5625</v>
+        <v>1959</v>
       </c>
       <c r="B386" s="8" t="s">
-        <v>384</v>
+        <v>383</v>
       </c>
       <c r="C386" s="1" t="s">
         <v>4</v>
@@ -6979,10 +6982,10 @@
     </row>
     <row r="387" spans="1:4" ht="15.75" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A387" s="6">
-        <v>1817</v>
+        <v>5625</v>
       </c>
       <c r="B387" s="8" t="s">
-        <v>389</v>
+        <v>384</v>
       </c>
       <c r="C387" s="1" t="s">
         <v>4</v>
@@ -6993,10 +6996,10 @@
     </row>
     <row r="388" spans="1:4" ht="15.75" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A388" s="6">
-        <v>5737</v>
+        <v>1817</v>
       </c>
       <c r="B388" s="8" t="s">
-        <v>390</v>
+        <v>389</v>
       </c>
       <c r="C388" s="1" t="s">
         <v>4</v>
@@ -7007,34 +7010,48 @@
     </row>
     <row r="389" spans="1:4" ht="15.75" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A389" s="6">
-        <v>60295</v>
+        <v>5737</v>
       </c>
       <c r="B389" s="8" t="s">
-        <v>385</v>
+        <v>390</v>
       </c>
       <c r="C389" s="1" t="s">
         <v>4</v>
       </c>
-      <c r="D389" s="9" t="s">
-        <v>9</v>
+      <c r="D389" s="12" t="s">
+        <v>8</v>
       </c>
     </row>
     <row r="390" spans="1:4" ht="15.75" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A390" s="6">
+        <v>60295</v>
+      </c>
+      <c r="B390" s="8" t="s">
+        <v>385</v>
+      </c>
+      <c r="C390" s="1" t="s">
+        <v>4</v>
+      </c>
+      <c r="D390" s="9" t="s">
+        <v>9</v>
+      </c>
+    </row>
+    <row r="391" spans="1:4" ht="15.75" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
+      <c r="A391" s="6">
         <v>1045</v>
       </c>
-      <c r="B390" s="8" t="s">
+      <c r="B391" s="8" t="s">
         <v>386</v>
       </c>
-      <c r="C390" s="1" t="s">
-        <v>4</v>
-      </c>
-      <c r="D390" s="9" t="s">
+      <c r="C391" s="1" t="s">
+        <v>4</v>
+      </c>
+      <c r="D391" s="9" t="s">
         <v>5</v>
       </c>
     </row>
   </sheetData>
-  <autoFilter ref="A1:D338"/>
+  <autoFilter ref="A1:D339"/>
   <sortState ref="A2:D374">
     <sortCondition ref="A277"/>
   </sortState>

</xml_diff>

<commit_message>
actualice esta de cuentas, subi iamgenes codigo ly-20-4-26
</commit_message>
<xml_diff>
--- a/excel/CLIENTES_PERMISOS.xlsx
+++ b/excel/CLIENTES_PERMISOS.xlsx
@@ -22,7 +22,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="1183" uniqueCount="401">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="1183" uniqueCount="402">
   <si>
     <t>CUENTA</t>
   </si>
@@ -1225,6 +1225,9 @@
   </si>
   <si>
     <t>FERRETERIA ALFA</t>
+  </si>
+  <si>
+    <t>C</t>
   </si>
 </sst>
 </file>
@@ -5335,7 +5338,7 @@
         <v>4</v>
       </c>
       <c r="D268" s="11" t="s">
-        <v>5</v>
+        <v>401</v>
       </c>
     </row>
     <row r="269" spans="1:4" ht="15.75" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">

</xml_diff>

<commit_message>
actualice esta de cuentas,listas de precios, subi iamgenes codigo ly-21-4-26
</commit_message>
<xml_diff>
--- a/excel/CLIENTES_PERMISOS.xlsx
+++ b/excel/CLIENTES_PERMISOS.xlsx
@@ -22,7 +22,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="1183" uniqueCount="402">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="1183" uniqueCount="401">
   <si>
     <t>CUENTA</t>
   </si>
@@ -1225,9 +1225,6 @@
   </si>
   <si>
     <t>FERRETERIA ALFA</t>
-  </si>
-  <si>
-    <t>C</t>
   </si>
 </sst>
 </file>
@@ -5338,7 +5335,7 @@
         <v>4</v>
       </c>
       <c r="D268" s="11" t="s">
-        <v>401</v>
+        <v>8</v>
       </c>
     </row>
     <row r="269" spans="1:4" ht="15.75" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">

</xml_diff>

<commit_message>
agregue cta 90713, subi imagenes de bremen-19-5-26
</commit_message>
<xml_diff>
--- a/excel/CLIENTES_PERMISOS.xlsx
+++ b/excel/CLIENTES_PERMISOS.xlsx
@@ -22,7 +22,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="1186" uniqueCount="402">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="1189" uniqueCount="403">
   <si>
     <t>CUENTA</t>
   </si>
@@ -1228,6 +1228,9 @@
   </si>
   <si>
     <t>FERRETERIA VIGO</t>
+  </si>
+  <si>
+    <t>SANTO DOMINGO</t>
   </si>
 </sst>
 </file>
@@ -1581,7 +1584,7 @@
   <sheetPr>
     <outlinePr summaryBelow="0" summaryRight="0"/>
   </sheetPr>
-  <dimension ref="A1:D395"/>
+  <dimension ref="A1:D396"/>
   <sheetFormatPr baseColWidth="10" defaultColWidth="12.5703125" defaultRowHeight="15.75" customHeight="1" x14ac:dyDescent="0.2"/>
   <cols>
     <col min="2" max="2" width="34" customWidth="1"/>
@@ -7023,24 +7026,24 @@
     </row>
     <row r="389" spans="1:4" ht="15.75" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A389" s="6">
-        <v>1218</v>
+        <v>90713</v>
       </c>
       <c r="B389" t="s">
-        <v>382</v>
+        <v>402</v>
       </c>
       <c r="C389" s="1" t="s">
         <v>4</v>
       </c>
       <c r="D389" s="12" t="s">
-        <v>8</v>
+        <v>5</v>
       </c>
     </row>
     <row r="390" spans="1:4" ht="15.75" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A390" s="6">
-        <v>1959</v>
-      </c>
-      <c r="B390" s="8" t="s">
-        <v>383</v>
+        <v>1218</v>
+      </c>
+      <c r="B390" t="s">
+        <v>382</v>
       </c>
       <c r="C390" s="1" t="s">
         <v>4</v>
@@ -7051,10 +7054,10 @@
     </row>
     <row r="391" spans="1:4" ht="15.75" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A391" s="6">
-        <v>5625</v>
+        <v>1959</v>
       </c>
       <c r="B391" s="8" t="s">
-        <v>384</v>
+        <v>383</v>
       </c>
       <c r="C391" s="1" t="s">
         <v>4</v>
@@ -7065,10 +7068,10 @@
     </row>
     <row r="392" spans="1:4" ht="15.75" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A392" s="6">
-        <v>1817</v>
+        <v>5625</v>
       </c>
       <c r="B392" s="8" t="s">
-        <v>389</v>
+        <v>384</v>
       </c>
       <c r="C392" s="1" t="s">
         <v>4</v>
@@ -7079,10 +7082,10 @@
     </row>
     <row r="393" spans="1:4" ht="15.75" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A393" s="6">
-        <v>5737</v>
+        <v>1817</v>
       </c>
       <c r="B393" s="8" t="s">
-        <v>390</v>
+        <v>389</v>
       </c>
       <c r="C393" s="1" t="s">
         <v>4</v>
@@ -7093,29 +7096,43 @@
     </row>
     <row r="394" spans="1:4" ht="15.75" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A394" s="6">
-        <v>60295</v>
+        <v>5737</v>
       </c>
       <c r="B394" s="8" t="s">
-        <v>385</v>
+        <v>390</v>
       </c>
       <c r="C394" s="1" t="s">
         <v>4</v>
       </c>
-      <c r="D394" s="9" t="s">
-        <v>9</v>
+      <c r="D394" s="12" t="s">
+        <v>8</v>
       </c>
     </row>
     <row r="395" spans="1:4" ht="15.75" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A395" s="6">
+        <v>60295</v>
+      </c>
+      <c r="B395" s="8" t="s">
+        <v>385</v>
+      </c>
+      <c r="C395" s="1" t="s">
+        <v>4</v>
+      </c>
+      <c r="D395" s="9" t="s">
+        <v>9</v>
+      </c>
+    </row>
+    <row r="396" spans="1:4" ht="15.75" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
+      <c r="A396" s="6">
         <v>1045</v>
       </c>
-      <c r="B395" s="8" t="s">
+      <c r="B396" s="8" t="s">
         <v>386</v>
       </c>
-      <c r="C395" s="1" t="s">
-        <v>4</v>
-      </c>
-      <c r="D395" s="9" t="s">
+      <c r="C396" s="1" t="s">
+        <v>4</v>
+      </c>
+      <c r="D396" s="9" t="s">
         <v>5</v>
       </c>
     </row>

</xml_diff>

<commit_message>
habilite cuenta 50831, listas de precios -2-6-26
</commit_message>
<xml_diff>
--- a/excel/CLIENTES_PERMISOS.xlsx
+++ b/excel/CLIENTES_PERMISOS.xlsx
@@ -22,7 +22,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="1189" uniqueCount="403">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="1192" uniqueCount="404">
   <si>
     <t>CUENTA</t>
   </si>
@@ -1231,6 +1231,9 @@
   </si>
   <si>
     <t>SANTO DOMINGO</t>
+  </si>
+  <si>
+    <t>FERRIYAN 2</t>
   </si>
 </sst>
 </file>
@@ -1584,7 +1587,7 @@
   <sheetPr>
     <outlinePr summaryBelow="0" summaryRight="0"/>
   </sheetPr>
-  <dimension ref="A1:D396"/>
+  <dimension ref="A1:D397"/>
   <sheetFormatPr baseColWidth="10" defaultColWidth="12.5703125" defaultRowHeight="15.75" customHeight="1" x14ac:dyDescent="0.2"/>
   <cols>
     <col min="2" max="2" width="34" customWidth="1"/>
@@ -6536,38 +6539,38 @@
     </row>
     <row r="354" spans="1:4" ht="15.75" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A354" s="6">
-        <v>61004</v>
+        <v>61001</v>
       </c>
       <c r="B354" t="s">
-        <v>293</v>
+        <v>403</v>
       </c>
       <c r="C354" s="1" t="s">
         <v>4</v>
       </c>
-      <c r="D354" s="15" t="s">
-        <v>5</v>
+      <c r="D354" s="12" t="s">
+        <v>8</v>
       </c>
     </row>
     <row r="355" spans="1:4" ht="15.75" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A355" s="6">
-        <v>61009</v>
+        <v>61004</v>
       </c>
       <c r="B355" t="s">
-        <v>294</v>
+        <v>293</v>
       </c>
       <c r="C355" s="1" t="s">
         <v>4</v>
       </c>
-      <c r="D355" s="12" t="s">
-        <v>8</v>
+      <c r="D355" s="15" t="s">
+        <v>5</v>
       </c>
     </row>
     <row r="356" spans="1:4" ht="15.75" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A356" s="6">
-        <v>61012</v>
+        <v>61009</v>
       </c>
       <c r="B356" t="s">
-        <v>295</v>
+        <v>294</v>
       </c>
       <c r="C356" s="1" t="s">
         <v>4</v>
@@ -6578,10 +6581,10 @@
     </row>
     <row r="357" spans="1:4" ht="15.75" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A357" s="6">
-        <v>61018</v>
+        <v>61012</v>
       </c>
       <c r="B357" t="s">
-        <v>296</v>
+        <v>295</v>
       </c>
       <c r="C357" s="1" t="s">
         <v>4</v>
@@ -6592,10 +6595,10 @@
     </row>
     <row r="358" spans="1:4" ht="15.75" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A358" s="6">
-        <v>61102</v>
+        <v>61018</v>
       </c>
       <c r="B358" t="s">
-        <v>297</v>
+        <v>296</v>
       </c>
       <c r="C358" s="1" t="s">
         <v>4</v>
@@ -6606,52 +6609,52 @@
     </row>
     <row r="359" spans="1:4" ht="15.75" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A359" s="6">
-        <v>61205</v>
+        <v>61102</v>
       </c>
       <c r="B359" t="s">
-        <v>298</v>
+        <v>297</v>
       </c>
       <c r="C359" s="1" t="s">
         <v>4</v>
       </c>
-      <c r="D359" s="15" t="s">
-        <v>5</v>
+      <c r="D359" s="12" t="s">
+        <v>8</v>
       </c>
     </row>
     <row r="360" spans="1:4" ht="15.75" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A360" s="6">
-        <v>70100</v>
+        <v>61205</v>
       </c>
       <c r="B360" t="s">
-        <v>299</v>
+        <v>298</v>
       </c>
       <c r="C360" s="1" t="s">
         <v>4</v>
       </c>
-      <c r="D360" s="12" t="s">
-        <v>8</v>
+      <c r="D360" s="15" t="s">
+        <v>5</v>
       </c>
     </row>
     <row r="361" spans="1:4" ht="15.75" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A361" s="6">
-        <v>70101</v>
+        <v>70100</v>
       </c>
       <c r="B361" t="s">
-        <v>300</v>
+        <v>299</v>
       </c>
       <c r="C361" s="1" t="s">
         <v>4</v>
       </c>
-      <c r="D361" s="15" t="s">
-        <v>5</v>
+      <c r="D361" s="12" t="s">
+        <v>8</v>
       </c>
     </row>
     <row r="362" spans="1:4" ht="15.75" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A362" s="6">
-        <v>70102</v>
+        <v>70101</v>
       </c>
       <c r="B362" t="s">
-        <v>301</v>
+        <v>300</v>
       </c>
       <c r="C362" s="1" t="s">
         <v>4</v>
@@ -6662,80 +6665,80 @@
     </row>
     <row r="363" spans="1:4" ht="15.75" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A363" s="6">
-        <v>70103</v>
+        <v>70102</v>
       </c>
       <c r="B363" t="s">
-        <v>302</v>
+        <v>301</v>
       </c>
       <c r="C363" s="1" t="s">
         <v>4</v>
       </c>
-      <c r="D363" s="12" t="s">
-        <v>8</v>
+      <c r="D363" s="15" t="s">
+        <v>5</v>
       </c>
     </row>
     <row r="364" spans="1:4" ht="15.75" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A364" s="6">
-        <v>70106</v>
+        <v>70103</v>
       </c>
       <c r="B364" t="s">
-        <v>303</v>
+        <v>302</v>
       </c>
       <c r="C364" s="1" t="s">
         <v>4</v>
       </c>
-      <c r="D364" s="15" t="s">
-        <v>5</v>
+      <c r="D364" s="12" t="s">
+        <v>8</v>
       </c>
     </row>
     <row r="365" spans="1:4" ht="15.75" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A365" s="6">
-        <v>70109</v>
+        <v>70106</v>
       </c>
       <c r="B365" t="s">
-        <v>304</v>
+        <v>303</v>
       </c>
       <c r="C365" s="1" t="s">
         <v>4</v>
       </c>
-      <c r="D365" s="12" t="s">
-        <v>8</v>
+      <c r="D365" s="15" t="s">
+        <v>5</v>
       </c>
     </row>
     <row r="366" spans="1:4" ht="15.75" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A366" s="6">
-        <v>70113</v>
+        <v>70109</v>
       </c>
       <c r="B366" t="s">
-        <v>305</v>
+        <v>304</v>
       </c>
       <c r="C366" s="1" t="s">
         <v>4</v>
       </c>
-      <c r="D366" s="15" t="s">
-        <v>5</v>
+      <c r="D366" s="12" t="s">
+        <v>8</v>
       </c>
     </row>
     <row r="367" spans="1:4" ht="15.75" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A367" s="6">
-        <v>70114</v>
+        <v>70113</v>
       </c>
       <c r="B367" t="s">
-        <v>325</v>
+        <v>305</v>
       </c>
       <c r="C367" s="1" t="s">
         <v>4</v>
       </c>
-      <c r="D367" s="9" t="s">
-        <v>9</v>
+      <c r="D367" s="15" t="s">
+        <v>5</v>
       </c>
     </row>
     <row r="368" spans="1:4" ht="15.75" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A368" s="6">
-        <v>70115</v>
+        <v>70114</v>
       </c>
       <c r="B368" t="s">
-        <v>331</v>
+        <v>325</v>
       </c>
       <c r="C368" s="1" t="s">
         <v>4</v>
@@ -6746,24 +6749,24 @@
     </row>
     <row r="369" spans="1:4" ht="15.75" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A369" s="6">
-        <v>70638</v>
+        <v>70115</v>
       </c>
       <c r="B369" t="s">
-        <v>306</v>
+        <v>331</v>
       </c>
       <c r="C369" s="1" t="s">
         <v>4</v>
       </c>
-      <c r="D369" s="12" t="s">
-        <v>8</v>
+      <c r="D369" s="9" t="s">
+        <v>9</v>
       </c>
     </row>
     <row r="370" spans="1:4" ht="15.75" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A370" s="6">
-        <v>70639</v>
+        <v>70638</v>
       </c>
       <c r="B370" t="s">
-        <v>307</v>
+        <v>306</v>
       </c>
       <c r="C370" s="1" t="s">
         <v>4</v>
@@ -6774,10 +6777,10 @@
     </row>
     <row r="371" spans="1:4" ht="15.75" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A371" s="6">
-        <v>70640</v>
+        <v>70639</v>
       </c>
       <c r="B371" t="s">
-        <v>308</v>
+        <v>307</v>
       </c>
       <c r="C371" s="1" t="s">
         <v>4</v>
@@ -6788,10 +6791,10 @@
     </row>
     <row r="372" spans="1:4" ht="15.75" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A372" s="6">
-        <v>70642</v>
+        <v>70640</v>
       </c>
       <c r="B372" t="s">
-        <v>309</v>
+        <v>308</v>
       </c>
       <c r="C372" s="1" t="s">
         <v>4</v>
@@ -6802,10 +6805,10 @@
     </row>
     <row r="373" spans="1:4" ht="15.75" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A373" s="6">
-        <v>90504</v>
+        <v>70642</v>
       </c>
       <c r="B373" t="s">
-        <v>310</v>
+        <v>309</v>
       </c>
       <c r="C373" s="1" t="s">
         <v>4</v>
@@ -6816,10 +6819,10 @@
     </row>
     <row r="374" spans="1:4" ht="15.75" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A374" s="6">
-        <v>90509</v>
+        <v>90504</v>
       </c>
       <c r="B374" t="s">
-        <v>311</v>
+        <v>310</v>
       </c>
       <c r="C374" s="1" t="s">
         <v>4</v>
@@ -6830,52 +6833,52 @@
     </row>
     <row r="375" spans="1:4" ht="15.75" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A375" s="6">
-        <v>90602</v>
+        <v>90509</v>
       </c>
       <c r="B375" t="s">
-        <v>312</v>
+        <v>311</v>
       </c>
       <c r="C375" s="1" t="s">
         <v>4</v>
       </c>
-      <c r="D375" s="15" t="s">
-        <v>5</v>
+      <c r="D375" s="12" t="s">
+        <v>8</v>
       </c>
     </row>
     <row r="376" spans="1:4" ht="15.75" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A376" s="6">
-        <v>90621</v>
+        <v>90602</v>
       </c>
       <c r="B376" t="s">
-        <v>313</v>
+        <v>312</v>
       </c>
       <c r="C376" s="1" t="s">
         <v>4</v>
       </c>
-      <c r="D376" s="12" t="s">
-        <v>8</v>
+      <c r="D376" s="15" t="s">
+        <v>5</v>
       </c>
     </row>
     <row r="377" spans="1:4" ht="15.75" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A377" s="6">
-        <v>90622</v>
+        <v>90621</v>
       </c>
       <c r="B377" t="s">
-        <v>333</v>
+        <v>313</v>
       </c>
       <c r="C377" s="1" t="s">
         <v>4</v>
       </c>
-      <c r="D377" s="9" t="s">
-        <v>5</v>
+      <c r="D377" s="12" t="s">
+        <v>8</v>
       </c>
     </row>
     <row r="378" spans="1:4" ht="15.75" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A378" s="6">
-        <v>90631</v>
-      </c>
-      <c r="B378" s="8" t="s">
-        <v>342</v>
+        <v>90622</v>
+      </c>
+      <c r="B378" t="s">
+        <v>333</v>
       </c>
       <c r="C378" s="1" t="s">
         <v>4</v>
@@ -6886,24 +6889,24 @@
     </row>
     <row r="379" spans="1:4" ht="15.75" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A379" s="6">
-        <v>90658</v>
-      </c>
-      <c r="B379" t="s">
-        <v>314</v>
+        <v>90631</v>
+      </c>
+      <c r="B379" s="8" t="s">
+        <v>342</v>
       </c>
       <c r="C379" s="1" t="s">
         <v>4</v>
       </c>
-      <c r="D379" s="12" t="s">
-        <v>8</v>
+      <c r="D379" s="9" t="s">
+        <v>5</v>
       </c>
     </row>
     <row r="380" spans="1:4" ht="15.75" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A380" s="6">
-        <v>90660</v>
+        <v>90658</v>
       </c>
       <c r="B380" t="s">
-        <v>315</v>
+        <v>314</v>
       </c>
       <c r="C380" s="1" t="s">
         <v>4</v>
@@ -6914,10 +6917,10 @@
     </row>
     <row r="381" spans="1:4" ht="15.75" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A381" s="6">
-        <v>90668</v>
+        <v>90660</v>
       </c>
       <c r="B381" t="s">
-        <v>316</v>
+        <v>315</v>
       </c>
       <c r="C381" s="1" t="s">
         <v>4</v>
@@ -6928,10 +6931,10 @@
     </row>
     <row r="382" spans="1:4" ht="15.75" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A382" s="6">
-        <v>90671</v>
+        <v>90668</v>
       </c>
       <c r="B382" t="s">
-        <v>317</v>
+        <v>316</v>
       </c>
       <c r="C382" s="1" t="s">
         <v>4</v>
@@ -6942,10 +6945,10 @@
     </row>
     <row r="383" spans="1:4" ht="15.75" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A383" s="6">
-        <v>90679</v>
+        <v>90671</v>
       </c>
       <c r="B383" t="s">
-        <v>318</v>
+        <v>317</v>
       </c>
       <c r="C383" s="1" t="s">
         <v>4</v>
@@ -6956,10 +6959,10 @@
     </row>
     <row r="384" spans="1:4" ht="15.75" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A384" s="6">
-        <v>90683</v>
+        <v>90679</v>
       </c>
       <c r="B384" t="s">
-        <v>319</v>
+        <v>318</v>
       </c>
       <c r="C384" s="1" t="s">
         <v>4</v>
@@ -6970,10 +6973,10 @@
     </row>
     <row r="385" spans="1:4" ht="15.75" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A385" s="6">
-        <v>90705</v>
+        <v>90683</v>
       </c>
       <c r="B385" t="s">
-        <v>320</v>
+        <v>319</v>
       </c>
       <c r="C385" s="1" t="s">
         <v>4</v>
@@ -6984,10 +6987,10 @@
     </row>
     <row r="386" spans="1:4" ht="15.75" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A386" s="6">
-        <v>90706</v>
+        <v>90705</v>
       </c>
       <c r="B386" t="s">
-        <v>321</v>
+        <v>320</v>
       </c>
       <c r="C386" s="1" t="s">
         <v>4</v>
@@ -6998,10 +7001,10 @@
     </row>
     <row r="387" spans="1:4" ht="15.75" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A387" s="6">
-        <v>90708</v>
+        <v>90706</v>
       </c>
       <c r="B387" t="s">
-        <v>322</v>
+        <v>321</v>
       </c>
       <c r="C387" s="1" t="s">
         <v>4</v>
@@ -7012,10 +7015,10 @@
     </row>
     <row r="388" spans="1:4" ht="15.75" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A388" s="6">
-        <v>90709</v>
+        <v>90708</v>
       </c>
       <c r="B388" t="s">
-        <v>323</v>
+        <v>322</v>
       </c>
       <c r="C388" s="1" t="s">
         <v>4</v>
@@ -7026,38 +7029,38 @@
     </row>
     <row r="389" spans="1:4" ht="15.75" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A389" s="6">
-        <v>90713</v>
+        <v>90709</v>
       </c>
       <c r="B389" t="s">
-        <v>402</v>
+        <v>323</v>
       </c>
       <c r="C389" s="1" t="s">
         <v>4</v>
       </c>
       <c r="D389" s="12" t="s">
-        <v>5</v>
+        <v>8</v>
       </c>
     </row>
     <row r="390" spans="1:4" ht="15.75" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A390" s="6">
-        <v>1218</v>
+        <v>90713</v>
       </c>
       <c r="B390" t="s">
-        <v>382</v>
+        <v>402</v>
       </c>
       <c r="C390" s="1" t="s">
         <v>4</v>
       </c>
       <c r="D390" s="12" t="s">
-        <v>8</v>
+        <v>5</v>
       </c>
     </row>
     <row r="391" spans="1:4" ht="15.75" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A391" s="6">
-        <v>1959</v>
-      </c>
-      <c r="B391" s="8" t="s">
-        <v>383</v>
+        <v>1218</v>
+      </c>
+      <c r="B391" t="s">
+        <v>382</v>
       </c>
       <c r="C391" s="1" t="s">
         <v>4</v>
@@ -7068,10 +7071,10 @@
     </row>
     <row r="392" spans="1:4" ht="15.75" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A392" s="6">
-        <v>5625</v>
+        <v>1959</v>
       </c>
       <c r="B392" s="8" t="s">
-        <v>384</v>
+        <v>383</v>
       </c>
       <c r="C392" s="1" t="s">
         <v>4</v>
@@ -7082,10 +7085,10 @@
     </row>
     <row r="393" spans="1:4" ht="15.75" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A393" s="6">
-        <v>1817</v>
+        <v>5625</v>
       </c>
       <c r="B393" s="8" t="s">
-        <v>389</v>
+        <v>384</v>
       </c>
       <c r="C393" s="1" t="s">
         <v>4</v>
@@ -7096,10 +7099,10 @@
     </row>
     <row r="394" spans="1:4" ht="15.75" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A394" s="6">
-        <v>5737</v>
+        <v>1817</v>
       </c>
       <c r="B394" s="8" t="s">
-        <v>390</v>
+        <v>389</v>
       </c>
       <c r="C394" s="1" t="s">
         <v>4</v>
@@ -7110,29 +7113,43 @@
     </row>
     <row r="395" spans="1:4" ht="15.75" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A395" s="6">
-        <v>60295</v>
+        <v>5737</v>
       </c>
       <c r="B395" s="8" t="s">
-        <v>385</v>
+        <v>390</v>
       </c>
       <c r="C395" s="1" t="s">
         <v>4</v>
       </c>
-      <c r="D395" s="9" t="s">
-        <v>9</v>
+      <c r="D395" s="12" t="s">
+        <v>8</v>
       </c>
     </row>
     <row r="396" spans="1:4" ht="15.75" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A396" s="6">
+        <v>60295</v>
+      </c>
+      <c r="B396" s="8" t="s">
+        <v>385</v>
+      </c>
+      <c r="C396" s="1" t="s">
+        <v>4</v>
+      </c>
+      <c r="D396" s="9" t="s">
+        <v>9</v>
+      </c>
+    </row>
+    <row r="397" spans="1:4" ht="15.75" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
+      <c r="A397" s="6">
         <v>1045</v>
       </c>
-      <c r="B396" s="8" t="s">
+      <c r="B397" s="8" t="s">
         <v>386</v>
       </c>
-      <c r="C396" s="1" t="s">
-        <v>4</v>
-      </c>
-      <c r="D396" s="9" t="s">
+      <c r="C397" s="1" t="s">
+        <v>4</v>
+      </c>
+      <c r="D397" s="9" t="s">
         <v>5</v>
       </c>
     </row>

</xml_diff>

<commit_message>
habilite cuenta 40147,update estado de cuentas 23-6-26
</commit_message>
<xml_diff>
--- a/excel/CLIENTES_PERMISOS.xlsx
+++ b/excel/CLIENTES_PERMISOS.xlsx
@@ -15,14 +15,14 @@
     <sheet name="Hoja 1" sheetId="1" r:id="rId1"/>
   </sheets>
   <definedNames>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'Hoja 1'!$A$1:$D$343</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'Hoja 1'!$A$1:$D$344</definedName>
   </definedNames>
   <calcPr calcId="162913"/>
 </workbook>
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="1195" uniqueCount="405">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="1198" uniqueCount="406">
   <si>
     <t>CUENTA</t>
   </si>
@@ -1237,6 +1237,9 @@
   </si>
   <si>
     <t>FERRETERIA BAUPI</t>
+  </si>
+  <si>
+    <t>ATR FERRETERIA</t>
   </si>
 </sst>
 </file>
@@ -1319,7 +1322,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="19">
+  <cellXfs count="20">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment wrapText="1"/>
@@ -1361,6 +1364,7 @@
     </xf>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1"/>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="2" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1"/>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
@@ -1590,7 +1594,7 @@
   <sheetPr>
     <outlinePr summaryBelow="0" summaryRight="0"/>
   </sheetPr>
-  <dimension ref="A1:D398"/>
+  <dimension ref="A1:D399"/>
   <sheetFormatPr baseColWidth="10" defaultColWidth="12.5703125" defaultRowHeight="15.75" customHeight="1" x14ac:dyDescent="0.2"/>
   <cols>
     <col min="2" max="2" width="34" customWidth="1"/>
@@ -4848,192 +4852,192 @@
     </row>
     <row r="233" spans="1:4" ht="15.75" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A233" s="6">
-        <v>40150</v>
+        <v>40147</v>
       </c>
       <c r="B233" t="s">
-        <v>221</v>
+        <v>405</v>
       </c>
       <c r="C233" s="1" t="s">
         <v>4</v>
       </c>
-      <c r="D233" s="10" t="s">
+      <c r="D233" s="19" t="s">
         <v>8</v>
       </c>
     </row>
     <row r="234" spans="1:4" ht="15.75" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A234" s="6">
-        <v>40151</v>
+        <v>40150</v>
       </c>
       <c r="B234" t="s">
-        <v>54</v>
+        <v>221</v>
       </c>
       <c r="C234" s="1" t="s">
         <v>4</v>
       </c>
-      <c r="D234" s="1" t="s">
+      <c r="D234" s="10" t="s">
         <v>8</v>
       </c>
     </row>
     <row r="235" spans="1:4" ht="15.75" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A235" s="6">
-        <v>50102</v>
+        <v>40151</v>
       </c>
       <c r="B235" t="s">
-        <v>67</v>
+        <v>54</v>
       </c>
       <c r="C235" s="1" t="s">
         <v>4</v>
       </c>
-      <c r="D235" s="13" t="s">
-        <v>5</v>
+      <c r="D235" s="1" t="s">
+        <v>8</v>
       </c>
     </row>
     <row r="236" spans="1:4" ht="15.75" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A236" s="6">
-        <v>50222</v>
+        <v>50102</v>
       </c>
       <c r="B236" t="s">
-        <v>215</v>
+        <v>67</v>
       </c>
       <c r="C236" s="1" t="s">
         <v>4</v>
       </c>
-      <c r="D236" s="1" t="s">
-        <v>8</v>
+      <c r="D236" s="13" t="s">
+        <v>5</v>
       </c>
     </row>
     <row r="237" spans="1:4" ht="15.75" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A237" s="6">
-        <v>50223</v>
+        <v>50222</v>
       </c>
       <c r="B237" t="s">
-        <v>194</v>
+        <v>215</v>
       </c>
       <c r="C237" s="1" t="s">
         <v>4</v>
       </c>
-      <c r="D237" s="10" t="s">
+      <c r="D237" s="1" t="s">
         <v>8</v>
       </c>
     </row>
     <row r="238" spans="1:4" ht="15.75" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A238" s="6">
-        <v>50224</v>
+        <v>50223</v>
       </c>
       <c r="B238" t="s">
-        <v>42</v>
+        <v>194</v>
       </c>
       <c r="C238" s="1" t="s">
         <v>4</v>
       </c>
-      <c r="D238" s="3" t="s">
-        <v>5</v>
+      <c r="D238" s="10" t="s">
+        <v>8</v>
       </c>
     </row>
     <row r="239" spans="1:4" ht="15.75" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A239" s="6">
-        <v>50444</v>
+        <v>50224</v>
       </c>
       <c r="B239" t="s">
-        <v>116</v>
+        <v>42</v>
       </c>
       <c r="C239" s="1" t="s">
         <v>4</v>
       </c>
-      <c r="D239" s="1" t="s">
-        <v>8</v>
+      <c r="D239" s="3" t="s">
+        <v>5</v>
       </c>
     </row>
     <row r="240" spans="1:4" ht="15.75" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A240" s="6">
-        <v>50445</v>
+        <v>50444</v>
       </c>
       <c r="B240" t="s">
-        <v>354</v>
+        <v>116</v>
       </c>
       <c r="C240" s="1" t="s">
         <v>4</v>
       </c>
-      <c r="D240" s="11" t="s">
-        <v>5</v>
+      <c r="D240" s="1" t="s">
+        <v>8</v>
       </c>
     </row>
     <row r="241" spans="1:4" ht="15.75" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A241" s="6">
-        <v>50607</v>
+        <v>50445</v>
       </c>
       <c r="B241" t="s">
-        <v>76</v>
+        <v>354</v>
       </c>
       <c r="C241" s="1" t="s">
         <v>4</v>
       </c>
-      <c r="D241" s="13" t="s">
+      <c r="D241" s="11" t="s">
         <v>5</v>
       </c>
     </row>
     <row r="242" spans="1:4" ht="15.75" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A242" s="6">
-        <v>50608</v>
+        <v>50607</v>
       </c>
       <c r="B242" t="s">
-        <v>177</v>
+        <v>76</v>
       </c>
       <c r="C242" s="1" t="s">
         <v>4</v>
       </c>
-      <c r="D242" s="1" t="s">
-        <v>8</v>
+      <c r="D242" s="13" t="s">
+        <v>5</v>
       </c>
     </row>
     <row r="243" spans="1:4" ht="15.75" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A243" s="6">
-        <v>50611</v>
-      </c>
-      <c r="B243" s="8" t="s">
-        <v>347</v>
+        <v>50608</v>
+      </c>
+      <c r="B243" t="s">
+        <v>177</v>
       </c>
       <c r="C243" s="1" t="s">
         <v>4</v>
       </c>
-      <c r="D243" s="14" t="s">
+      <c r="D243" s="1" t="s">
         <v>8</v>
       </c>
     </row>
     <row r="244" spans="1:4" ht="15.75" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A244" s="6">
-        <v>50622</v>
-      </c>
-      <c r="B244" t="s">
-        <v>95</v>
+        <v>50611</v>
+      </c>
+      <c r="B244" s="8" t="s">
+        <v>347</v>
       </c>
       <c r="C244" s="1" t="s">
         <v>4</v>
       </c>
-      <c r="D244" s="16" t="s">
+      <c r="D244" s="14" t="s">
         <v>8</v>
       </c>
     </row>
     <row r="245" spans="1:4" ht="15.75" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A245" s="6">
-        <v>50623</v>
+        <v>50622</v>
       </c>
       <c r="B245" t="s">
-        <v>110</v>
+        <v>95</v>
       </c>
       <c r="C245" s="1" t="s">
         <v>4</v>
       </c>
-      <c r="D245" s="10" t="s">
+      <c r="D245" s="16" t="s">
         <v>8</v>
       </c>
     </row>
     <row r="246" spans="1:4" ht="15.75" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A246" s="6">
-        <v>50625</v>
+        <v>50623</v>
       </c>
       <c r="B246" t="s">
-        <v>204</v>
+        <v>110</v>
       </c>
       <c r="C246" s="1" t="s">
         <v>4</v>
@@ -5044,94 +5048,94 @@
     </row>
     <row r="247" spans="1:4" ht="15.75" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A247" s="6">
-        <v>50629</v>
+        <v>50625</v>
       </c>
       <c r="B247" t="s">
-        <v>188</v>
+        <v>204</v>
       </c>
       <c r="C247" s="1" t="s">
         <v>4</v>
       </c>
-      <c r="D247" s="1" t="s">
+      <c r="D247" s="10" t="s">
         <v>8</v>
       </c>
     </row>
     <row r="248" spans="1:4" ht="15.75" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A248" s="6">
-        <v>50630</v>
+        <v>50629</v>
       </c>
       <c r="B248" t="s">
-        <v>360</v>
+        <v>188</v>
       </c>
       <c r="C248" s="1" t="s">
         <v>4</v>
       </c>
-      <c r="D248" s="14" t="s">
+      <c r="D248" s="1" t="s">
         <v>8</v>
       </c>
     </row>
     <row r="249" spans="1:4" ht="15.75" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A249" s="6">
-        <v>50803</v>
+        <v>50630</v>
       </c>
       <c r="B249" t="s">
-        <v>82</v>
+        <v>360</v>
       </c>
       <c r="C249" s="1" t="s">
         <v>4</v>
       </c>
-      <c r="D249" s="1" t="s">
+      <c r="D249" s="14" t="s">
         <v>8</v>
       </c>
     </row>
     <row r="250" spans="1:4" ht="15.75" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A250" s="6">
-        <v>50805</v>
+        <v>50803</v>
       </c>
       <c r="B250" t="s">
-        <v>135</v>
+        <v>82</v>
       </c>
       <c r="C250" s="1" t="s">
         <v>4</v>
       </c>
-      <c r="D250" s="10" t="s">
+      <c r="D250" s="1" t="s">
         <v>8</v>
       </c>
     </row>
     <row r="251" spans="1:4" ht="15.75" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A251" s="6">
-        <v>50806</v>
+        <v>50805</v>
       </c>
       <c r="B251" t="s">
-        <v>156</v>
+        <v>135</v>
       </c>
       <c r="C251" s="1" t="s">
         <v>4</v>
       </c>
-      <c r="D251" s="1" t="s">
+      <c r="D251" s="10" t="s">
         <v>8</v>
       </c>
     </row>
     <row r="252" spans="1:4" ht="15.75" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A252" s="6">
-        <v>50808</v>
+        <v>50806</v>
       </c>
       <c r="B252" t="s">
-        <v>16</v>
+        <v>156</v>
       </c>
       <c r="C252" s="1" t="s">
         <v>4</v>
       </c>
-      <c r="D252" s="13" t="s">
-        <v>5</v>
+      <c r="D252" s="1" t="s">
+        <v>8</v>
       </c>
     </row>
     <row r="253" spans="1:4" ht="15.75" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A253" s="6">
-        <v>50809</v>
+        <v>50808</v>
       </c>
       <c r="B253" t="s">
-        <v>98</v>
+        <v>16</v>
       </c>
       <c r="C253" s="1" t="s">
         <v>4</v>
@@ -5142,24 +5146,24 @@
     </row>
     <row r="254" spans="1:4" ht="15.75" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A254" s="6">
-        <v>50810</v>
+        <v>50809</v>
       </c>
       <c r="B254" t="s">
-        <v>175</v>
+        <v>98</v>
       </c>
       <c r="C254" s="1" t="s">
         <v>4</v>
       </c>
-      <c r="D254" s="1" t="s">
-        <v>8</v>
+      <c r="D254" s="13" t="s">
+        <v>5</v>
       </c>
     </row>
     <row r="255" spans="1:4" ht="15.75" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A255" s="6">
-        <v>50812</v>
+        <v>50810</v>
       </c>
       <c r="B255" t="s">
-        <v>184</v>
+        <v>175</v>
       </c>
       <c r="C255" s="1" t="s">
         <v>4</v>
@@ -5170,80 +5174,80 @@
     </row>
     <row r="256" spans="1:4" ht="15.75" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A256" s="6">
-        <v>50813</v>
+        <v>50812</v>
       </c>
       <c r="B256" t="s">
-        <v>71</v>
+        <v>184</v>
       </c>
       <c r="C256" s="1" t="s">
         <v>4</v>
       </c>
-      <c r="D256" s="17" t="s">
-        <v>9</v>
+      <c r="D256" s="1" t="s">
+        <v>8</v>
       </c>
     </row>
     <row r="257" spans="1:4" ht="15.75" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A257" s="6">
-        <v>50815</v>
+        <v>50813</v>
       </c>
       <c r="B257" t="s">
-        <v>114</v>
+        <v>71</v>
       </c>
       <c r="C257" s="1" t="s">
         <v>4</v>
       </c>
-      <c r="D257" s="10" t="s">
-        <v>8</v>
+      <c r="D257" s="17" t="s">
+        <v>9</v>
       </c>
     </row>
     <row r="258" spans="1:4" ht="15.75" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A258" s="6">
-        <v>50816</v>
+        <v>50815</v>
       </c>
       <c r="B258" t="s">
-        <v>205</v>
+        <v>114</v>
       </c>
       <c r="C258" s="1" t="s">
         <v>4</v>
       </c>
-      <c r="D258" s="1" t="s">
+      <c r="D258" s="10" t="s">
         <v>8</v>
       </c>
     </row>
     <row r="259" spans="1:4" ht="15.75" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A259" s="6">
-        <v>50818</v>
+        <v>50816</v>
       </c>
       <c r="B259" t="s">
-        <v>227</v>
+        <v>205</v>
       </c>
       <c r="C259" s="1" t="s">
         <v>4</v>
       </c>
-      <c r="D259" s="13" t="s">
-        <v>5</v>
+      <c r="D259" s="1" t="s">
+        <v>8</v>
       </c>
     </row>
     <row r="260" spans="1:4" ht="15.75" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A260" s="6">
-        <v>50819</v>
+        <v>50818</v>
       </c>
       <c r="B260" t="s">
-        <v>228</v>
+        <v>227</v>
       </c>
       <c r="C260" s="1" t="s">
         <v>4</v>
       </c>
-      <c r="D260" s="10" t="s">
-        <v>8</v>
+      <c r="D260" s="13" t="s">
+        <v>5</v>
       </c>
     </row>
     <row r="261" spans="1:4" ht="15.75" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A261" s="6">
-        <v>50820</v>
+        <v>50819</v>
       </c>
       <c r="B261" t="s">
-        <v>229</v>
+        <v>228</v>
       </c>
       <c r="C261" s="1" t="s">
         <v>4</v>
@@ -5254,66 +5258,66 @@
     </row>
     <row r="262" spans="1:4" ht="15.75" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A262" s="6">
-        <v>50821</v>
+        <v>50820</v>
       </c>
       <c r="B262" t="s">
-        <v>230</v>
+        <v>229</v>
       </c>
       <c r="C262" s="1" t="s">
         <v>4</v>
       </c>
-      <c r="D262" s="1" t="s">
+      <c r="D262" s="10" t="s">
         <v>8</v>
       </c>
     </row>
     <row r="263" spans="1:4" ht="15.75" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A263" s="6">
-        <v>50823</v>
+        <v>50821</v>
       </c>
       <c r="B263" t="s">
-        <v>231</v>
+        <v>230</v>
       </c>
       <c r="C263" s="1" t="s">
         <v>4</v>
       </c>
-      <c r="D263" s="17" t="s">
-        <v>9</v>
+      <c r="D263" s="1" t="s">
+        <v>8</v>
       </c>
     </row>
     <row r="264" spans="1:4" ht="15.75" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A264" s="6">
-        <v>50824</v>
+        <v>50823</v>
       </c>
       <c r="B264" t="s">
-        <v>232</v>
+        <v>231</v>
       </c>
       <c r="C264" s="1" t="s">
         <v>4</v>
       </c>
-      <c r="D264" s="13" t="s">
-        <v>5</v>
+      <c r="D264" s="17" t="s">
+        <v>9</v>
       </c>
     </row>
     <row r="265" spans="1:4" ht="15.75" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A265" s="6">
-        <v>50825</v>
+        <v>50824</v>
       </c>
       <c r="B265" t="s">
-        <v>233</v>
+        <v>232</v>
       </c>
       <c r="C265" s="1" t="s">
         <v>4</v>
       </c>
-      <c r="D265" s="10" t="s">
-        <v>8</v>
+      <c r="D265" s="13" t="s">
+        <v>5</v>
       </c>
     </row>
     <row r="266" spans="1:4" ht="15.75" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A266" s="6">
-        <v>50826</v>
+        <v>50825</v>
       </c>
       <c r="B266" t="s">
-        <v>234</v>
+        <v>233</v>
       </c>
       <c r="C266" s="1" t="s">
         <v>4</v>
@@ -5324,24 +5328,24 @@
     </row>
     <row r="267" spans="1:4" ht="15.75" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A267" s="6">
-        <v>50827</v>
+        <v>50826</v>
       </c>
       <c r="B267" t="s">
-        <v>235</v>
+        <v>234</v>
       </c>
       <c r="C267" s="1" t="s">
         <v>4</v>
       </c>
-      <c r="D267" s="1" t="s">
+      <c r="D267" s="10" t="s">
         <v>8</v>
       </c>
     </row>
     <row r="268" spans="1:4" ht="15.75" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A268" s="6">
-        <v>50829</v>
+        <v>50827</v>
       </c>
       <c r="B268" t="s">
-        <v>236</v>
+        <v>235</v>
       </c>
       <c r="C268" s="1" t="s">
         <v>4</v>
@@ -5352,122 +5356,122 @@
     </row>
     <row r="269" spans="1:4" ht="15.75" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A269" s="6">
-        <v>50830</v>
+        <v>50829</v>
       </c>
       <c r="B269" t="s">
-        <v>366</v>
+        <v>236</v>
       </c>
       <c r="C269" s="1" t="s">
         <v>4</v>
       </c>
-      <c r="D269" s="11" t="s">
+      <c r="D269" s="1" t="s">
         <v>8</v>
       </c>
     </row>
     <row r="270" spans="1:4" ht="15.75" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A270" s="6">
-        <v>50831</v>
+        <v>50830</v>
       </c>
       <c r="B270" t="s">
-        <v>351</v>
+        <v>366</v>
       </c>
       <c r="C270" s="1" t="s">
         <v>4</v>
       </c>
       <c r="D270" s="11" t="s">
-        <v>9</v>
+        <v>8</v>
       </c>
     </row>
     <row r="271" spans="1:4" ht="15.75" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A271" s="6">
-        <v>50832</v>
-      </c>
-      <c r="B271" s="8" t="s">
-        <v>349</v>
+        <v>50831</v>
+      </c>
+      <c r="B271" t="s">
+        <v>351</v>
       </c>
       <c r="C271" s="1" t="s">
         <v>4</v>
       </c>
       <c r="D271" s="11" t="s">
-        <v>5</v>
+        <v>9</v>
       </c>
     </row>
     <row r="272" spans="1:4" ht="15.75" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A272" s="6">
-        <v>50833</v>
+        <v>50832</v>
       </c>
       <c r="B272" s="8" t="s">
-        <v>397</v>
+        <v>349</v>
       </c>
       <c r="C272" s="1" t="s">
         <v>4</v>
       </c>
       <c r="D272" s="11" t="s">
-        <v>8</v>
+        <v>5</v>
       </c>
     </row>
     <row r="273" spans="1:4" ht="15.75" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A273" s="6">
-        <v>50230</v>
+        <v>50833</v>
       </c>
       <c r="B273" s="8" t="s">
-        <v>379</v>
+        <v>397</v>
       </c>
       <c r="C273" s="1" t="s">
         <v>4</v>
       </c>
       <c r="D273" s="11" t="s">
-        <v>5</v>
+        <v>8</v>
       </c>
     </row>
     <row r="274" spans="1:4" ht="15.75" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A274" s="6">
-        <v>60103</v>
-      </c>
-      <c r="B274" t="s">
-        <v>237</v>
+        <v>50230</v>
+      </c>
+      <c r="B274" s="8" t="s">
+        <v>379</v>
       </c>
       <c r="C274" s="1" t="s">
         <v>4</v>
       </c>
-      <c r="D274" s="13" t="s">
+      <c r="D274" s="11" t="s">
         <v>5</v>
       </c>
     </row>
     <row r="275" spans="1:4" ht="15.75" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A275" s="6">
-        <v>60109</v>
+        <v>60103</v>
       </c>
       <c r="B275" t="s">
-        <v>328</v>
+        <v>237</v>
       </c>
       <c r="C275" s="1" t="s">
         <v>4</v>
       </c>
-      <c r="D275" s="11" t="s">
-        <v>9</v>
+      <c r="D275" s="13" t="s">
+        <v>5</v>
       </c>
     </row>
     <row r="276" spans="1:4" ht="15.75" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A276" s="6">
-        <v>60124</v>
+        <v>60109</v>
       </c>
       <c r="B276" t="s">
-        <v>238</v>
+        <v>328</v>
       </c>
       <c r="C276" s="1" t="s">
         <v>4</v>
       </c>
-      <c r="D276" s="13" t="s">
-        <v>5</v>
+      <c r="D276" s="11" t="s">
+        <v>9</v>
       </c>
     </row>
     <row r="277" spans="1:4" ht="15.75" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A277" s="6">
-        <v>60125</v>
+        <v>60124</v>
       </c>
       <c r="B277" t="s">
-        <v>239</v>
+        <v>238</v>
       </c>
       <c r="C277" s="1" t="s">
         <v>4</v>
@@ -5478,80 +5482,80 @@
     </row>
     <row r="278" spans="1:4" ht="15.75" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A278" s="6">
-        <v>60126</v>
+        <v>60125</v>
       </c>
       <c r="B278" t="s">
-        <v>240</v>
+        <v>239</v>
       </c>
       <c r="C278" s="1" t="s">
         <v>4</v>
       </c>
-      <c r="D278" s="10" t="s">
-        <v>8</v>
+      <c r="D278" s="13" t="s">
+        <v>5</v>
       </c>
     </row>
     <row r="279" spans="1:4" ht="15.75" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A279" s="6">
-        <v>60128</v>
+        <v>60126</v>
       </c>
       <c r="B279" t="s">
-        <v>241</v>
+        <v>240</v>
       </c>
       <c r="C279" s="1" t="s">
         <v>4</v>
       </c>
-      <c r="D279" s="3" t="s">
-        <v>5</v>
+      <c r="D279" s="10" t="s">
+        <v>8</v>
       </c>
     </row>
     <row r="280" spans="1:4" ht="15.75" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A280" s="6">
-        <v>60130</v>
+        <v>60128</v>
       </c>
       <c r="B280" t="s">
-        <v>242</v>
+        <v>241</v>
       </c>
       <c r="C280" s="1" t="s">
         <v>4</v>
       </c>
-      <c r="D280" s="1" t="s">
-        <v>8</v>
+      <c r="D280" s="3" t="s">
+        <v>5</v>
       </c>
     </row>
     <row r="281" spans="1:4" ht="15.75" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A281" s="6">
-        <v>60133</v>
+        <v>60130</v>
       </c>
       <c r="B281" t="s">
-        <v>243</v>
+        <v>242</v>
       </c>
       <c r="C281" s="1" t="s">
         <v>4</v>
       </c>
-      <c r="D281" s="13" t="s">
-        <v>5</v>
+      <c r="D281" s="1" t="s">
+        <v>8</v>
       </c>
     </row>
     <row r="282" spans="1:4" ht="15.75" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A282" s="6">
-        <v>60134</v>
+        <v>60133</v>
       </c>
       <c r="B282" t="s">
-        <v>244</v>
+        <v>243</v>
       </c>
       <c r="C282" s="1" t="s">
         <v>4</v>
       </c>
-      <c r="D282" s="1" t="s">
-        <v>8</v>
+      <c r="D282" s="13" t="s">
+        <v>5</v>
       </c>
     </row>
     <row r="283" spans="1:4" ht="15.75" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A283" s="6">
-        <v>60137</v>
+        <v>60134</v>
       </c>
       <c r="B283" t="s">
-        <v>245</v>
+        <v>244</v>
       </c>
       <c r="C283" s="1" t="s">
         <v>4</v>
@@ -5562,10 +5566,10 @@
     </row>
     <row r="284" spans="1:4" ht="15.75" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A284" s="6">
-        <v>60139</v>
+        <v>60137</v>
       </c>
       <c r="B284" t="s">
-        <v>246</v>
+        <v>245</v>
       </c>
       <c r="C284" s="1" t="s">
         <v>4</v>
@@ -5576,10 +5580,10 @@
     </row>
     <row r="285" spans="1:4" ht="15.75" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A285" s="6">
-        <v>60142</v>
+        <v>60139</v>
       </c>
       <c r="B285" t="s">
-        <v>247</v>
+        <v>246</v>
       </c>
       <c r="C285" s="1" t="s">
         <v>4</v>
@@ -5590,10 +5594,10 @@
     </row>
     <row r="286" spans="1:4" ht="15.75" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A286" s="6">
-        <v>60148</v>
+        <v>60142</v>
       </c>
       <c r="B286" t="s">
-        <v>248</v>
+        <v>247</v>
       </c>
       <c r="C286" s="1" t="s">
         <v>4</v>
@@ -5604,10 +5608,10 @@
     </row>
     <row r="287" spans="1:4" ht="15.75" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A287" s="6">
-        <v>60149</v>
+        <v>60148</v>
       </c>
       <c r="B287" t="s">
-        <v>249</v>
+        <v>248</v>
       </c>
       <c r="C287" s="1" t="s">
         <v>4</v>
@@ -5618,66 +5622,66 @@
     </row>
     <row r="288" spans="1:4" ht="15.75" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A288" s="6">
-        <v>60150</v>
+        <v>60149</v>
       </c>
       <c r="B288" t="s">
-        <v>332</v>
+        <v>249</v>
       </c>
       <c r="C288" s="1" t="s">
         <v>4</v>
       </c>
-      <c r="D288" s="13" t="s">
-        <v>5</v>
+      <c r="D288" s="1" t="s">
+        <v>8</v>
       </c>
     </row>
     <row r="289" spans="1:4" ht="15.75" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A289" s="6">
-        <v>60158</v>
+        <v>60150</v>
       </c>
       <c r="B289" t="s">
-        <v>250</v>
+        <v>332</v>
       </c>
       <c r="C289" s="1" t="s">
         <v>4</v>
       </c>
-      <c r="D289" s="10" t="s">
-        <v>8</v>
+      <c r="D289" s="13" t="s">
+        <v>5</v>
       </c>
     </row>
     <row r="290" spans="1:4" ht="15.75" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A290" s="6">
-        <v>60159</v>
+        <v>60158</v>
       </c>
       <c r="B290" t="s">
-        <v>251</v>
+        <v>250</v>
       </c>
       <c r="C290" s="1" t="s">
         <v>4</v>
       </c>
-      <c r="D290" s="1" t="s">
+      <c r="D290" s="10" t="s">
         <v>8</v>
       </c>
     </row>
     <row r="291" spans="1:4" ht="15.75" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A291" s="6">
-        <v>60162</v>
+        <v>60159</v>
       </c>
       <c r="B291" t="s">
-        <v>252</v>
+        <v>251</v>
       </c>
       <c r="C291" s="1" t="s">
         <v>4</v>
       </c>
-      <c r="D291" s="13" t="s">
-        <v>5</v>
+      <c r="D291" s="1" t="s">
+        <v>8</v>
       </c>
     </row>
     <row r="292" spans="1:4" ht="15.75" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A292" s="6">
-        <v>60163</v>
+        <v>60162</v>
       </c>
       <c r="B292" t="s">
-        <v>253</v>
+        <v>252</v>
       </c>
       <c r="C292" s="1" t="s">
         <v>4</v>
@@ -5688,24 +5692,24 @@
     </row>
     <row r="293" spans="1:4" ht="15.75" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A293" s="6">
-        <v>60165</v>
+        <v>60163</v>
       </c>
       <c r="B293" t="s">
-        <v>254</v>
+        <v>253</v>
       </c>
       <c r="C293" s="1" t="s">
         <v>4</v>
       </c>
-      <c r="D293" s="1" t="s">
-        <v>8</v>
+      <c r="D293" s="13" t="s">
+        <v>5</v>
       </c>
     </row>
     <row r="294" spans="1:4" ht="15.75" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A294" s="6">
-        <v>60169</v>
+        <v>60165</v>
       </c>
       <c r="B294" t="s">
-        <v>255</v>
+        <v>254</v>
       </c>
       <c r="C294" s="1" t="s">
         <v>4</v>
@@ -5716,52 +5720,52 @@
     </row>
     <row r="295" spans="1:4" ht="15.75" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A295" s="6">
-        <v>60170</v>
-      </c>
-      <c r="B295" s="8" t="s">
-        <v>337</v>
+        <v>60169</v>
+      </c>
+      <c r="B295" t="s">
+        <v>255</v>
       </c>
       <c r="C295" s="1" t="s">
         <v>4</v>
       </c>
-      <c r="D295" s="11" t="s">
+      <c r="D295" s="1" t="s">
         <v>8</v>
       </c>
     </row>
     <row r="296" spans="1:4" ht="15.75" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A296" s="6">
-        <v>60172</v>
-      </c>
-      <c r="B296" t="s">
-        <v>256</v>
+        <v>60170</v>
+      </c>
+      <c r="B296" s="8" t="s">
+        <v>337</v>
       </c>
       <c r="C296" s="1" t="s">
         <v>4</v>
       </c>
-      <c r="D296" s="1" t="s">
+      <c r="D296" s="11" t="s">
         <v>8</v>
       </c>
     </row>
     <row r="297" spans="1:4" ht="15.75" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A297" s="6">
-        <v>60174</v>
+        <v>60172</v>
       </c>
       <c r="B297" t="s">
-        <v>257</v>
+        <v>256</v>
       </c>
       <c r="C297" s="1" t="s">
         <v>4</v>
       </c>
-      <c r="D297" s="13" t="s">
-        <v>5</v>
+      <c r="D297" s="1" t="s">
+        <v>8</v>
       </c>
     </row>
     <row r="298" spans="1:4" ht="15.75" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A298" s="6">
-        <v>60176</v>
+        <v>60174</v>
       </c>
       <c r="B298" t="s">
-        <v>258</v>
+        <v>257</v>
       </c>
       <c r="C298" s="1" t="s">
         <v>4</v>
@@ -5772,52 +5776,52 @@
     </row>
     <row r="299" spans="1:4" ht="15.75" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A299" s="6">
-        <v>60178</v>
+        <v>60176</v>
       </c>
       <c r="B299" t="s">
-        <v>259</v>
+        <v>258</v>
       </c>
       <c r="C299" s="1" t="s">
         <v>4</v>
       </c>
-      <c r="D299" s="1" t="s">
-        <v>8</v>
+      <c r="D299" s="13" t="s">
+        <v>5</v>
       </c>
     </row>
     <row r="300" spans="1:4" ht="15.75" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A300" s="6">
-        <v>60180</v>
+        <v>60178</v>
       </c>
       <c r="B300" t="s">
-        <v>260</v>
+        <v>259</v>
       </c>
       <c r="C300" s="1" t="s">
         <v>4</v>
       </c>
-      <c r="D300" s="10" t="s">
+      <c r="D300" s="1" t="s">
         <v>8</v>
       </c>
     </row>
     <row r="301" spans="1:4" ht="15.75" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A301" s="6">
-        <v>60184</v>
+        <v>60180</v>
       </c>
       <c r="B301" t="s">
-        <v>261</v>
+        <v>260</v>
       </c>
       <c r="C301" s="1" t="s">
         <v>4</v>
       </c>
-      <c r="D301" s="1" t="s">
+      <c r="D301" s="10" t="s">
         <v>8</v>
       </c>
     </row>
     <row r="302" spans="1:4" ht="15.75" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A302" s="6">
-        <v>60190</v>
+        <v>60184</v>
       </c>
       <c r="B302" t="s">
-        <v>262</v>
+        <v>261</v>
       </c>
       <c r="C302" s="1" t="s">
         <v>4</v>
@@ -5828,24 +5832,24 @@
     </row>
     <row r="303" spans="1:4" ht="15.75" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A303" s="6">
-        <v>60191</v>
+        <v>60190</v>
       </c>
       <c r="B303" t="s">
-        <v>263</v>
+        <v>262</v>
       </c>
       <c r="C303" s="1" t="s">
         <v>4</v>
       </c>
-      <c r="D303" s="10" t="s">
+      <c r="D303" s="1" t="s">
         <v>8</v>
       </c>
     </row>
     <row r="304" spans="1:4" ht="15.75" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A304" s="6">
-        <v>60192</v>
+        <v>60191</v>
       </c>
       <c r="B304" t="s">
-        <v>264</v>
+        <v>263</v>
       </c>
       <c r="C304" s="1" t="s">
         <v>4</v>
@@ -5856,10 +5860,10 @@
     </row>
     <row r="305" spans="1:4" ht="15.75" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A305" s="6">
-        <v>60195</v>
+        <v>60192</v>
       </c>
       <c r="B305" t="s">
-        <v>265</v>
+        <v>264</v>
       </c>
       <c r="C305" s="1" t="s">
         <v>4</v>
@@ -5870,10 +5874,10 @@
     </row>
     <row r="306" spans="1:4" ht="15.75" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A306" s="6">
-        <v>60196</v>
+        <v>60195</v>
       </c>
       <c r="B306" t="s">
-        <v>266</v>
+        <v>265</v>
       </c>
       <c r="C306" s="1" t="s">
         <v>4</v>
@@ -5884,10 +5888,10 @@
     </row>
     <row r="307" spans="1:4" ht="15.75" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A307" s="6">
-        <v>60198</v>
+        <v>60196</v>
       </c>
       <c r="B307" t="s">
-        <v>267</v>
+        <v>266</v>
       </c>
       <c r="C307" s="1" t="s">
         <v>4</v>
@@ -5898,52 +5902,52 @@
     </row>
     <row r="308" spans="1:4" ht="15.75" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A308" s="6">
-        <v>60201</v>
+        <v>60198</v>
       </c>
       <c r="B308" t="s">
-        <v>268</v>
+        <v>267</v>
       </c>
       <c r="C308" s="1" t="s">
         <v>4</v>
       </c>
-      <c r="D308" t="s">
-        <v>9</v>
+      <c r="D308" s="10" t="s">
+        <v>8</v>
       </c>
     </row>
     <row r="309" spans="1:4" ht="15.75" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A309" s="6">
-        <v>60202</v>
+        <v>60201</v>
       </c>
       <c r="B309" t="s">
-        <v>269</v>
+        <v>268</v>
       </c>
       <c r="C309" s="1" t="s">
         <v>4</v>
       </c>
-      <c r="D309" s="13" t="s">
-        <v>5</v>
+      <c r="D309" t="s">
+        <v>9</v>
       </c>
     </row>
     <row r="310" spans="1:4" ht="15.75" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A310" s="6">
-        <v>60204</v>
+        <v>60202</v>
       </c>
       <c r="B310" t="s">
-        <v>270</v>
+        <v>269</v>
       </c>
       <c r="C310" s="1" t="s">
         <v>4</v>
       </c>
-      <c r="D310" s="1" t="s">
-        <v>8</v>
+      <c r="D310" s="13" t="s">
+        <v>5</v>
       </c>
     </row>
     <row r="311" spans="1:4" ht="15.75" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A311" s="6">
-        <v>60205</v>
+        <v>60204</v>
       </c>
       <c r="B311" t="s">
-        <v>271</v>
+        <v>270</v>
       </c>
       <c r="C311" s="1" t="s">
         <v>4</v>
@@ -5954,10 +5958,10 @@
     </row>
     <row r="312" spans="1:4" ht="15.75" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A312" s="6">
-        <v>60206</v>
+        <v>60205</v>
       </c>
       <c r="B312" t="s">
-        <v>272</v>
+        <v>271</v>
       </c>
       <c r="C312" s="1" t="s">
         <v>4</v>
@@ -5968,220 +5972,220 @@
     </row>
     <row r="313" spans="1:4" ht="15.75" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A313" s="6">
-        <v>60209</v>
+        <v>60206</v>
       </c>
       <c r="B313" t="s">
-        <v>273</v>
+        <v>272</v>
       </c>
       <c r="C313" s="1" t="s">
         <v>4</v>
       </c>
-      <c r="D313" s="10" t="s">
+      <c r="D313" s="1" t="s">
         <v>8</v>
       </c>
     </row>
     <row r="314" spans="1:4" ht="15.75" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A314" s="6">
-        <v>60211</v>
+        <v>60209</v>
       </c>
       <c r="B314" t="s">
-        <v>274</v>
+        <v>273</v>
       </c>
       <c r="C314" s="1" t="s">
         <v>4</v>
       </c>
-      <c r="D314" s="1" t="s">
+      <c r="D314" s="10" t="s">
         <v>8</v>
       </c>
     </row>
     <row r="315" spans="1:4" ht="15.75" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A315" s="6">
-        <v>60215</v>
+        <v>60211</v>
       </c>
       <c r="B315" t="s">
-        <v>275</v>
+        <v>274</v>
       </c>
       <c r="C315" s="1" t="s">
         <v>4</v>
       </c>
-      <c r="D315" s="10" t="s">
+      <c r="D315" s="1" t="s">
         <v>8</v>
       </c>
     </row>
     <row r="316" spans="1:4" ht="15.75" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A316" s="6">
-        <v>60216</v>
+        <v>60215</v>
       </c>
       <c r="B316" t="s">
-        <v>381</v>
+        <v>275</v>
       </c>
       <c r="C316" s="1" t="s">
         <v>4</v>
       </c>
       <c r="D316" s="10" t="s">
-        <v>9</v>
+        <v>8</v>
       </c>
     </row>
     <row r="317" spans="1:4" ht="15.75" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A317" s="6">
-        <v>60217</v>
+        <v>60216</v>
       </c>
       <c r="B317" t="s">
-        <v>276</v>
+        <v>381</v>
       </c>
       <c r="C317" s="1" t="s">
         <v>4</v>
       </c>
       <c r="D317" s="10" t="s">
-        <v>8</v>
+        <v>9</v>
       </c>
     </row>
     <row r="318" spans="1:4" ht="15.75" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A318" s="6">
-        <v>60219</v>
+        <v>60217</v>
       </c>
       <c r="B318" t="s">
-        <v>277</v>
+        <v>276</v>
       </c>
       <c r="C318" s="1" t="s">
         <v>4</v>
       </c>
-      <c r="D318" s="1" t="s">
+      <c r="D318" s="10" t="s">
         <v>8</v>
       </c>
     </row>
     <row r="319" spans="1:4" ht="15.75" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A319" s="6">
-        <v>60222</v>
+        <v>60219</v>
       </c>
       <c r="B319" t="s">
-        <v>278</v>
+        <v>277</v>
       </c>
       <c r="C319" s="1" t="s">
         <v>4</v>
       </c>
-      <c r="D319" s="10" t="s">
+      <c r="D319" s="1" t="s">
         <v>8</v>
       </c>
     </row>
     <row r="320" spans="1:4" ht="15.75" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A320" s="6">
-        <v>60225</v>
+        <v>60222</v>
       </c>
       <c r="B320" t="s">
-        <v>279</v>
+        <v>278</v>
       </c>
       <c r="C320" s="1" t="s">
         <v>4</v>
       </c>
-      <c r="D320" s="17" t="s">
-        <v>9</v>
+      <c r="D320" s="10" t="s">
+        <v>8</v>
       </c>
     </row>
     <row r="321" spans="1:4" ht="15.75" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A321" s="6">
-        <v>60230</v>
+        <v>60225</v>
       </c>
       <c r="B321" t="s">
-        <v>280</v>
+        <v>279</v>
       </c>
       <c r="C321" s="1" t="s">
         <v>4</v>
       </c>
-      <c r="D321" s="10" t="s">
-        <v>8</v>
+      <c r="D321" s="17" t="s">
+        <v>9</v>
       </c>
     </row>
     <row r="322" spans="1:4" ht="15.75" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A322" s="6">
-        <v>60241</v>
-      </c>
-      <c r="B322" s="8" t="s">
-        <v>338</v>
+        <v>60230</v>
+      </c>
+      <c r="B322" t="s">
+        <v>280</v>
       </c>
       <c r="C322" s="1" t="s">
         <v>4</v>
       </c>
-      <c r="D322" s="7" t="s">
-        <v>9</v>
+      <c r="D322" s="10" t="s">
+        <v>8</v>
       </c>
     </row>
     <row r="323" spans="1:4" ht="15.75" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A323" s="6">
-        <v>60242</v>
+        <v>60241</v>
       </c>
       <c r="B323" s="8" t="s">
-        <v>341</v>
+        <v>338</v>
       </c>
       <c r="C323" s="1" t="s">
         <v>4</v>
       </c>
       <c r="D323" s="7" t="s">
-        <v>5</v>
+        <v>9</v>
       </c>
     </row>
     <row r="324" spans="1:4" ht="15.75" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A324" s="6">
-        <v>60243</v>
+        <v>60242</v>
       </c>
       <c r="B324" s="8" t="s">
-        <v>395</v>
+        <v>341</v>
       </c>
       <c r="C324" s="1" t="s">
         <v>4</v>
       </c>
       <c r="D324" s="7" t="s">
-        <v>9</v>
+        <v>5</v>
       </c>
     </row>
     <row r="325" spans="1:4" ht="15.75" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A325" s="6">
-        <v>60245</v>
+        <v>60243</v>
       </c>
       <c r="B325" s="8" t="s">
-        <v>387</v>
+        <v>395</v>
       </c>
       <c r="C325" s="1" t="s">
         <v>4</v>
       </c>
       <c r="D325" s="7" t="s">
-        <v>5</v>
+        <v>9</v>
       </c>
     </row>
     <row r="326" spans="1:4" ht="15.75" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A326" s="6">
-        <v>60250</v>
+        <v>60245</v>
       </c>
       <c r="B326" s="8" t="s">
-        <v>339</v>
+        <v>387</v>
       </c>
       <c r="C326" s="1" t="s">
         <v>4</v>
       </c>
-      <c r="D326" s="11" t="s">
-        <v>8</v>
+      <c r="D326" s="7" t="s">
+        <v>5</v>
       </c>
     </row>
     <row r="327" spans="1:4" ht="15.75" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A327" s="6">
-        <v>60253</v>
-      </c>
-      <c r="B327" t="s">
-        <v>281</v>
+        <v>60250</v>
+      </c>
+      <c r="B327" s="8" t="s">
+        <v>339</v>
       </c>
       <c r="C327" s="1" t="s">
         <v>4</v>
       </c>
-      <c r="D327" s="1" t="s">
+      <c r="D327" s="11" t="s">
         <v>8</v>
       </c>
     </row>
     <row r="328" spans="1:4" ht="15.75" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A328" s="6">
-        <v>60254</v>
+        <v>60253</v>
       </c>
       <c r="B328" t="s">
-        <v>282</v>
+        <v>281</v>
       </c>
       <c r="C328" s="1" t="s">
         <v>4</v>
@@ -6192,10 +6196,10 @@
     </row>
     <row r="329" spans="1:4" ht="15.75" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A329" s="6">
-        <v>60257</v>
+        <v>60254</v>
       </c>
       <c r="B329" t="s">
-        <v>283</v>
+        <v>282</v>
       </c>
       <c r="C329" s="1" t="s">
         <v>4</v>
@@ -6206,10 +6210,10 @@
     </row>
     <row r="330" spans="1:4" ht="15.75" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A330" s="6">
-        <v>60258</v>
+        <v>60257</v>
       </c>
       <c r="B330" t="s">
-        <v>284</v>
+        <v>283</v>
       </c>
       <c r="C330" s="1" t="s">
         <v>4</v>
@@ -6220,66 +6224,66 @@
     </row>
     <row r="331" spans="1:4" ht="15.75" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A331" s="6">
-        <v>60266</v>
-      </c>
-      <c r="B331" s="8" t="s">
-        <v>343</v>
+        <v>60258</v>
+      </c>
+      <c r="B331" t="s">
+        <v>284</v>
       </c>
       <c r="C331" s="1" t="s">
         <v>4</v>
       </c>
-      <c r="D331" s="11" t="s">
+      <c r="D331" s="1" t="s">
         <v>8</v>
       </c>
     </row>
     <row r="332" spans="1:4" ht="15.75" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A332" s="6">
-        <v>60269</v>
-      </c>
-      <c r="B332" t="s">
-        <v>285</v>
+        <v>60266</v>
+      </c>
+      <c r="B332" s="8" t="s">
+        <v>343</v>
       </c>
       <c r="C332" s="1" t="s">
         <v>4</v>
       </c>
-      <c r="D332" s="10" t="s">
+      <c r="D332" s="11" t="s">
         <v>8</v>
       </c>
     </row>
     <row r="333" spans="1:4" ht="15.75" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A333" s="6">
-        <v>60270</v>
+        <v>60269</v>
       </c>
       <c r="B333" t="s">
-        <v>286</v>
+        <v>285</v>
       </c>
       <c r="C333" s="1" t="s">
         <v>4</v>
       </c>
-      <c r="D333" s="1" t="s">
-        <v>9</v>
+      <c r="D333" s="10" t="s">
+        <v>8</v>
       </c>
     </row>
     <row r="334" spans="1:4" ht="15.75" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A334" s="6">
-        <v>60272</v>
+        <v>60270</v>
       </c>
       <c r="B334" t="s">
-        <v>287</v>
+        <v>286</v>
       </c>
       <c r="C334" s="1" t="s">
         <v>4</v>
       </c>
       <c r="D334" s="1" t="s">
-        <v>8</v>
+        <v>9</v>
       </c>
     </row>
     <row r="335" spans="1:4" ht="15.75" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A335" s="6">
-        <v>60274</v>
+        <v>60272</v>
       </c>
       <c r="B335" t="s">
-        <v>380</v>
+        <v>287</v>
       </c>
       <c r="C335" s="1" t="s">
         <v>4</v>
@@ -6290,10 +6294,10 @@
     </row>
     <row r="336" spans="1:4" ht="15.75" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A336" s="6">
-        <v>60275</v>
+        <v>60274</v>
       </c>
       <c r="B336" t="s">
-        <v>288</v>
+        <v>380</v>
       </c>
       <c r="C336" s="1" t="s">
         <v>4</v>
@@ -6304,10 +6308,10 @@
     </row>
     <row r="337" spans="1:4" ht="15.75" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A337" s="6">
-        <v>60276</v>
+        <v>60275</v>
       </c>
       <c r="B337" t="s">
-        <v>289</v>
+        <v>288</v>
       </c>
       <c r="C337" s="1" t="s">
         <v>4</v>
@@ -6318,108 +6322,108 @@
     </row>
     <row r="338" spans="1:4" ht="15.75" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A338" s="6">
-        <v>60278</v>
+        <v>60276</v>
       </c>
       <c r="B338" t="s">
-        <v>290</v>
+        <v>289</v>
       </c>
       <c r="C338" s="1" t="s">
         <v>4</v>
       </c>
-      <c r="D338" s="13" t="s">
+      <c r="D338" s="1" t="s">
         <v>8</v>
       </c>
     </row>
     <row r="339" spans="1:4" ht="15.75" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A339" s="6">
-        <v>60279</v>
+        <v>60278</v>
       </c>
       <c r="B339" t="s">
-        <v>291</v>
+        <v>290</v>
       </c>
       <c r="C339" s="1" t="s">
         <v>4</v>
       </c>
-      <c r="D339" s="1" t="s">
+      <c r="D339" s="13" t="s">
         <v>8</v>
       </c>
     </row>
     <row r="340" spans="1:4" ht="15.75" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A340" s="6">
-        <v>60280</v>
+        <v>60279</v>
       </c>
       <c r="B340" t="s">
-        <v>292</v>
+        <v>291</v>
       </c>
       <c r="C340" s="1" t="s">
         <v>4</v>
       </c>
       <c r="D340" s="1" t="s">
-        <v>5</v>
+        <v>8</v>
       </c>
     </row>
     <row r="341" spans="1:4" ht="15.75" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A341" s="6">
-        <v>60281</v>
-      </c>
-      <c r="B341" s="8" t="s">
-        <v>336</v>
+        <v>60280</v>
+      </c>
+      <c r="B341" t="s">
+        <v>292</v>
       </c>
       <c r="C341" s="1" t="s">
         <v>4</v>
       </c>
-      <c r="D341" s="11" t="s">
-        <v>9</v>
+      <c r="D341" s="1" t="s">
+        <v>5</v>
       </c>
     </row>
     <row r="342" spans="1:4" ht="15.75" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A342" s="6">
-        <v>60282</v>
+        <v>60281</v>
       </c>
       <c r="B342" s="8" t="s">
-        <v>340</v>
+        <v>336</v>
       </c>
       <c r="C342" s="1" t="s">
         <v>4</v>
       </c>
       <c r="D342" s="11" t="s">
-        <v>5</v>
+        <v>9</v>
       </c>
     </row>
     <row r="343" spans="1:4" ht="15.75" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A343" s="6">
-        <v>60283</v>
-      </c>
-      <c r="B343" t="s">
-        <v>378</v>
+        <v>60282</v>
+      </c>
+      <c r="B343" s="8" t="s">
+        <v>340</v>
       </c>
       <c r="C343" s="1" t="s">
         <v>4</v>
       </c>
-      <c r="D343" s="1" t="s">
-        <v>8</v>
+      <c r="D343" s="11" t="s">
+        <v>5</v>
       </c>
     </row>
     <row r="344" spans="1:4" ht="15.75" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A344" s="6">
-        <v>60284</v>
-      </c>
-      <c r="B344" s="8" t="s">
-        <v>335</v>
+        <v>60283</v>
+      </c>
+      <c r="B344" t="s">
+        <v>378</v>
       </c>
       <c r="C344" s="1" t="s">
         <v>4</v>
       </c>
-      <c r="D344" s="9" t="s">
-        <v>5</v>
+      <c r="D344" s="1" t="s">
+        <v>8</v>
       </c>
     </row>
     <row r="345" spans="1:4" ht="15.75" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A345" s="6">
-        <v>60285</v>
+        <v>60284</v>
       </c>
       <c r="B345" s="8" t="s">
-        <v>350</v>
+        <v>335</v>
       </c>
       <c r="C345" s="1" t="s">
         <v>4</v>
@@ -6430,10 +6434,10 @@
     </row>
     <row r="346" spans="1:4" ht="15.75" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A346" s="6">
-        <v>60286</v>
+        <v>60285</v>
       </c>
       <c r="B346" s="8" t="s">
-        <v>334</v>
+        <v>350</v>
       </c>
       <c r="C346" s="1" t="s">
         <v>4</v>
@@ -6444,52 +6448,52 @@
     </row>
     <row r="347" spans="1:4" ht="15.75" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A347" s="6">
-        <v>60287</v>
-      </c>
-      <c r="B347" t="s">
-        <v>377</v>
+        <v>60286</v>
+      </c>
+      <c r="B347" s="8" t="s">
+        <v>334</v>
       </c>
       <c r="C347" s="1" t="s">
         <v>4</v>
       </c>
-      <c r="D347" s="12" t="s">
+      <c r="D347" s="9" t="s">
         <v>5</v>
       </c>
     </row>
     <row r="348" spans="1:4" ht="15.75" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A348" s="6">
-        <v>60289</v>
+        <v>60287</v>
       </c>
       <c r="B348" t="s">
-        <v>374</v>
+        <v>377</v>
       </c>
       <c r="C348" s="1" t="s">
         <v>4</v>
       </c>
       <c r="D348" s="12" t="s">
-        <v>9</v>
+        <v>5</v>
       </c>
     </row>
     <row r="349" spans="1:4" ht="15.75" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A349" s="6">
-        <v>60290</v>
+        <v>60289</v>
       </c>
       <c r="B349" t="s">
-        <v>375</v>
+        <v>374</v>
       </c>
       <c r="C349" s="1" t="s">
         <v>4</v>
       </c>
       <c r="D349" s="12" t="s">
-        <v>5</v>
+        <v>9</v>
       </c>
     </row>
     <row r="350" spans="1:4" ht="15.75" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A350" s="6">
-        <v>60291</v>
+        <v>60290</v>
       </c>
       <c r="B350" t="s">
-        <v>376</v>
+        <v>375</v>
       </c>
       <c r="C350" s="1" t="s">
         <v>4</v>
@@ -6500,24 +6504,24 @@
     </row>
     <row r="351" spans="1:4" ht="15.75" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A351" s="6">
-        <v>60292</v>
-      </c>
-      <c r="B351" s="18" t="s">
-        <v>400</v>
+        <v>60291</v>
+      </c>
+      <c r="B351" t="s">
+        <v>376</v>
       </c>
       <c r="C351" s="1" t="s">
         <v>4</v>
       </c>
       <c r="D351" s="12" t="s">
-        <v>8</v>
+        <v>5</v>
       </c>
     </row>
     <row r="352" spans="1:4" ht="15.75" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A352" s="6">
-        <v>60296</v>
-      </c>
-      <c r="B352" t="s">
-        <v>391</v>
+        <v>60292</v>
+      </c>
+      <c r="B352" s="18" t="s">
+        <v>400</v>
       </c>
       <c r="C352" s="1" t="s">
         <v>4</v>
@@ -6528,24 +6532,24 @@
     </row>
     <row r="353" spans="1:4" ht="15.75" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A353" s="6">
-        <v>60297</v>
+        <v>60296</v>
       </c>
       <c r="B353" t="s">
-        <v>392</v>
+        <v>391</v>
       </c>
       <c r="C353" s="1" t="s">
         <v>4</v>
       </c>
       <c r="D353" s="12" t="s">
-        <v>5</v>
+        <v>8</v>
       </c>
     </row>
     <row r="354" spans="1:4" ht="15.75" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A354" s="6">
-        <v>60299</v>
+        <v>60297</v>
       </c>
       <c r="B354" t="s">
-        <v>388</v>
+        <v>392</v>
       </c>
       <c r="C354" s="1" t="s">
         <v>4</v>
@@ -6556,52 +6560,52 @@
     </row>
     <row r="355" spans="1:4" ht="15.75" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A355" s="6">
-        <v>61001</v>
+        <v>60299</v>
       </c>
       <c r="B355" t="s">
-        <v>403</v>
+        <v>388</v>
       </c>
       <c r="C355" s="1" t="s">
         <v>4</v>
       </c>
       <c r="D355" s="12" t="s">
-        <v>8</v>
+        <v>5</v>
       </c>
     </row>
     <row r="356" spans="1:4" ht="15.75" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A356" s="6">
-        <v>61004</v>
+        <v>61001</v>
       </c>
       <c r="B356" t="s">
-        <v>293</v>
+        <v>403</v>
       </c>
       <c r="C356" s="1" t="s">
         <v>4</v>
       </c>
-      <c r="D356" s="15" t="s">
-        <v>5</v>
+      <c r="D356" s="12" t="s">
+        <v>8</v>
       </c>
     </row>
     <row r="357" spans="1:4" ht="15.75" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A357" s="6">
-        <v>61009</v>
+        <v>61004</v>
       </c>
       <c r="B357" t="s">
-        <v>294</v>
+        <v>293</v>
       </c>
       <c r="C357" s="1" t="s">
         <v>4</v>
       </c>
-      <c r="D357" s="12" t="s">
-        <v>8</v>
+      <c r="D357" s="15" t="s">
+        <v>5</v>
       </c>
     </row>
     <row r="358" spans="1:4" ht="15.75" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A358" s="6">
-        <v>61012</v>
+        <v>61009</v>
       </c>
       <c r="B358" t="s">
-        <v>295</v>
+        <v>294</v>
       </c>
       <c r="C358" s="1" t="s">
         <v>4</v>
@@ -6612,10 +6616,10 @@
     </row>
     <row r="359" spans="1:4" ht="15.75" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A359" s="6">
-        <v>61018</v>
+        <v>61012</v>
       </c>
       <c r="B359" t="s">
-        <v>296</v>
+        <v>295</v>
       </c>
       <c r="C359" s="1" t="s">
         <v>4</v>
@@ -6626,10 +6630,10 @@
     </row>
     <row r="360" spans="1:4" ht="15.75" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A360" s="6">
-        <v>61102</v>
+        <v>61018</v>
       </c>
       <c r="B360" t="s">
-        <v>297</v>
+        <v>296</v>
       </c>
       <c r="C360" s="1" t="s">
         <v>4</v>
@@ -6640,52 +6644,52 @@
     </row>
     <row r="361" spans="1:4" ht="15.75" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A361" s="6">
-        <v>61205</v>
+        <v>61102</v>
       </c>
       <c r="B361" t="s">
-        <v>298</v>
+        <v>297</v>
       </c>
       <c r="C361" s="1" t="s">
         <v>4</v>
       </c>
-      <c r="D361" s="15" t="s">
-        <v>5</v>
+      <c r="D361" s="12" t="s">
+        <v>8</v>
       </c>
     </row>
     <row r="362" spans="1:4" ht="15.75" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A362" s="6">
-        <v>70100</v>
+        <v>61205</v>
       </c>
       <c r="B362" t="s">
-        <v>299</v>
+        <v>298</v>
       </c>
       <c r="C362" s="1" t="s">
         <v>4</v>
       </c>
-      <c r="D362" s="12" t="s">
-        <v>8</v>
+      <c r="D362" s="15" t="s">
+        <v>5</v>
       </c>
     </row>
     <row r="363" spans="1:4" ht="15.75" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A363" s="6">
-        <v>70101</v>
+        <v>70100</v>
       </c>
       <c r="B363" t="s">
-        <v>300</v>
+        <v>299</v>
       </c>
       <c r="C363" s="1" t="s">
         <v>4</v>
       </c>
-      <c r="D363" s="15" t="s">
-        <v>5</v>
+      <c r="D363" s="12" t="s">
+        <v>8</v>
       </c>
     </row>
     <row r="364" spans="1:4" ht="15.75" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A364" s="6">
-        <v>70102</v>
+        <v>70101</v>
       </c>
       <c r="B364" t="s">
-        <v>301</v>
+        <v>300</v>
       </c>
       <c r="C364" s="1" t="s">
         <v>4</v>
@@ -6696,80 +6700,80 @@
     </row>
     <row r="365" spans="1:4" ht="15.75" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A365" s="6">
-        <v>70103</v>
+        <v>70102</v>
       </c>
       <c r="B365" t="s">
-        <v>302</v>
+        <v>301</v>
       </c>
       <c r="C365" s="1" t="s">
         <v>4</v>
       </c>
-      <c r="D365" s="12" t="s">
-        <v>8</v>
+      <c r="D365" s="15" t="s">
+        <v>5</v>
       </c>
     </row>
     <row r="366" spans="1:4" ht="15.75" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A366" s="6">
-        <v>70106</v>
+        <v>70103</v>
       </c>
       <c r="B366" t="s">
-        <v>303</v>
+        <v>302</v>
       </c>
       <c r="C366" s="1" t="s">
         <v>4</v>
       </c>
-      <c r="D366" s="15" t="s">
-        <v>5</v>
+      <c r="D366" s="12" t="s">
+        <v>8</v>
       </c>
     </row>
     <row r="367" spans="1:4" ht="15.75" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A367" s="6">
-        <v>70109</v>
+        <v>70106</v>
       </c>
       <c r="B367" t="s">
-        <v>304</v>
+        <v>303</v>
       </c>
       <c r="C367" s="1" t="s">
         <v>4</v>
       </c>
-      <c r="D367" s="12" t="s">
-        <v>8</v>
+      <c r="D367" s="15" t="s">
+        <v>5</v>
       </c>
     </row>
     <row r="368" spans="1:4" ht="15.75" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A368" s="6">
-        <v>70113</v>
+        <v>70109</v>
       </c>
       <c r="B368" t="s">
-        <v>305</v>
+        <v>304</v>
       </c>
       <c r="C368" s="1" t="s">
         <v>4</v>
       </c>
-      <c r="D368" s="15" t="s">
-        <v>5</v>
+      <c r="D368" s="12" t="s">
+        <v>8</v>
       </c>
     </row>
     <row r="369" spans="1:4" ht="15.75" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A369" s="6">
-        <v>70114</v>
+        <v>70113</v>
       </c>
       <c r="B369" t="s">
-        <v>325</v>
+        <v>305</v>
       </c>
       <c r="C369" s="1" t="s">
         <v>4</v>
       </c>
-      <c r="D369" s="9" t="s">
-        <v>9</v>
+      <c r="D369" s="15" t="s">
+        <v>5</v>
       </c>
     </row>
     <row r="370" spans="1:4" ht="15.75" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A370" s="6">
-        <v>70115</v>
+        <v>70114</v>
       </c>
       <c r="B370" t="s">
-        <v>331</v>
+        <v>325</v>
       </c>
       <c r="C370" s="1" t="s">
         <v>4</v>
@@ -6780,24 +6784,24 @@
     </row>
     <row r="371" spans="1:4" ht="15.75" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A371" s="6">
-        <v>70638</v>
+        <v>70115</v>
       </c>
       <c r="B371" t="s">
-        <v>306</v>
+        <v>331</v>
       </c>
       <c r="C371" s="1" t="s">
         <v>4</v>
       </c>
-      <c r="D371" s="12" t="s">
-        <v>8</v>
+      <c r="D371" s="9" t="s">
+        <v>9</v>
       </c>
     </row>
     <row r="372" spans="1:4" ht="15.75" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A372" s="6">
-        <v>70639</v>
+        <v>70638</v>
       </c>
       <c r="B372" t="s">
-        <v>307</v>
+        <v>306</v>
       </c>
       <c r="C372" s="1" t="s">
         <v>4</v>
@@ -6808,10 +6812,10 @@
     </row>
     <row r="373" spans="1:4" ht="15.75" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A373" s="6">
-        <v>70640</v>
+        <v>70639</v>
       </c>
       <c r="B373" t="s">
-        <v>308</v>
+        <v>307</v>
       </c>
       <c r="C373" s="1" t="s">
         <v>4</v>
@@ -6822,10 +6826,10 @@
     </row>
     <row r="374" spans="1:4" ht="15.75" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A374" s="6">
-        <v>70642</v>
+        <v>70640</v>
       </c>
       <c r="B374" t="s">
-        <v>309</v>
+        <v>308</v>
       </c>
       <c r="C374" s="1" t="s">
         <v>4</v>
@@ -6836,10 +6840,10 @@
     </row>
     <row r="375" spans="1:4" ht="15.75" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A375" s="6">
-        <v>90504</v>
+        <v>70642</v>
       </c>
       <c r="B375" t="s">
-        <v>310</v>
+        <v>309</v>
       </c>
       <c r="C375" s="1" t="s">
         <v>4</v>
@@ -6850,10 +6854,10 @@
     </row>
     <row r="376" spans="1:4" ht="15.75" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A376" s="6">
-        <v>90509</v>
+        <v>90504</v>
       </c>
       <c r="B376" t="s">
-        <v>311</v>
+        <v>310</v>
       </c>
       <c r="C376" s="1" t="s">
         <v>4</v>
@@ -6864,52 +6868,52 @@
     </row>
     <row r="377" spans="1:4" ht="15.75" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A377" s="6">
-        <v>90602</v>
+        <v>90509</v>
       </c>
       <c r="B377" t="s">
-        <v>312</v>
+        <v>311</v>
       </c>
       <c r="C377" s="1" t="s">
         <v>4</v>
       </c>
-      <c r="D377" s="15" t="s">
-        <v>5</v>
+      <c r="D377" s="12" t="s">
+        <v>8</v>
       </c>
     </row>
     <row r="378" spans="1:4" ht="15.75" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A378" s="6">
-        <v>90621</v>
+        <v>90602</v>
       </c>
       <c r="B378" t="s">
-        <v>313</v>
+        <v>312</v>
       </c>
       <c r="C378" s="1" t="s">
         <v>4</v>
       </c>
-      <c r="D378" s="12" t="s">
-        <v>8</v>
+      <c r="D378" s="15" t="s">
+        <v>5</v>
       </c>
     </row>
     <row r="379" spans="1:4" ht="15.75" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A379" s="6">
-        <v>90622</v>
+        <v>90621</v>
       </c>
       <c r="B379" t="s">
-        <v>333</v>
+        <v>313</v>
       </c>
       <c r="C379" s="1" t="s">
         <v>4</v>
       </c>
-      <c r="D379" s="9" t="s">
-        <v>5</v>
+      <c r="D379" s="12" t="s">
+        <v>8</v>
       </c>
     </row>
     <row r="380" spans="1:4" ht="15.75" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A380" s="6">
-        <v>90631</v>
-      </c>
-      <c r="B380" s="8" t="s">
-        <v>342</v>
+        <v>90622</v>
+      </c>
+      <c r="B380" t="s">
+        <v>333</v>
       </c>
       <c r="C380" s="1" t="s">
         <v>4</v>
@@ -6920,24 +6924,24 @@
     </row>
     <row r="381" spans="1:4" ht="15.75" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A381" s="6">
-        <v>90658</v>
-      </c>
-      <c r="B381" t="s">
-        <v>314</v>
+        <v>90631</v>
+      </c>
+      <c r="B381" s="8" t="s">
+        <v>342</v>
       </c>
       <c r="C381" s="1" t="s">
         <v>4</v>
       </c>
-      <c r="D381" s="12" t="s">
-        <v>8</v>
+      <c r="D381" s="9" t="s">
+        <v>5</v>
       </c>
     </row>
     <row r="382" spans="1:4" ht="15.75" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A382" s="6">
-        <v>90660</v>
+        <v>90658</v>
       </c>
       <c r="B382" t="s">
-        <v>315</v>
+        <v>314</v>
       </c>
       <c r="C382" s="1" t="s">
         <v>4</v>
@@ -6948,10 +6952,10 @@
     </row>
     <row r="383" spans="1:4" ht="15.75" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A383" s="6">
-        <v>90668</v>
+        <v>90660</v>
       </c>
       <c r="B383" t="s">
-        <v>316</v>
+        <v>315</v>
       </c>
       <c r="C383" s="1" t="s">
         <v>4</v>
@@ -6962,10 +6966,10 @@
     </row>
     <row r="384" spans="1:4" ht="15.75" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A384" s="6">
-        <v>90671</v>
+        <v>90668</v>
       </c>
       <c r="B384" t="s">
-        <v>317</v>
+        <v>316</v>
       </c>
       <c r="C384" s="1" t="s">
         <v>4</v>
@@ -6976,10 +6980,10 @@
     </row>
     <row r="385" spans="1:4" ht="15.75" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A385" s="6">
-        <v>90679</v>
+        <v>90671</v>
       </c>
       <c r="B385" t="s">
-        <v>318</v>
+        <v>317</v>
       </c>
       <c r="C385" s="1" t="s">
         <v>4</v>
@@ -6990,10 +6994,10 @@
     </row>
     <row r="386" spans="1:4" ht="15.75" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A386" s="6">
-        <v>90683</v>
+        <v>90679</v>
       </c>
       <c r="B386" t="s">
-        <v>319</v>
+        <v>318</v>
       </c>
       <c r="C386" s="1" t="s">
         <v>4</v>
@@ -7004,10 +7008,10 @@
     </row>
     <row r="387" spans="1:4" ht="15.75" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A387" s="6">
-        <v>90705</v>
+        <v>90683</v>
       </c>
       <c r="B387" t="s">
-        <v>320</v>
+        <v>319</v>
       </c>
       <c r="C387" s="1" t="s">
         <v>4</v>
@@ -7018,10 +7022,10 @@
     </row>
     <row r="388" spans="1:4" ht="15.75" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A388" s="6">
-        <v>90706</v>
+        <v>90705</v>
       </c>
       <c r="B388" t="s">
-        <v>321</v>
+        <v>320</v>
       </c>
       <c r="C388" s="1" t="s">
         <v>4</v>
@@ -7032,10 +7036,10 @@
     </row>
     <row r="389" spans="1:4" ht="15.75" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A389" s="6">
-        <v>90708</v>
+        <v>90706</v>
       </c>
       <c r="B389" t="s">
-        <v>322</v>
+        <v>321</v>
       </c>
       <c r="C389" s="1" t="s">
         <v>4</v>
@@ -7046,10 +7050,10 @@
     </row>
     <row r="390" spans="1:4" ht="15.75" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A390" s="6">
-        <v>90709</v>
+        <v>90708</v>
       </c>
       <c r="B390" t="s">
-        <v>323</v>
+        <v>322</v>
       </c>
       <c r="C390" s="1" t="s">
         <v>4</v>
@@ -7060,38 +7064,38 @@
     </row>
     <row r="391" spans="1:4" ht="15.75" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A391" s="6">
-        <v>90713</v>
+        <v>90709</v>
       </c>
       <c r="B391" t="s">
-        <v>402</v>
+        <v>323</v>
       </c>
       <c r="C391" s="1" t="s">
         <v>4</v>
       </c>
       <c r="D391" s="12" t="s">
-        <v>5</v>
+        <v>8</v>
       </c>
     </row>
     <row r="392" spans="1:4" ht="15.75" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A392" s="6">
-        <v>1218</v>
+        <v>90713</v>
       </c>
       <c r="B392" t="s">
-        <v>382</v>
+        <v>402</v>
       </c>
       <c r="C392" s="1" t="s">
         <v>4</v>
       </c>
       <c r="D392" s="12" t="s">
-        <v>8</v>
+        <v>5</v>
       </c>
     </row>
     <row r="393" spans="1:4" ht="15.75" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A393" s="6">
-        <v>1959</v>
-      </c>
-      <c r="B393" s="8" t="s">
-        <v>383</v>
+        <v>1218</v>
+      </c>
+      <c r="B393" t="s">
+        <v>382</v>
       </c>
       <c r="C393" s="1" t="s">
         <v>4</v>
@@ -7102,10 +7106,10 @@
     </row>
     <row r="394" spans="1:4" ht="15.75" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A394" s="6">
-        <v>5625</v>
+        <v>1959</v>
       </c>
       <c r="B394" s="8" t="s">
-        <v>384</v>
+        <v>383</v>
       </c>
       <c r="C394" s="1" t="s">
         <v>4</v>
@@ -7116,10 +7120,10 @@
     </row>
     <row r="395" spans="1:4" ht="15.75" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A395" s="6">
-        <v>1817</v>
+        <v>5625</v>
       </c>
       <c r="B395" s="8" t="s">
-        <v>389</v>
+        <v>384</v>
       </c>
       <c r="C395" s="1" t="s">
         <v>4</v>
@@ -7130,10 +7134,10 @@
     </row>
     <row r="396" spans="1:4" ht="15.75" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A396" s="6">
-        <v>5737</v>
+        <v>1817</v>
       </c>
       <c r="B396" s="8" t="s">
-        <v>390</v>
+        <v>389</v>
       </c>
       <c r="C396" s="1" t="s">
         <v>4</v>
@@ -7144,34 +7148,48 @@
     </row>
     <row r="397" spans="1:4" ht="15.75" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A397" s="6">
-        <v>60295</v>
+        <v>5737</v>
       </c>
       <c r="B397" s="8" t="s">
-        <v>385</v>
+        <v>390</v>
       </c>
       <c r="C397" s="1" t="s">
         <v>4</v>
       </c>
-      <c r="D397" s="9" t="s">
-        <v>9</v>
+      <c r="D397" s="12" t="s">
+        <v>8</v>
       </c>
     </row>
     <row r="398" spans="1:4" ht="15.75" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A398" s="6">
+        <v>60295</v>
+      </c>
+      <c r="B398" s="8" t="s">
+        <v>385</v>
+      </c>
+      <c r="C398" s="1" t="s">
+        <v>4</v>
+      </c>
+      <c r="D398" s="9" t="s">
+        <v>9</v>
+      </c>
+    </row>
+    <row r="399" spans="1:4" ht="15.75" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
+      <c r="A399" s="6">
         <v>1045</v>
       </c>
-      <c r="B398" s="8" t="s">
+      <c r="B399" s="8" t="s">
         <v>386</v>
       </c>
-      <c r="C398" s="1" t="s">
-        <v>4</v>
-      </c>
-      <c r="D398" s="9" t="s">
+      <c r="C399" s="1" t="s">
+        <v>4</v>
+      </c>
+      <c r="D399" s="9" t="s">
         <v>5</v>
       </c>
     </row>
   </sheetData>
-  <autoFilter ref="A1:D343"/>
+  <autoFilter ref="A1:D344"/>
   <sortState ref="A2:D374">
     <sortCondition ref="A277"/>
   </sortState>

</xml_diff>

<commit_message>
update active cuenta 60194, estado de cuentas clientes 27-8-26
</commit_message>
<xml_diff>
--- a/excel/CLIENTES_PERMISOS.xlsx
+++ b/excel/CLIENTES_PERMISOS.xlsx
@@ -15,14 +15,14 @@
     <sheet name="Hoja 1" sheetId="1" r:id="rId1"/>
   </sheets>
   <definedNames>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'Hoja 1'!$A$1:$D$348</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'Hoja 1'!$A$1:$D$349</definedName>
   </definedNames>
   <calcPr calcId="162913"/>
 </workbook>
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="1210" uniqueCount="410">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="1213" uniqueCount="411">
   <si>
     <t>CUENTA</t>
   </si>
@@ -1252,6 +1252,9 @@
   </si>
   <si>
     <t>FERRETERIA BM</t>
+  </si>
+  <si>
+    <t>EL BUHO FERRETERIA</t>
   </si>
 </sst>
 </file>
@@ -1606,7 +1609,7 @@
   <sheetPr>
     <outlinePr summaryBelow="0" summaryRight="0"/>
   </sheetPr>
-  <dimension ref="A1:D403"/>
+  <dimension ref="A1:D404"/>
   <sheetFormatPr baseColWidth="10" defaultColWidth="12.5703125" defaultRowHeight="15.75" customHeight="1" x14ac:dyDescent="0.2"/>
   <cols>
     <col min="2" max="2" width="34" customWidth="1"/>
@@ -5914,10 +5917,10 @@
     </row>
     <row r="308" spans="1:4" ht="15.75" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A308" s="6">
-        <v>60195</v>
-      </c>
-      <c r="B308" t="s">
-        <v>265</v>
+        <v>60194</v>
+      </c>
+      <c r="B308" s="18" t="s">
+        <v>410</v>
       </c>
       <c r="C308" s="1" t="s">
         <v>4</v>
@@ -5928,10 +5931,10 @@
     </row>
     <row r="309" spans="1:4" ht="15.75" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A309" s="6">
-        <v>60196</v>
+        <v>60195</v>
       </c>
       <c r="B309" t="s">
-        <v>266</v>
+        <v>265</v>
       </c>
       <c r="C309" s="1" t="s">
         <v>4</v>
@@ -5942,10 +5945,10 @@
     </row>
     <row r="310" spans="1:4" ht="15.75" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A310" s="6">
-        <v>60198</v>
+        <v>60196</v>
       </c>
       <c r="B310" t="s">
-        <v>267</v>
+        <v>266</v>
       </c>
       <c r="C310" s="1" t="s">
         <v>4</v>
@@ -5956,52 +5959,52 @@
     </row>
     <row r="311" spans="1:4" ht="15.75" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A311" s="6">
-        <v>60201</v>
+        <v>60198</v>
       </c>
       <c r="B311" t="s">
-        <v>268</v>
+        <v>267</v>
       </c>
       <c r="C311" s="1" t="s">
         <v>4</v>
       </c>
-      <c r="D311" t="s">
-        <v>9</v>
+      <c r="D311" s="10" t="s">
+        <v>8</v>
       </c>
     </row>
     <row r="312" spans="1:4" ht="15.75" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A312" s="6">
-        <v>60202</v>
+        <v>60201</v>
       </c>
       <c r="B312" t="s">
-        <v>269</v>
+        <v>268</v>
       </c>
       <c r="C312" s="1" t="s">
         <v>4</v>
       </c>
-      <c r="D312" s="13" t="s">
-        <v>5</v>
+      <c r="D312" t="s">
+        <v>9</v>
       </c>
     </row>
     <row r="313" spans="1:4" ht="15.75" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A313" s="6">
-        <v>60204</v>
+        <v>60202</v>
       </c>
       <c r="B313" t="s">
-        <v>270</v>
+        <v>269</v>
       </c>
       <c r="C313" s="1" t="s">
         <v>4</v>
       </c>
-      <c r="D313" s="1" t="s">
-        <v>8</v>
+      <c r="D313" s="13" t="s">
+        <v>5</v>
       </c>
     </row>
     <row r="314" spans="1:4" ht="15.75" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A314" s="6">
-        <v>60205</v>
+        <v>60204</v>
       </c>
       <c r="B314" t="s">
-        <v>271</v>
+        <v>270</v>
       </c>
       <c r="C314" s="1" t="s">
         <v>4</v>
@@ -6012,10 +6015,10 @@
     </row>
     <row r="315" spans="1:4" ht="15.75" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A315" s="6">
-        <v>60206</v>
+        <v>60205</v>
       </c>
       <c r="B315" t="s">
-        <v>272</v>
+        <v>271</v>
       </c>
       <c r="C315" s="1" t="s">
         <v>4</v>
@@ -6026,192 +6029,192 @@
     </row>
     <row r="316" spans="1:4" ht="15.75" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A316" s="6">
-        <v>60209</v>
+        <v>60206</v>
       </c>
       <c r="B316" t="s">
-        <v>273</v>
+        <v>272</v>
       </c>
       <c r="C316" s="1" t="s">
         <v>4</v>
       </c>
-      <c r="D316" s="10" t="s">
+      <c r="D316" s="1" t="s">
         <v>8</v>
       </c>
     </row>
     <row r="317" spans="1:4" ht="15.75" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A317" s="6">
-        <v>60211</v>
+        <v>60209</v>
       </c>
       <c r="B317" t="s">
-        <v>274</v>
+        <v>273</v>
       </c>
       <c r="C317" s="1" t="s">
         <v>4</v>
       </c>
-      <c r="D317" s="1" t="s">
+      <c r="D317" s="10" t="s">
         <v>8</v>
       </c>
     </row>
     <row r="318" spans="1:4" ht="15.75" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A318" s="6">
-        <v>60215</v>
+        <v>60211</v>
       </c>
       <c r="B318" t="s">
-        <v>275</v>
+        <v>274</v>
       </c>
       <c r="C318" s="1" t="s">
         <v>4</v>
       </c>
-      <c r="D318" s="10" t="s">
+      <c r="D318" s="1" t="s">
         <v>8</v>
       </c>
     </row>
     <row r="319" spans="1:4" ht="15.75" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A319" s="6">
-        <v>60216</v>
+        <v>60215</v>
       </c>
       <c r="B319" t="s">
-        <v>381</v>
+        <v>275</v>
       </c>
       <c r="C319" s="1" t="s">
         <v>4</v>
       </c>
       <c r="D319" s="10" t="s">
-        <v>9</v>
+        <v>8</v>
       </c>
     </row>
     <row r="320" spans="1:4" ht="15.75" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A320" s="6">
-        <v>60217</v>
+        <v>60216</v>
       </c>
       <c r="B320" t="s">
-        <v>276</v>
+        <v>381</v>
       </c>
       <c r="C320" s="1" t="s">
         <v>4</v>
       </c>
       <c r="D320" s="10" t="s">
-        <v>8</v>
+        <v>9</v>
       </c>
     </row>
     <row r="321" spans="1:4" ht="15.75" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A321" s="6">
-        <v>60219</v>
+        <v>60217</v>
       </c>
       <c r="B321" t="s">
-        <v>277</v>
+        <v>276</v>
       </c>
       <c r="C321" s="1" t="s">
         <v>4</v>
       </c>
-      <c r="D321" s="1" t="s">
+      <c r="D321" s="10" t="s">
         <v>8</v>
       </c>
     </row>
     <row r="322" spans="1:4" ht="15.75" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A322" s="6">
-        <v>60222</v>
+        <v>60219</v>
       </c>
       <c r="B322" t="s">
-        <v>278</v>
+        <v>277</v>
       </c>
       <c r="C322" s="1" t="s">
         <v>4</v>
       </c>
-      <c r="D322" s="10" t="s">
+      <c r="D322" s="1" t="s">
         <v>8</v>
       </c>
     </row>
     <row r="323" spans="1:4" ht="15.75" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A323" s="6">
-        <v>60225</v>
+        <v>60222</v>
       </c>
       <c r="B323" t="s">
-        <v>279</v>
+        <v>278</v>
       </c>
       <c r="C323" s="1" t="s">
         <v>4</v>
       </c>
-      <c r="D323" s="17" t="s">
-        <v>9</v>
+      <c r="D323" s="10" t="s">
+        <v>8</v>
       </c>
     </row>
     <row r="324" spans="1:4" ht="15.75" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A324" s="6">
-        <v>60230</v>
+        <v>60225</v>
       </c>
       <c r="B324" t="s">
-        <v>280</v>
+        <v>279</v>
       </c>
       <c r="C324" s="1" t="s">
         <v>4</v>
       </c>
-      <c r="D324" s="10" t="s">
-        <v>8</v>
+      <c r="D324" s="17" t="s">
+        <v>9</v>
       </c>
     </row>
     <row r="325" spans="1:4" ht="15.75" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A325" s="6">
-        <v>60241</v>
-      </c>
-      <c r="B325" s="8" t="s">
-        <v>338</v>
+        <v>60230</v>
+      </c>
+      <c r="B325" t="s">
+        <v>280</v>
       </c>
       <c r="C325" s="1" t="s">
         <v>4</v>
       </c>
-      <c r="D325" s="7" t="s">
-        <v>9</v>
+      <c r="D325" s="10" t="s">
+        <v>8</v>
       </c>
     </row>
     <row r="326" spans="1:4" ht="15.75" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A326" s="6">
-        <v>60242</v>
+        <v>60241</v>
       </c>
       <c r="B326" s="8" t="s">
-        <v>341</v>
+        <v>338</v>
       </c>
       <c r="C326" s="1" t="s">
         <v>4</v>
       </c>
       <c r="D326" s="7" t="s">
-        <v>5</v>
+        <v>9</v>
       </c>
     </row>
     <row r="327" spans="1:4" ht="15.75" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A327" s="6">
-        <v>60243</v>
+        <v>60242</v>
       </c>
       <c r="B327" s="8" t="s">
-        <v>395</v>
+        <v>341</v>
       </c>
       <c r="C327" s="1" t="s">
         <v>4</v>
       </c>
       <c r="D327" s="7" t="s">
-        <v>9</v>
+        <v>5</v>
       </c>
     </row>
     <row r="328" spans="1:4" ht="15.75" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A328" s="6">
-        <v>60245</v>
+        <v>60243</v>
       </c>
       <c r="B328" s="8" t="s">
-        <v>387</v>
+        <v>395</v>
       </c>
       <c r="C328" s="1" t="s">
         <v>4</v>
       </c>
       <c r="D328" s="7" t="s">
-        <v>5</v>
+        <v>9</v>
       </c>
     </row>
     <row r="329" spans="1:4" ht="15.75" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A329" s="6">
-        <v>60246</v>
+        <v>60245</v>
       </c>
       <c r="B329" s="8" t="s">
-        <v>407</v>
+        <v>387</v>
       </c>
       <c r="C329" s="1" t="s">
         <v>4</v>
@@ -6222,10 +6225,10 @@
     </row>
     <row r="330" spans="1:4" ht="15.75" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A330" s="6">
-        <v>60249</v>
-      </c>
-      <c r="B330" s="18" t="s">
-        <v>408</v>
+        <v>60246</v>
+      </c>
+      <c r="B330" s="8" t="s">
+        <v>407</v>
       </c>
       <c r="C330" s="1" t="s">
         <v>4</v>
@@ -6236,38 +6239,38 @@
     </row>
     <row r="331" spans="1:4" ht="15.75" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A331" s="6">
-        <v>60250</v>
-      </c>
-      <c r="B331" s="8" t="s">
-        <v>339</v>
+        <v>60249</v>
+      </c>
+      <c r="B331" s="18" t="s">
+        <v>408</v>
       </c>
       <c r="C331" s="1" t="s">
         <v>4</v>
       </c>
-      <c r="D331" s="11" t="s">
-        <v>8</v>
+      <c r="D331" s="7" t="s">
+        <v>5</v>
       </c>
     </row>
     <row r="332" spans="1:4" ht="15.75" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A332" s="6">
-        <v>60253</v>
-      </c>
-      <c r="B332" t="s">
-        <v>281</v>
+        <v>60250</v>
+      </c>
+      <c r="B332" s="8" t="s">
+        <v>339</v>
       </c>
       <c r="C332" s="1" t="s">
         <v>4</v>
       </c>
-      <c r="D332" s="1" t="s">
+      <c r="D332" s="11" t="s">
         <v>8</v>
       </c>
     </row>
     <row r="333" spans="1:4" ht="15.75" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A333" s="6">
-        <v>60254</v>
+        <v>60253</v>
       </c>
       <c r="B333" t="s">
-        <v>282</v>
+        <v>281</v>
       </c>
       <c r="C333" s="1" t="s">
         <v>4</v>
@@ -6278,10 +6281,10 @@
     </row>
     <row r="334" spans="1:4" ht="15.75" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A334" s="6">
-        <v>60257</v>
+        <v>60254</v>
       </c>
       <c r="B334" t="s">
-        <v>283</v>
+        <v>282</v>
       </c>
       <c r="C334" s="1" t="s">
         <v>4</v>
@@ -6292,10 +6295,10 @@
     </row>
     <row r="335" spans="1:4" ht="15.75" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A335" s="6">
-        <v>60258</v>
+        <v>60257</v>
       </c>
       <c r="B335" t="s">
-        <v>284</v>
+        <v>283</v>
       </c>
       <c r="C335" s="1" t="s">
         <v>4</v>
@@ -6306,66 +6309,66 @@
     </row>
     <row r="336" spans="1:4" ht="15.75" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A336" s="6">
-        <v>60266</v>
-      </c>
-      <c r="B336" s="8" t="s">
-        <v>343</v>
+        <v>60258</v>
+      </c>
+      <c r="B336" t="s">
+        <v>284</v>
       </c>
       <c r="C336" s="1" t="s">
         <v>4</v>
       </c>
-      <c r="D336" s="11" t="s">
+      <c r="D336" s="1" t="s">
         <v>8</v>
       </c>
     </row>
     <row r="337" spans="1:4" ht="15.75" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A337" s="6">
-        <v>60269</v>
-      </c>
-      <c r="B337" t="s">
-        <v>285</v>
+        <v>60266</v>
+      </c>
+      <c r="B337" s="8" t="s">
+        <v>343</v>
       </c>
       <c r="C337" s="1" t="s">
         <v>4</v>
       </c>
-      <c r="D337" s="10" t="s">
+      <c r="D337" s="11" t="s">
         <v>8</v>
       </c>
     </row>
     <row r="338" spans="1:4" ht="15.75" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A338" s="6">
-        <v>60270</v>
+        <v>60269</v>
       </c>
       <c r="B338" t="s">
-        <v>286</v>
+        <v>285</v>
       </c>
       <c r="C338" s="1" t="s">
         <v>4</v>
       </c>
-      <c r="D338" s="1" t="s">
-        <v>9</v>
+      <c r="D338" s="10" t="s">
+        <v>8</v>
       </c>
     </row>
     <row r="339" spans="1:4" ht="15.75" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A339" s="6">
-        <v>60272</v>
+        <v>60270</v>
       </c>
       <c r="B339" t="s">
-        <v>287</v>
+        <v>286</v>
       </c>
       <c r="C339" s="1" t="s">
         <v>4</v>
       </c>
       <c r="D339" s="1" t="s">
-        <v>8</v>
+        <v>9</v>
       </c>
     </row>
     <row r="340" spans="1:4" ht="15.75" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A340" s="6">
-        <v>60274</v>
+        <v>60272</v>
       </c>
       <c r="B340" t="s">
-        <v>380</v>
+        <v>287</v>
       </c>
       <c r="C340" s="1" t="s">
         <v>4</v>
@@ -6376,10 +6379,10 @@
     </row>
     <row r="341" spans="1:4" ht="15.75" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A341" s="6">
-        <v>60275</v>
+        <v>60274</v>
       </c>
       <c r="B341" t="s">
-        <v>288</v>
+        <v>380</v>
       </c>
       <c r="C341" s="1" t="s">
         <v>4</v>
@@ -6390,10 +6393,10 @@
     </row>
     <row r="342" spans="1:4" ht="15.75" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A342" s="6">
-        <v>60276</v>
+        <v>60275</v>
       </c>
       <c r="B342" t="s">
-        <v>289</v>
+        <v>288</v>
       </c>
       <c r="C342" s="1" t="s">
         <v>4</v>
@@ -6404,108 +6407,108 @@
     </row>
     <row r="343" spans="1:4" ht="15.75" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A343" s="6">
-        <v>60278</v>
+        <v>60276</v>
       </c>
       <c r="B343" t="s">
-        <v>290</v>
+        <v>289</v>
       </c>
       <c r="C343" s="1" t="s">
         <v>4</v>
       </c>
-      <c r="D343" s="13" t="s">
+      <c r="D343" s="1" t="s">
         <v>8</v>
       </c>
     </row>
     <row r="344" spans="1:4" ht="15.75" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A344" s="6">
-        <v>60279</v>
+        <v>60278</v>
       </c>
       <c r="B344" t="s">
-        <v>291</v>
+        <v>290</v>
       </c>
       <c r="C344" s="1" t="s">
         <v>4</v>
       </c>
-      <c r="D344" s="1" t="s">
+      <c r="D344" s="13" t="s">
         <v>8</v>
       </c>
     </row>
     <row r="345" spans="1:4" ht="15.75" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A345" s="6">
-        <v>60280</v>
+        <v>60279</v>
       </c>
       <c r="B345" t="s">
-        <v>292</v>
+        <v>291</v>
       </c>
       <c r="C345" s="1" t="s">
         <v>4</v>
       </c>
       <c r="D345" s="1" t="s">
-        <v>5</v>
+        <v>8</v>
       </c>
     </row>
     <row r="346" spans="1:4" ht="15.75" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A346" s="6">
-        <v>60281</v>
-      </c>
-      <c r="B346" s="8" t="s">
-        <v>336</v>
+        <v>60280</v>
+      </c>
+      <c r="B346" t="s">
+        <v>292</v>
       </c>
       <c r="C346" s="1" t="s">
         <v>4</v>
       </c>
-      <c r="D346" s="11" t="s">
-        <v>9</v>
+      <c r="D346" s="1" t="s">
+        <v>5</v>
       </c>
     </row>
     <row r="347" spans="1:4" ht="15.75" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A347" s="6">
-        <v>60282</v>
+        <v>60281</v>
       </c>
       <c r="B347" s="8" t="s">
-        <v>340</v>
+        <v>336</v>
       </c>
       <c r="C347" s="1" t="s">
         <v>4</v>
       </c>
       <c r="D347" s="11" t="s">
-        <v>5</v>
+        <v>9</v>
       </c>
     </row>
     <row r="348" spans="1:4" ht="15.75" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A348" s="6">
-        <v>60283</v>
-      </c>
-      <c r="B348" t="s">
-        <v>378</v>
+        <v>60282</v>
+      </c>
+      <c r="B348" s="8" t="s">
+        <v>340</v>
       </c>
       <c r="C348" s="1" t="s">
         <v>4</v>
       </c>
-      <c r="D348" s="1" t="s">
-        <v>8</v>
+      <c r="D348" s="11" t="s">
+        <v>5</v>
       </c>
     </row>
     <row r="349" spans="1:4" ht="15.75" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A349" s="6">
-        <v>60284</v>
-      </c>
-      <c r="B349" s="8" t="s">
-        <v>335</v>
+        <v>60283</v>
+      </c>
+      <c r="B349" t="s">
+        <v>378</v>
       </c>
       <c r="C349" s="1" t="s">
         <v>4</v>
       </c>
-      <c r="D349" s="9" t="s">
-        <v>5</v>
+      <c r="D349" s="1" t="s">
+        <v>8</v>
       </c>
     </row>
     <row r="350" spans="1:4" ht="15.75" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A350" s="6">
-        <v>60285</v>
+        <v>60284</v>
       </c>
       <c r="B350" s="8" t="s">
-        <v>350</v>
+        <v>335</v>
       </c>
       <c r="C350" s="1" t="s">
         <v>4</v>
@@ -6516,10 +6519,10 @@
     </row>
     <row r="351" spans="1:4" ht="15.75" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A351" s="6">
-        <v>60286</v>
+        <v>60285</v>
       </c>
       <c r="B351" s="8" t="s">
-        <v>334</v>
+        <v>350</v>
       </c>
       <c r="C351" s="1" t="s">
         <v>4</v>
@@ -6530,52 +6533,52 @@
     </row>
     <row r="352" spans="1:4" ht="15.75" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A352" s="6">
-        <v>60287</v>
-      </c>
-      <c r="B352" t="s">
-        <v>377</v>
+        <v>60286</v>
+      </c>
+      <c r="B352" s="8" t="s">
+        <v>334</v>
       </c>
       <c r="C352" s="1" t="s">
         <v>4</v>
       </c>
-      <c r="D352" s="12" t="s">
+      <c r="D352" s="9" t="s">
         <v>5</v>
       </c>
     </row>
     <row r="353" spans="1:4" ht="15.75" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A353" s="6">
-        <v>60289</v>
+        <v>60287</v>
       </c>
       <c r="B353" t="s">
-        <v>374</v>
+        <v>377</v>
       </c>
       <c r="C353" s="1" t="s">
         <v>4</v>
       </c>
       <c r="D353" s="12" t="s">
-        <v>9</v>
+        <v>5</v>
       </c>
     </row>
     <row r="354" spans="1:4" ht="15.75" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A354" s="6">
-        <v>60290</v>
+        <v>60289</v>
       </c>
       <c r="B354" t="s">
-        <v>375</v>
+        <v>374</v>
       </c>
       <c r="C354" s="1" t="s">
         <v>4</v>
       </c>
       <c r="D354" s="12" t="s">
-        <v>5</v>
+        <v>9</v>
       </c>
     </row>
     <row r="355" spans="1:4" ht="15.75" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A355" s="6">
-        <v>60291</v>
+        <v>60290</v>
       </c>
       <c r="B355" t="s">
-        <v>376</v>
+        <v>375</v>
       </c>
       <c r="C355" s="1" t="s">
         <v>4</v>
@@ -6586,24 +6589,24 @@
     </row>
     <row r="356" spans="1:4" ht="15.75" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A356" s="6">
-        <v>60292</v>
-      </c>
-      <c r="B356" s="18" t="s">
-        <v>400</v>
+        <v>60291</v>
+      </c>
+      <c r="B356" t="s">
+        <v>376</v>
       </c>
       <c r="C356" s="1" t="s">
         <v>4</v>
       </c>
       <c r="D356" s="12" t="s">
-        <v>8</v>
+        <v>5</v>
       </c>
     </row>
     <row r="357" spans="1:4" ht="15.75" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A357" s="6">
-        <v>60296</v>
-      </c>
-      <c r="B357" t="s">
-        <v>391</v>
+        <v>60292</v>
+      </c>
+      <c r="B357" s="18" t="s">
+        <v>400</v>
       </c>
       <c r="C357" s="1" t="s">
         <v>4</v>
@@ -6614,24 +6617,24 @@
     </row>
     <row r="358" spans="1:4" ht="15.75" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A358" s="6">
-        <v>60297</v>
+        <v>60296</v>
       </c>
       <c r="B358" t="s">
-        <v>392</v>
+        <v>391</v>
       </c>
       <c r="C358" s="1" t="s">
         <v>4</v>
       </c>
       <c r="D358" s="12" t="s">
-        <v>5</v>
+        <v>8</v>
       </c>
     </row>
     <row r="359" spans="1:4" ht="15.75" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A359" s="6">
-        <v>60299</v>
+        <v>60297</v>
       </c>
       <c r="B359" t="s">
-        <v>388</v>
+        <v>392</v>
       </c>
       <c r="C359" s="1" t="s">
         <v>4</v>
@@ -6642,52 +6645,52 @@
     </row>
     <row r="360" spans="1:4" ht="15.75" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A360" s="6">
-        <v>61001</v>
+        <v>60299</v>
       </c>
       <c r="B360" t="s">
-        <v>403</v>
+        <v>388</v>
       </c>
       <c r="C360" s="1" t="s">
         <v>4</v>
       </c>
       <c r="D360" s="12" t="s">
-        <v>8</v>
+        <v>5</v>
       </c>
     </row>
     <row r="361" spans="1:4" ht="15.75" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A361" s="6">
-        <v>61004</v>
+        <v>61001</v>
       </c>
       <c r="B361" t="s">
-        <v>293</v>
+        <v>403</v>
       </c>
       <c r="C361" s="1" t="s">
         <v>4</v>
       </c>
-      <c r="D361" s="15" t="s">
-        <v>5</v>
+      <c r="D361" s="12" t="s">
+        <v>8</v>
       </c>
     </row>
     <row r="362" spans="1:4" ht="15.75" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A362" s="6">
-        <v>61009</v>
+        <v>61004</v>
       </c>
       <c r="B362" t="s">
-        <v>294</v>
+        <v>293</v>
       </c>
       <c r="C362" s="1" t="s">
         <v>4</v>
       </c>
-      <c r="D362" s="12" t="s">
-        <v>8</v>
+      <c r="D362" s="15" t="s">
+        <v>5</v>
       </c>
     </row>
     <row r="363" spans="1:4" ht="15.75" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A363" s="6">
-        <v>61012</v>
+        <v>61009</v>
       </c>
       <c r="B363" t="s">
-        <v>295</v>
+        <v>294</v>
       </c>
       <c r="C363" s="1" t="s">
         <v>4</v>
@@ -6698,10 +6701,10 @@
     </row>
     <row r="364" spans="1:4" ht="15.75" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A364" s="6">
-        <v>61018</v>
+        <v>61012</v>
       </c>
       <c r="B364" t="s">
-        <v>296</v>
+        <v>295</v>
       </c>
       <c r="C364" s="1" t="s">
         <v>4</v>
@@ -6712,10 +6715,10 @@
     </row>
     <row r="365" spans="1:4" ht="15.75" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A365" s="6">
-        <v>61102</v>
+        <v>61018</v>
       </c>
       <c r="B365" t="s">
-        <v>297</v>
+        <v>296</v>
       </c>
       <c r="C365" s="1" t="s">
         <v>4</v>
@@ -6726,52 +6729,52 @@
     </row>
     <row r="366" spans="1:4" ht="15.75" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A366" s="6">
-        <v>61205</v>
+        <v>61102</v>
       </c>
       <c r="B366" t="s">
-        <v>298</v>
+        <v>297</v>
       </c>
       <c r="C366" s="1" t="s">
         <v>4</v>
       </c>
-      <c r="D366" s="15" t="s">
-        <v>5</v>
+      <c r="D366" s="12" t="s">
+        <v>8</v>
       </c>
     </row>
     <row r="367" spans="1:4" ht="15.75" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A367" s="6">
-        <v>70100</v>
+        <v>61205</v>
       </c>
       <c r="B367" t="s">
-        <v>299</v>
+        <v>298</v>
       </c>
       <c r="C367" s="1" t="s">
         <v>4</v>
       </c>
-      <c r="D367" s="12" t="s">
-        <v>8</v>
+      <c r="D367" s="15" t="s">
+        <v>5</v>
       </c>
     </row>
     <row r="368" spans="1:4" ht="15.75" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A368" s="6">
-        <v>70101</v>
+        <v>70100</v>
       </c>
       <c r="B368" t="s">
-        <v>300</v>
+        <v>299</v>
       </c>
       <c r="C368" s="1" t="s">
         <v>4</v>
       </c>
-      <c r="D368" s="15" t="s">
-        <v>5</v>
+      <c r="D368" s="12" t="s">
+        <v>8</v>
       </c>
     </row>
     <row r="369" spans="1:4" ht="15.75" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A369" s="6">
-        <v>70102</v>
+        <v>70101</v>
       </c>
       <c r="B369" t="s">
-        <v>301</v>
+        <v>300</v>
       </c>
       <c r="C369" s="1" t="s">
         <v>4</v>
@@ -6782,80 +6785,80 @@
     </row>
     <row r="370" spans="1:4" ht="15.75" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A370" s="6">
-        <v>70103</v>
+        <v>70102</v>
       </c>
       <c r="B370" t="s">
-        <v>302</v>
+        <v>301</v>
       </c>
       <c r="C370" s="1" t="s">
         <v>4</v>
       </c>
-      <c r="D370" s="12" t="s">
-        <v>8</v>
+      <c r="D370" s="15" t="s">
+        <v>5</v>
       </c>
     </row>
     <row r="371" spans="1:4" ht="15.75" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A371" s="6">
-        <v>70106</v>
+        <v>70103</v>
       </c>
       <c r="B371" t="s">
-        <v>303</v>
+        <v>302</v>
       </c>
       <c r="C371" s="1" t="s">
         <v>4</v>
       </c>
-      <c r="D371" s="15" t="s">
-        <v>5</v>
+      <c r="D371" s="12" t="s">
+        <v>8</v>
       </c>
     </row>
     <row r="372" spans="1:4" ht="15.75" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A372" s="6">
-        <v>70109</v>
+        <v>70106</v>
       </c>
       <c r="B372" t="s">
-        <v>304</v>
+        <v>303</v>
       </c>
       <c r="C372" s="1" t="s">
         <v>4</v>
       </c>
-      <c r="D372" s="12" t="s">
-        <v>8</v>
+      <c r="D372" s="15" t="s">
+        <v>5</v>
       </c>
     </row>
     <row r="373" spans="1:4" ht="15.75" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A373" s="6">
-        <v>70113</v>
+        <v>70109</v>
       </c>
       <c r="B373" t="s">
-        <v>305</v>
+        <v>304</v>
       </c>
       <c r="C373" s="1" t="s">
         <v>4</v>
       </c>
-      <c r="D373" s="15" t="s">
-        <v>5</v>
+      <c r="D373" s="12" t="s">
+        <v>8</v>
       </c>
     </row>
     <row r="374" spans="1:4" ht="15.75" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A374" s="6">
-        <v>70114</v>
+        <v>70113</v>
       </c>
       <c r="B374" t="s">
-        <v>325</v>
+        <v>305</v>
       </c>
       <c r="C374" s="1" t="s">
         <v>4</v>
       </c>
-      <c r="D374" s="9" t="s">
-        <v>9</v>
+      <c r="D374" s="15" t="s">
+        <v>5</v>
       </c>
     </row>
     <row r="375" spans="1:4" ht="15.75" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A375" s="6">
-        <v>70115</v>
+        <v>70114</v>
       </c>
       <c r="B375" t="s">
-        <v>331</v>
+        <v>325</v>
       </c>
       <c r="C375" s="1" t="s">
         <v>4</v>
@@ -6866,24 +6869,24 @@
     </row>
     <row r="376" spans="1:4" ht="15.75" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A376" s="6">
-        <v>70638</v>
+        <v>70115</v>
       </c>
       <c r="B376" t="s">
-        <v>306</v>
+        <v>331</v>
       </c>
       <c r="C376" s="1" t="s">
         <v>4</v>
       </c>
-      <c r="D376" s="12" t="s">
-        <v>8</v>
+      <c r="D376" s="9" t="s">
+        <v>9</v>
       </c>
     </row>
     <row r="377" spans="1:4" ht="15.75" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A377" s="6">
-        <v>70639</v>
+        <v>70638</v>
       </c>
       <c r="B377" t="s">
-        <v>307</v>
+        <v>306</v>
       </c>
       <c r="C377" s="1" t="s">
         <v>4</v>
@@ -6894,10 +6897,10 @@
     </row>
     <row r="378" spans="1:4" ht="15.75" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A378" s="6">
-        <v>70640</v>
+        <v>70639</v>
       </c>
       <c r="B378" t="s">
-        <v>308</v>
+        <v>307</v>
       </c>
       <c r="C378" s="1" t="s">
         <v>4</v>
@@ -6908,10 +6911,10 @@
     </row>
     <row r="379" spans="1:4" ht="15.75" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A379" s="6">
-        <v>70642</v>
+        <v>70640</v>
       </c>
       <c r="B379" t="s">
-        <v>309</v>
+        <v>308</v>
       </c>
       <c r="C379" s="1" t="s">
         <v>4</v>
@@ -6922,10 +6925,10 @@
     </row>
     <row r="380" spans="1:4" ht="15.75" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A380" s="6">
-        <v>90504</v>
+        <v>70642</v>
       </c>
       <c r="B380" t="s">
-        <v>310</v>
+        <v>309</v>
       </c>
       <c r="C380" s="1" t="s">
         <v>4</v>
@@ -6936,10 +6939,10 @@
     </row>
     <row r="381" spans="1:4" ht="15.75" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A381" s="6">
-        <v>90509</v>
+        <v>90504</v>
       </c>
       <c r="B381" t="s">
-        <v>311</v>
+        <v>310</v>
       </c>
       <c r="C381" s="1" t="s">
         <v>4</v>
@@ -6950,52 +6953,52 @@
     </row>
     <row r="382" spans="1:4" ht="15.75" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A382" s="6">
-        <v>90602</v>
+        <v>90509</v>
       </c>
       <c r="B382" t="s">
-        <v>312</v>
+        <v>311</v>
       </c>
       <c r="C382" s="1" t="s">
         <v>4</v>
       </c>
-      <c r="D382" s="15" t="s">
-        <v>5</v>
+      <c r="D382" s="12" t="s">
+        <v>8</v>
       </c>
     </row>
     <row r="383" spans="1:4" ht="15.75" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A383" s="6">
-        <v>90621</v>
+        <v>90602</v>
       </c>
       <c r="B383" t="s">
-        <v>313</v>
+        <v>312</v>
       </c>
       <c r="C383" s="1" t="s">
         <v>4</v>
       </c>
-      <c r="D383" s="12" t="s">
-        <v>8</v>
+      <c r="D383" s="15" t="s">
+        <v>5</v>
       </c>
     </row>
     <row r="384" spans="1:4" ht="15.75" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A384" s="6">
-        <v>90622</v>
+        <v>90621</v>
       </c>
       <c r="B384" t="s">
-        <v>333</v>
+        <v>313</v>
       </c>
       <c r="C384" s="1" t="s">
         <v>4</v>
       </c>
-      <c r="D384" s="9" t="s">
-        <v>5</v>
+      <c r="D384" s="12" t="s">
+        <v>8</v>
       </c>
     </row>
     <row r="385" spans="1:4" ht="15.75" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A385" s="6">
-        <v>90631</v>
-      </c>
-      <c r="B385" s="8" t="s">
-        <v>342</v>
+        <v>90622</v>
+      </c>
+      <c r="B385" t="s">
+        <v>333</v>
       </c>
       <c r="C385" s="1" t="s">
         <v>4</v>
@@ -7006,24 +7009,24 @@
     </row>
     <row r="386" spans="1:4" ht="15.75" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A386" s="6">
-        <v>90658</v>
-      </c>
-      <c r="B386" t="s">
-        <v>314</v>
+        <v>90631</v>
+      </c>
+      <c r="B386" s="8" t="s">
+        <v>342</v>
       </c>
       <c r="C386" s="1" t="s">
         <v>4</v>
       </c>
-      <c r="D386" s="12" t="s">
-        <v>8</v>
+      <c r="D386" s="9" t="s">
+        <v>5</v>
       </c>
     </row>
     <row r="387" spans="1:4" ht="15.75" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A387" s="6">
-        <v>90660</v>
+        <v>90658</v>
       </c>
       <c r="B387" t="s">
-        <v>315</v>
+        <v>314</v>
       </c>
       <c r="C387" s="1" t="s">
         <v>4</v>
@@ -7034,10 +7037,10 @@
     </row>
     <row r="388" spans="1:4" ht="15.75" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A388" s="6">
-        <v>90668</v>
+        <v>90660</v>
       </c>
       <c r="B388" t="s">
-        <v>316</v>
+        <v>315</v>
       </c>
       <c r="C388" s="1" t="s">
         <v>4</v>
@@ -7048,10 +7051,10 @@
     </row>
     <row r="389" spans="1:4" ht="15.75" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A389" s="6">
-        <v>90671</v>
+        <v>90668</v>
       </c>
       <c r="B389" t="s">
-        <v>317</v>
+        <v>316</v>
       </c>
       <c r="C389" s="1" t="s">
         <v>4</v>
@@ -7062,10 +7065,10 @@
     </row>
     <row r="390" spans="1:4" ht="15.75" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A390" s="6">
-        <v>90679</v>
+        <v>90671</v>
       </c>
       <c r="B390" t="s">
-        <v>318</v>
+        <v>317</v>
       </c>
       <c r="C390" s="1" t="s">
         <v>4</v>
@@ -7076,10 +7079,10 @@
     </row>
     <row r="391" spans="1:4" ht="15.75" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A391" s="6">
-        <v>90683</v>
+        <v>90679</v>
       </c>
       <c r="B391" t="s">
-        <v>319</v>
+        <v>318</v>
       </c>
       <c r="C391" s="1" t="s">
         <v>4</v>
@@ -7090,10 +7093,10 @@
     </row>
     <row r="392" spans="1:4" ht="15.75" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A392" s="6">
-        <v>90705</v>
+        <v>90683</v>
       </c>
       <c r="B392" t="s">
-        <v>320</v>
+        <v>319</v>
       </c>
       <c r="C392" s="1" t="s">
         <v>4</v>
@@ -7104,10 +7107,10 @@
     </row>
     <row r="393" spans="1:4" ht="15.75" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A393" s="6">
-        <v>90706</v>
+        <v>90705</v>
       </c>
       <c r="B393" t="s">
-        <v>321</v>
+        <v>320</v>
       </c>
       <c r="C393" s="1" t="s">
         <v>4</v>
@@ -7118,10 +7121,10 @@
     </row>
     <row r="394" spans="1:4" ht="15.75" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A394" s="6">
-        <v>90708</v>
+        <v>90706</v>
       </c>
       <c r="B394" t="s">
-        <v>322</v>
+        <v>321</v>
       </c>
       <c r="C394" s="1" t="s">
         <v>4</v>
@@ -7132,10 +7135,10 @@
     </row>
     <row r="395" spans="1:4" ht="15.75" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A395" s="6">
-        <v>90709</v>
+        <v>90708</v>
       </c>
       <c r="B395" t="s">
-        <v>323</v>
+        <v>322</v>
       </c>
       <c r="C395" s="1" t="s">
         <v>4</v>
@@ -7146,38 +7149,38 @@
     </row>
     <row r="396" spans="1:4" ht="15.75" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A396" s="6">
-        <v>90713</v>
+        <v>90709</v>
       </c>
       <c r="B396" t="s">
-        <v>402</v>
+        <v>323</v>
       </c>
       <c r="C396" s="1" t="s">
         <v>4</v>
       </c>
       <c r="D396" s="12" t="s">
-        <v>5</v>
+        <v>8</v>
       </c>
     </row>
     <row r="397" spans="1:4" ht="15.75" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A397" s="6">
-        <v>1218</v>
+        <v>90713</v>
       </c>
       <c r="B397" t="s">
-        <v>382</v>
+        <v>402</v>
       </c>
       <c r="C397" s="1" t="s">
         <v>4</v>
       </c>
       <c r="D397" s="12" t="s">
-        <v>8</v>
+        <v>5</v>
       </c>
     </row>
     <row r="398" spans="1:4" ht="15.75" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A398" s="6">
-        <v>1959</v>
-      </c>
-      <c r="B398" s="8" t="s">
-        <v>383</v>
+        <v>1218</v>
+      </c>
+      <c r="B398" t="s">
+        <v>382</v>
       </c>
       <c r="C398" s="1" t="s">
         <v>4</v>
@@ -7188,10 +7191,10 @@
     </row>
     <row r="399" spans="1:4" ht="15.75" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A399" s="6">
-        <v>5625</v>
+        <v>1959</v>
       </c>
       <c r="B399" s="8" t="s">
-        <v>384</v>
+        <v>383</v>
       </c>
       <c r="C399" s="1" t="s">
         <v>4</v>
@@ -7202,10 +7205,10 @@
     </row>
     <row r="400" spans="1:4" ht="15.75" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A400" s="6">
-        <v>1817</v>
+        <v>5625</v>
       </c>
       <c r="B400" s="8" t="s">
-        <v>389</v>
+        <v>384</v>
       </c>
       <c r="C400" s="1" t="s">
         <v>4</v>
@@ -7216,10 +7219,10 @@
     </row>
     <row r="401" spans="1:4" ht="15.75" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A401" s="6">
-        <v>5737</v>
+        <v>1817</v>
       </c>
       <c r="B401" s="8" t="s">
-        <v>390</v>
+        <v>389</v>
       </c>
       <c r="C401" s="1" t="s">
         <v>4</v>
@@ -7230,34 +7233,48 @@
     </row>
     <row r="402" spans="1:4" ht="15.75" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A402" s="6">
-        <v>60295</v>
+        <v>5737</v>
       </c>
       <c r="B402" s="8" t="s">
-        <v>385</v>
+        <v>390</v>
       </c>
       <c r="C402" s="1" t="s">
         <v>4</v>
       </c>
-      <c r="D402" s="9" t="s">
-        <v>9</v>
+      <c r="D402" s="12" t="s">
+        <v>8</v>
       </c>
     </row>
     <row r="403" spans="1:4" ht="15.75" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A403" s="6">
+        <v>60295</v>
+      </c>
+      <c r="B403" s="8" t="s">
+        <v>385</v>
+      </c>
+      <c r="C403" s="1" t="s">
+        <v>4</v>
+      </c>
+      <c r="D403" s="9" t="s">
+        <v>9</v>
+      </c>
+    </row>
+    <row r="404" spans="1:4" ht="15.75" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
+      <c r="A404" s="6">
         <v>1045</v>
       </c>
-      <c r="B403" s="8" t="s">
+      <c r="B404" s="8" t="s">
         <v>386</v>
       </c>
-      <c r="C403" s="1" t="s">
-        <v>4</v>
-      </c>
-      <c r="D403" s="9" t="s">
+      <c r="C404" s="1" t="s">
+        <v>4</v>
+      </c>
+      <c r="D404" s="9" t="s">
         <v>5</v>
       </c>
     </row>
   </sheetData>
-  <autoFilter ref="A1:D348"/>
+  <autoFilter ref="A1:D349"/>
   <sortState ref="A2:D374">
     <sortCondition ref="A277"/>
   </sortState>

</xml_diff>

<commit_message>
update listas de precios, active ctas 60302,60303 60194 y estado cuentas clientes 28-8-26
</commit_message>
<xml_diff>
--- a/excel/CLIENTES_PERMISOS.xlsx
+++ b/excel/CLIENTES_PERMISOS.xlsx
@@ -22,7 +22,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="1213" uniqueCount="411">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="1219" uniqueCount="413">
   <si>
     <t>CUENTA</t>
   </si>
@@ -1255,6 +1255,12 @@
   </si>
   <si>
     <t>EL BUHO FERRETERIA</t>
+  </si>
+  <si>
+    <t>FERRETERIA L y C</t>
+  </si>
+  <si>
+    <t>FERRETERIA EBER</t>
   </si>
 </sst>
 </file>
@@ -1609,7 +1615,7 @@
   <sheetPr>
     <outlinePr summaryBelow="0" summaryRight="0"/>
   </sheetPr>
-  <dimension ref="A1:D404"/>
+  <dimension ref="A1:D406"/>
   <sheetFormatPr baseColWidth="10" defaultColWidth="12.5703125" defaultRowHeight="15.75" customHeight="1" x14ac:dyDescent="0.2"/>
   <cols>
     <col min="2" max="2" width="34" customWidth="1"/>
@@ -6659,38 +6665,38 @@
     </row>
     <row r="361" spans="1:4" ht="15.75" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A361" s="6">
-        <v>61001</v>
-      </c>
-      <c r="B361" t="s">
-        <v>403</v>
+        <v>60302</v>
+      </c>
+      <c r="B361" s="18" t="s">
+        <v>411</v>
       </c>
       <c r="C361" s="1" t="s">
         <v>4</v>
       </c>
       <c r="D361" s="12" t="s">
-        <v>8</v>
+        <v>5</v>
       </c>
     </row>
     <row r="362" spans="1:4" ht="15.75" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A362" s="6">
-        <v>61004</v>
-      </c>
-      <c r="B362" t="s">
-        <v>293</v>
+        <v>60303</v>
+      </c>
+      <c r="B362" s="18" t="s">
+        <v>412</v>
       </c>
       <c r="C362" s="1" t="s">
         <v>4</v>
       </c>
-      <c r="D362" s="15" t="s">
+      <c r="D362" s="12" t="s">
         <v>5</v>
       </c>
     </row>
     <row r="363" spans="1:4" ht="15.75" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A363" s="6">
-        <v>61009</v>
+        <v>61001</v>
       </c>
       <c r="B363" t="s">
-        <v>294</v>
+        <v>403</v>
       </c>
       <c r="C363" s="1" t="s">
         <v>4</v>
@@ -6701,24 +6707,24 @@
     </row>
     <row r="364" spans="1:4" ht="15.75" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A364" s="6">
-        <v>61012</v>
+        <v>61004</v>
       </c>
       <c r="B364" t="s">
-        <v>295</v>
+        <v>293</v>
       </c>
       <c r="C364" s="1" t="s">
         <v>4</v>
       </c>
-      <c r="D364" s="12" t="s">
-        <v>8</v>
+      <c r="D364" s="15" t="s">
+        <v>5</v>
       </c>
     </row>
     <row r="365" spans="1:4" ht="15.75" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A365" s="6">
-        <v>61018</v>
+        <v>61009</v>
       </c>
       <c r="B365" t="s">
-        <v>296</v>
+        <v>294</v>
       </c>
       <c r="C365" s="1" t="s">
         <v>4</v>
@@ -6729,10 +6735,10 @@
     </row>
     <row r="366" spans="1:4" ht="15.75" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A366" s="6">
-        <v>61102</v>
+        <v>61012</v>
       </c>
       <c r="B366" t="s">
-        <v>297</v>
+        <v>295</v>
       </c>
       <c r="C366" s="1" t="s">
         <v>4</v>
@@ -6743,24 +6749,24 @@
     </row>
     <row r="367" spans="1:4" ht="15.75" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A367" s="6">
-        <v>61205</v>
+        <v>61018</v>
       </c>
       <c r="B367" t="s">
-        <v>298</v>
+        <v>296</v>
       </c>
       <c r="C367" s="1" t="s">
         <v>4</v>
       </c>
-      <c r="D367" s="15" t="s">
-        <v>5</v>
+      <c r="D367" s="12" t="s">
+        <v>8</v>
       </c>
     </row>
     <row r="368" spans="1:4" ht="15.75" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A368" s="6">
-        <v>70100</v>
+        <v>61102</v>
       </c>
       <c r="B368" t="s">
-        <v>299</v>
+        <v>297</v>
       </c>
       <c r="C368" s="1" t="s">
         <v>4</v>
@@ -6771,10 +6777,10 @@
     </row>
     <row r="369" spans="1:4" ht="15.75" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A369" s="6">
-        <v>70101</v>
+        <v>61205</v>
       </c>
       <c r="B369" t="s">
-        <v>300</v>
+        <v>298</v>
       </c>
       <c r="C369" s="1" t="s">
         <v>4</v>
@@ -6785,38 +6791,38 @@
     </row>
     <row r="370" spans="1:4" ht="15.75" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A370" s="6">
-        <v>70102</v>
+        <v>70100</v>
       </c>
       <c r="B370" t="s">
-        <v>301</v>
+        <v>299</v>
       </c>
       <c r="C370" s="1" t="s">
         <v>4</v>
       </c>
-      <c r="D370" s="15" t="s">
-        <v>5</v>
+      <c r="D370" s="12" t="s">
+        <v>8</v>
       </c>
     </row>
     <row r="371" spans="1:4" ht="15.75" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A371" s="6">
-        <v>70103</v>
+        <v>70101</v>
       </c>
       <c r="B371" t="s">
-        <v>302</v>
+        <v>300</v>
       </c>
       <c r="C371" s="1" t="s">
         <v>4</v>
       </c>
-      <c r="D371" s="12" t="s">
-        <v>8</v>
+      <c r="D371" s="15" t="s">
+        <v>5</v>
       </c>
     </row>
     <row r="372" spans="1:4" ht="15.75" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A372" s="6">
-        <v>70106</v>
+        <v>70102</v>
       </c>
       <c r="B372" t="s">
-        <v>303</v>
+        <v>301</v>
       </c>
       <c r="C372" s="1" t="s">
         <v>4</v>
@@ -6827,10 +6833,10 @@
     </row>
     <row r="373" spans="1:4" ht="15.75" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A373" s="6">
-        <v>70109</v>
+        <v>70103</v>
       </c>
       <c r="B373" t="s">
-        <v>304</v>
+        <v>302</v>
       </c>
       <c r="C373" s="1" t="s">
         <v>4</v>
@@ -6841,10 +6847,10 @@
     </row>
     <row r="374" spans="1:4" ht="15.75" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A374" s="6">
-        <v>70113</v>
+        <v>70106</v>
       </c>
       <c r="B374" t="s">
-        <v>305</v>
+        <v>303</v>
       </c>
       <c r="C374" s="1" t="s">
         <v>4</v>
@@ -6855,66 +6861,66 @@
     </row>
     <row r="375" spans="1:4" ht="15.75" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A375" s="6">
-        <v>70114</v>
+        <v>70109</v>
       </c>
       <c r="B375" t="s">
-        <v>325</v>
+        <v>304</v>
       </c>
       <c r="C375" s="1" t="s">
         <v>4</v>
       </c>
-      <c r="D375" s="9" t="s">
-        <v>9</v>
+      <c r="D375" s="12" t="s">
+        <v>8</v>
       </c>
     </row>
     <row r="376" spans="1:4" ht="15.75" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A376" s="6">
-        <v>70115</v>
+        <v>70113</v>
       </c>
       <c r="B376" t="s">
-        <v>331</v>
+        <v>305</v>
       </c>
       <c r="C376" s="1" t="s">
         <v>4</v>
       </c>
-      <c r="D376" s="9" t="s">
-        <v>9</v>
+      <c r="D376" s="15" t="s">
+        <v>5</v>
       </c>
     </row>
     <row r="377" spans="1:4" ht="15.75" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A377" s="6">
-        <v>70638</v>
+        <v>70114</v>
       </c>
       <c r="B377" t="s">
-        <v>306</v>
+        <v>325</v>
       </c>
       <c r="C377" s="1" t="s">
         <v>4</v>
       </c>
-      <c r="D377" s="12" t="s">
-        <v>8</v>
+      <c r="D377" s="9" t="s">
+        <v>9</v>
       </c>
     </row>
     <row r="378" spans="1:4" ht="15.75" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A378" s="6">
-        <v>70639</v>
+        <v>70115</v>
       </c>
       <c r="B378" t="s">
-        <v>307</v>
+        <v>331</v>
       </c>
       <c r="C378" s="1" t="s">
         <v>4</v>
       </c>
-      <c r="D378" s="12" t="s">
-        <v>8</v>
+      <c r="D378" s="9" t="s">
+        <v>9</v>
       </c>
     </row>
     <row r="379" spans="1:4" ht="15.75" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A379" s="6">
-        <v>70640</v>
+        <v>70638</v>
       </c>
       <c r="B379" t="s">
-        <v>308</v>
+        <v>306</v>
       </c>
       <c r="C379" s="1" t="s">
         <v>4</v>
@@ -6925,10 +6931,10 @@
     </row>
     <row r="380" spans="1:4" ht="15.75" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A380" s="6">
-        <v>70642</v>
+        <v>70639</v>
       </c>
       <c r="B380" t="s">
-        <v>309</v>
+        <v>307</v>
       </c>
       <c r="C380" s="1" t="s">
         <v>4</v>
@@ -6939,10 +6945,10 @@
     </row>
     <row r="381" spans="1:4" ht="15.75" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A381" s="6">
-        <v>90504</v>
+        <v>70640</v>
       </c>
       <c r="B381" t="s">
-        <v>310</v>
+        <v>308</v>
       </c>
       <c r="C381" s="1" t="s">
         <v>4</v>
@@ -6953,10 +6959,10 @@
     </row>
     <row r="382" spans="1:4" ht="15.75" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A382" s="6">
-        <v>90509</v>
+        <v>70642</v>
       </c>
       <c r="B382" t="s">
-        <v>311</v>
+        <v>309</v>
       </c>
       <c r="C382" s="1" t="s">
         <v>4</v>
@@ -6967,24 +6973,24 @@
     </row>
     <row r="383" spans="1:4" ht="15.75" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A383" s="6">
-        <v>90602</v>
+        <v>90504</v>
       </c>
       <c r="B383" t="s">
-        <v>312</v>
+        <v>310</v>
       </c>
       <c r="C383" s="1" t="s">
         <v>4</v>
       </c>
-      <c r="D383" s="15" t="s">
-        <v>5</v>
+      <c r="D383" s="12" t="s">
+        <v>8</v>
       </c>
     </row>
     <row r="384" spans="1:4" ht="15.75" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A384" s="6">
-        <v>90621</v>
+        <v>90509</v>
       </c>
       <c r="B384" t="s">
-        <v>313</v>
+        <v>311</v>
       </c>
       <c r="C384" s="1" t="s">
         <v>4</v>
@@ -6995,66 +7001,66 @@
     </row>
     <row r="385" spans="1:4" ht="15.75" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A385" s="6">
-        <v>90622</v>
+        <v>90602</v>
       </c>
       <c r="B385" t="s">
-        <v>333</v>
+        <v>312</v>
       </c>
       <c r="C385" s="1" t="s">
         <v>4</v>
       </c>
-      <c r="D385" s="9" t="s">
+      <c r="D385" s="15" t="s">
         <v>5</v>
       </c>
     </row>
     <row r="386" spans="1:4" ht="15.75" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A386" s="6">
-        <v>90631</v>
-      </c>
-      <c r="B386" s="8" t="s">
-        <v>342</v>
+        <v>90621</v>
+      </c>
+      <c r="B386" t="s">
+        <v>313</v>
       </c>
       <c r="C386" s="1" t="s">
         <v>4</v>
       </c>
-      <c r="D386" s="9" t="s">
-        <v>5</v>
+      <c r="D386" s="12" t="s">
+        <v>8</v>
       </c>
     </row>
     <row r="387" spans="1:4" ht="15.75" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A387" s="6">
-        <v>90658</v>
+        <v>90622</v>
       </c>
       <c r="B387" t="s">
-        <v>314</v>
+        <v>333</v>
       </c>
       <c r="C387" s="1" t="s">
         <v>4</v>
       </c>
-      <c r="D387" s="12" t="s">
-        <v>8</v>
+      <c r="D387" s="9" t="s">
+        <v>5</v>
       </c>
     </row>
     <row r="388" spans="1:4" ht="15.75" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A388" s="6">
-        <v>90660</v>
-      </c>
-      <c r="B388" t="s">
-        <v>315</v>
+        <v>90631</v>
+      </c>
+      <c r="B388" s="8" t="s">
+        <v>342</v>
       </c>
       <c r="C388" s="1" t="s">
         <v>4</v>
       </c>
-      <c r="D388" s="12" t="s">
-        <v>8</v>
+      <c r="D388" s="9" t="s">
+        <v>5</v>
       </c>
     </row>
     <row r="389" spans="1:4" ht="15.75" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A389" s="6">
-        <v>90668</v>
+        <v>90658</v>
       </c>
       <c r="B389" t="s">
-        <v>316</v>
+        <v>314</v>
       </c>
       <c r="C389" s="1" t="s">
         <v>4</v>
@@ -7065,10 +7071,10 @@
     </row>
     <row r="390" spans="1:4" ht="15.75" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A390" s="6">
-        <v>90671</v>
+        <v>90660</v>
       </c>
       <c r="B390" t="s">
-        <v>317</v>
+        <v>315</v>
       </c>
       <c r="C390" s="1" t="s">
         <v>4</v>
@@ -7079,10 +7085,10 @@
     </row>
     <row r="391" spans="1:4" ht="15.75" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A391" s="6">
-        <v>90679</v>
+        <v>90668</v>
       </c>
       <c r="B391" t="s">
-        <v>318</v>
+        <v>316</v>
       </c>
       <c r="C391" s="1" t="s">
         <v>4</v>
@@ -7093,10 +7099,10 @@
     </row>
     <row r="392" spans="1:4" ht="15.75" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A392" s="6">
-        <v>90683</v>
+        <v>90671</v>
       </c>
       <c r="B392" t="s">
-        <v>319</v>
+        <v>317</v>
       </c>
       <c r="C392" s="1" t="s">
         <v>4</v>
@@ -7107,10 +7113,10 @@
     </row>
     <row r="393" spans="1:4" ht="15.75" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A393" s="6">
-        <v>90705</v>
+        <v>90679</v>
       </c>
       <c r="B393" t="s">
-        <v>320</v>
+        <v>318</v>
       </c>
       <c r="C393" s="1" t="s">
         <v>4</v>
@@ -7121,10 +7127,10 @@
     </row>
     <row r="394" spans="1:4" ht="15.75" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A394" s="6">
-        <v>90706</v>
+        <v>90683</v>
       </c>
       <c r="B394" t="s">
-        <v>321</v>
+        <v>319</v>
       </c>
       <c r="C394" s="1" t="s">
         <v>4</v>
@@ -7135,10 +7141,10 @@
     </row>
     <row r="395" spans="1:4" ht="15.75" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A395" s="6">
-        <v>90708</v>
+        <v>90705</v>
       </c>
       <c r="B395" t="s">
-        <v>322</v>
+        <v>320</v>
       </c>
       <c r="C395" s="1" t="s">
         <v>4</v>
@@ -7149,10 +7155,10 @@
     </row>
     <row r="396" spans="1:4" ht="15.75" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A396" s="6">
-        <v>90709</v>
+        <v>90706</v>
       </c>
       <c r="B396" t="s">
-        <v>323</v>
+        <v>321</v>
       </c>
       <c r="C396" s="1" t="s">
         <v>4</v>
@@ -7163,24 +7169,24 @@
     </row>
     <row r="397" spans="1:4" ht="15.75" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A397" s="6">
-        <v>90713</v>
+        <v>90708</v>
       </c>
       <c r="B397" t="s">
-        <v>402</v>
+        <v>322</v>
       </c>
       <c r="C397" s="1" t="s">
         <v>4</v>
       </c>
       <c r="D397" s="12" t="s">
-        <v>5</v>
+        <v>8</v>
       </c>
     </row>
     <row r="398" spans="1:4" ht="15.75" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A398" s="6">
-        <v>1218</v>
+        <v>90709</v>
       </c>
       <c r="B398" t="s">
-        <v>382</v>
+        <v>323</v>
       </c>
       <c r="C398" s="1" t="s">
         <v>4</v>
@@ -7191,24 +7197,24 @@
     </row>
     <row r="399" spans="1:4" ht="15.75" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A399" s="6">
-        <v>1959</v>
-      </c>
-      <c r="B399" s="8" t="s">
-        <v>383</v>
+        <v>90713</v>
+      </c>
+      <c r="B399" t="s">
+        <v>402</v>
       </c>
       <c r="C399" s="1" t="s">
         <v>4</v>
       </c>
       <c r="D399" s="12" t="s">
-        <v>8</v>
+        <v>5</v>
       </c>
     </row>
     <row r="400" spans="1:4" ht="15.75" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A400" s="6">
-        <v>5625</v>
-      </c>
-      <c r="B400" s="8" t="s">
-        <v>384</v>
+        <v>1218</v>
+      </c>
+      <c r="B400" t="s">
+        <v>382</v>
       </c>
       <c r="C400" s="1" t="s">
         <v>4</v>
@@ -7219,10 +7225,10 @@
     </row>
     <row r="401" spans="1:4" ht="15.75" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A401" s="6">
-        <v>1817</v>
+        <v>1959</v>
       </c>
       <c r="B401" s="8" t="s">
-        <v>389</v>
+        <v>383</v>
       </c>
       <c r="C401" s="1" t="s">
         <v>4</v>
@@ -7233,10 +7239,10 @@
     </row>
     <row r="402" spans="1:4" ht="15.75" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A402" s="6">
-        <v>5737</v>
+        <v>5625</v>
       </c>
       <c r="B402" s="8" t="s">
-        <v>390</v>
+        <v>384</v>
       </c>
       <c r="C402" s="1" t="s">
         <v>4</v>
@@ -7247,29 +7253,57 @@
     </row>
     <row r="403" spans="1:4" ht="15.75" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A403" s="6">
-        <v>60295</v>
+        <v>1817</v>
       </c>
       <c r="B403" s="8" t="s">
-        <v>385</v>
+        <v>389</v>
       </c>
       <c r="C403" s="1" t="s">
         <v>4</v>
       </c>
-      <c r="D403" s="9" t="s">
-        <v>9</v>
+      <c r="D403" s="12" t="s">
+        <v>8</v>
       </c>
     </row>
     <row r="404" spans="1:4" ht="15.75" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A404" s="6">
+        <v>5737</v>
+      </c>
+      <c r="B404" s="8" t="s">
+        <v>390</v>
+      </c>
+      <c r="C404" s="1" t="s">
+        <v>4</v>
+      </c>
+      <c r="D404" s="12" t="s">
+        <v>8</v>
+      </c>
+    </row>
+    <row r="405" spans="1:4" ht="15.75" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
+      <c r="A405" s="6">
+        <v>60295</v>
+      </c>
+      <c r="B405" s="8" t="s">
+        <v>385</v>
+      </c>
+      <c r="C405" s="1" t="s">
+        <v>4</v>
+      </c>
+      <c r="D405" s="9" t="s">
+        <v>9</v>
+      </c>
+    </row>
+    <row r="406" spans="1:4" ht="15.75" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
+      <c r="A406" s="6">
         <v>1045</v>
       </c>
-      <c r="B404" s="8" t="s">
+      <c r="B406" s="8" t="s">
         <v>386</v>
       </c>
-      <c r="C404" s="1" t="s">
-        <v>4</v>
-      </c>
-      <c r="D404" s="9" t="s">
+      <c r="C406" s="1" t="s">
+        <v>4</v>
+      </c>
+      <c r="D406" s="9" t="s">
         <v>5</v>
       </c>
     </row>

</xml_diff>